<commit_message>
Started working on NVDA
</commit_message>
<xml_diff>
--- a/INTC.xlsx
+++ b/INTC.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/KINGSTON/MyStockData/Finance-StockLists/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{546458A5-898E-8A44-B4BF-C4B914BEC026}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{827F1DB6-3DE9-3540-B461-125F6B35ED3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="14400" activeTab="2" xr2:uid="{AEC0C047-6E16-294C-82BD-58123BA913A1}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="14400" xr2:uid="{AEC0C047-6E16-294C-82BD-58123BA913A1}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -119,7 +119,7 @@
       </extLst>
     </bk>
   </futureMetadata>
-  <futureMetadata name="XLRICHVALUE" count="5">
+  <futureMetadata name="XLRICHVALUE" count="2">
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
@@ -130,28 +130,7 @@
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="3"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="4"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
           <xlrd:rvb i="5"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="8"/>
         </ext>
       </extLst>
     </bk>
@@ -161,21 +140,12 @@
       <rc t="1" v="0"/>
     </bk>
   </cellMetadata>
-  <valueMetadata count="5">
+  <valueMetadata count="2">
     <bk>
       <rc t="2" v="0"/>
     </bk>
     <bk>
       <rc t="2" v="1"/>
-    </bk>
-    <bk>
-      <rc t="2" v="2"/>
-    </bk>
-    <bk>
-      <rc t="2" v="3"/>
-    </bk>
-    <bk>
-      <rc t="2" v="4"/>
     </bk>
   </valueMetadata>
 </metadata>
@@ -2278,6 +2248,12 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="168" fontId="18" fillId="17" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="18" fillId="17" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2285,12 +2261,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="18" fillId="17" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="18" fillId="17" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -11704,7 +11674,7 @@
 </file>
 
 <file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="9">
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="6">
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1vmf2&amp;q=XNAS%3aINTC&amp;form=skydnc</v>
     <v>Learn more on Bing</v>
@@ -11724,8 +11694,10 @@
     <v>132.75</v>
     <v>18.965</v>
     <v>2.2317999999999998</v>
-    <v>3.355</v>
-    <v>3.1084999999999998E-2</v>
+    <v>4.78</v>
+    <v>4.4288000000000001E-2</v>
+    <v>-1.89</v>
+    <v>-1.6768999999999999E-2</v>
     <v>USD</v>
     <v>Intel Corporation is a global designer and manufacturer of semiconductor products. The Company's segments include Intel Products, Intel Foundry, and All Other. Its Intel Products comprise Client Computing Group (CCG) and Data Center and AI (DCAI). CCG delivers platforms and processors that power PCs and edge devices, enabling enhanced performance, connectivity and user experience for consumer and commercial markets with capabilities that also support retail, industrial robotics and AI ecosystems at the edge. DCAI delivers workload-optimized solutions based upon its x86 architecture for data centers, including CPUs, AI accelerators, NICs, IPUs and custom ASICs, enabling performance and scalability for cloud, enterprise, telecommunication and HPC environments. The Intel Foundry segment comprises technology development, manufacturing and foundry services, developing new semiconductor process technologies and advanced packaging technologies. All Other segments include Mobileye and Other.</v>
     <v>83200</v>
@@ -11736,46 +11708,32 @@
     <v>118.29</v>
     <v>Semiconductors &amp; Semiconductor Equipment</v>
     <v>Stock</v>
-    <v>46176.724033205472</v>
+    <v>46176.925423043751</v>
     <v>0</v>
     <v>110.86</v>
-    <v>559318410000</v>
+    <v>566480460000</v>
     <v>INTEL CORPORATION</v>
     <v>INTEL CORPORATION</v>
-    <v>116.43</v>
+    <v>116.42</v>
     <v>0</v>
     <v>107.93</v>
-    <v>111.285</v>
+    <v>112.71</v>
+    <v>110.82</v>
     <v>5026000000</v>
     <v>INTC</v>
     <v>INTEL CORPORATION (XNAS:INTC)</v>
-    <v>84379814</v>
+    <v>118418472</v>
     <v>145048030</v>
     <v>1989</v>
   </rv>
   <rv s="2">
     <v>1</v>
   </rv>
-  <rv s="3">
-    <v>12</v>
-    <v>Price (Extended hours)</v>
-    <v>0</v>
-  </rv>
-  <rv s="3">
-    <v>12</v>
-    <v>Change (extended hours)</v>
-    <v>0</v>
-  </rv>
-  <rv s="3">
-    <v>12</v>
-    <v>Change % (extended hours)</v>
-    <v>0</v>
-  </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a33knm&amp;q=10+Y+TSY+YLD+NDX&amp;form=skydnc</v>
     <v>Learn more on Bing</v>
   </rv>
-  <rv s="4">
+  <rv s="3">
     <v>5</v>
     <v>10 Y TSY YLD NDX</v>
     <v>6</v>
@@ -11794,7 +11752,7 @@
     <v>US</v>
     <v>44.63</v>
     <v>Index</v>
-    <v>6</v>
+    <v>3</v>
     <v>44.28</v>
     <v>10 Y TSY YLD NDX</v>
     <v>44.3</v>
@@ -11804,13 +11762,13 @@
     <v>10 Y TSY YLD NDX</v>
   </rv>
   <rv s="2">
-    <v>7</v>
+    <v>4</v>
   </rv>
 </rvData>
 </file>
 
 <file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
-<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="5">
+<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="4">
   <s t="_hyperlink">
     <k n="Address" t="s"/>
     <k n="Text" t="s"/>
@@ -11832,6 +11790,8 @@
     <k n="Beta"/>
     <k n="Change"/>
     <k n="Change (%)"/>
+    <k n="Change (Extended hours)"/>
+    <k n="Change % (Extended hours)"/>
     <k n="Currency" t="s"/>
     <k n="Description" t="s"/>
     <k n="Employees"/>
@@ -11852,6 +11812,7 @@
     <k n="P/E"/>
     <k n="Previous close"/>
     <k n="Price"/>
+    <k n="Price (Extended hours)"/>
     <k n="Shares outstanding"/>
     <k n="Ticker symbol" t="s"/>
     <k n="UniqueName" t="s"/>
@@ -11861,11 +11822,6 @@
   </s>
   <s t="_linkedentity">
     <k n="%cvi" t="r"/>
-  </s>
-  <s t="_error">
-    <k n="errorType" t="i"/>
-    <k n="field" t="s"/>
-    <k n="subType" t="i"/>
   </s>
   <s t="_linkedentitycore">
     <k n="_Display" t="spb"/>
@@ -11901,7 +11857,7 @@
 <file path=xl/richData/rdsupportingpropertybag.xml><?xml version="1.0" encoding="utf-8"?>
 <supportingPropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2">
   <spbArrays count="2">
-    <a count="42">
+    <a count="45">
       <v t="s">%EntityServiceId</v>
       <v t="s">_Format</v>
       <v t="s">%IsRefreshable</v>
@@ -11912,13 +11868,16 @@
       <v t="s">Name</v>
       <v t="s">_SubLabel</v>
       <v t="s">Price</v>
+      <v t="s">Price (Extended hours)</v>
       <v t="s">Exchange</v>
       <v t="s">Official name</v>
       <v t="s">Last trade time</v>
       <v t="s">Ticker symbol</v>
       <v t="s">Exchange abbreviation</v>
       <v t="s">Change</v>
+      <v t="s">Change (Extended hours)</v>
       <v t="s">Change (%)</v>
+      <v t="s">Change % (Extended hours)</v>
       <v t="s">Currency</v>
       <v t="s">Previous close</v>
       <v t="s">Open</v>
@@ -12012,13 +11971,19 @@
       <v>8</v>
       <v>9</v>
       <v>4</v>
+      <v>1</v>
+      <v>1</v>
+      <v>5</v>
     </spb>
     <spb s="4">
-      <v>Real-Time Nasdaq Last Sale</v>
+      <v>at close</v>
       <v>from previous close</v>
       <v>from previous close</v>
       <v>Source: Nasdaq Last Sale</v>
       <v>GMT</v>
+      <v>Real-Time Nasdaq Last Sale</v>
+      <v>from close</v>
+      <v>from close</v>
     </spb>
     <spb s="0">
       <v>1</v>
@@ -12090,6 +12055,9 @@
     <k n="Year incorporated" t="i"/>
     <k n="`%EntityServiceId" t="i"/>
     <k n="Shares outstanding" t="i"/>
+    <k n="Price (Extended hours)" t="i"/>
+    <k n="Change (Extended hours)" t="i"/>
+    <k n="Change % (Extended hours)" t="i"/>
   </s>
   <s>
     <k n="Price" t="s"/>
@@ -12097,6 +12065,9 @@
     <k n="Change (%)" t="s"/>
     <k n="ExchangeID" t="s"/>
     <k n="Last trade time" t="s"/>
+    <k n="Price (Extended hours)" t="s"/>
+    <k n="Change (Extended hours)" t="s"/>
+    <k n="Change % (Extended hours)" t="s"/>
   </s>
   <s>
     <k n="UniqueName" t="spb"/>
@@ -12610,7 +12581,7 @@
       </c>
       <c r="F3" s="189">
         <f ca="1">Statement!AC171</f>
-        <v>559318.41</v>
+        <v>566480.46</v>
       </c>
       <c r="H3" s="187" t="str">
         <f>'AVG target price'!B5</f>
@@ -12618,7 +12589,7 @@
       </c>
       <c r="I3" s="213">
         <f ca="1">'AVG target price'!C5</f>
-        <v>-8.808241809556387</v>
+        <v>-8.8046952175618021</v>
       </c>
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.2">
@@ -12634,7 +12605,7 @@
       </c>
       <c r="F4" s="190">
         <f ca="1">Statement!AC172</f>
-        <v>585155.41</v>
+        <v>592317.46</v>
       </c>
       <c r="H4" s="187" t="str">
         <f>'AVG target price'!B6</f>
@@ -12642,7 +12613,7 @@
       </c>
       <c r="I4" s="213">
         <f ca="1">'AVG target price'!C6</f>
-        <v>32.333922448813013</v>
+        <v>32.321232777928991</v>
       </c>
     </row>
     <row r="5" spans="2:9" x14ac:dyDescent="0.2">
@@ -12651,7 +12622,7 @@
       </c>
       <c r="C5" s="210" cm="1">
         <f t="array" aca="1" ref="C5" ca="1">_FV(C3,"Price",TRUE)</f>
-        <v>111.285</v>
+        <v>112.71</v>
       </c>
       <c r="E5" s="187" t="s">
         <v>246</v>
@@ -12666,23 +12637,23 @@
       </c>
       <c r="I5" s="213">
         <f ca="1">'AVG target price'!C7</f>
-        <v>36.483298773483725</v>
+        <v>36.468980651241303</v>
       </c>
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B6" s="187" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="210" t="e" cm="1" vm="2">
-        <f t="array" ref="C6">_FV(C3,"Price (Extended hours)",TRUE)</f>
-        <v>#VALUE!</v>
+      <c r="C6" s="210" cm="1">
+        <f t="array" aca="1" ref="C6" ca="1">_FV(C3,"Price (Extended hours)",TRUE)</f>
+        <v>110.82</v>
       </c>
       <c r="E6" s="187" t="s">
         <v>240</v>
       </c>
       <c r="F6" s="192">
         <f ca="1">Statement!AC168</f>
-        <v>-179.49193548387098</v>
+        <v>-181.79032258064515</v>
       </c>
       <c r="H6" s="187" t="str">
         <f>'AVG target price'!B8</f>
@@ -12690,7 +12661,7 @@
       </c>
       <c r="I6" s="213">
         <f ca="1">'AVG target price'!C8</f>
-        <v>-10.988884344918722</v>
+        <v>-10.984571681463171</v>
       </c>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.2">
@@ -12699,14 +12670,14 @@
       </c>
       <c r="C7" s="6" cm="1">
         <f t="array" aca="1" ref="C7" ca="1">_FV(C3,"Change")</f>
-        <v>3.355</v>
+        <v>4.78</v>
       </c>
       <c r="E7" s="188" t="s">
         <v>197</v>
       </c>
       <c r="F7" s="193">
         <f ca="1">Statement!AC169</f>
-        <v>9.7399990234919915</v>
+        <v>9.8647193236984538</v>
       </c>
       <c r="H7" s="186" t="str">
         <f>'AVG target price'!B9</f>
@@ -12714,23 +12685,23 @@
       </c>
       <c r="I7" s="214">
         <f ca="1">'AVG target price'!C9</f>
-        <v>12.255023766955407</v>
+        <v>12.25023663253633</v>
       </c>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B8" s="187" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="6" t="e" cm="1" vm="3">
-        <f t="array" ref="C8">_FV(C3,"Change (extended hours)",TRUE)</f>
-        <v>#VALUE!</v>
+      <c r="C8" s="6" cm="1">
+        <f t="array" aca="1" ref="C8" ca="1">_FV(C3,"Change (extended hours)",TRUE)</f>
+        <v>-1.89</v>
       </c>
       <c r="E8" s="187" t="s">
         <v>268</v>
       </c>
       <c r="F8" s="194">
         <f ca="1">Statement!AC179</f>
-        <v>-9.8155181410889015E-3</v>
+        <v>-9.6914198946950452E-3</v>
       </c>
       <c r="H8" s="186" t="str">
         <f>'AVG target price'!B11</f>
@@ -12738,7 +12709,7 @@
       </c>
       <c r="I8" s="215">
         <f ca="1">'AVG target price'!C11</f>
-        <v>-0.88987712839146871</v>
+        <v>-0.8913118921787212</v>
       </c>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.2">
@@ -12747,23 +12718,23 @@
       </c>
       <c r="C9" s="72" cm="1">
         <f t="array" aca="1" ref="C9" ca="1">_FV(C3,"Change (%)",TRUE)</f>
-        <v>3.1084999999999998E-2</v>
+        <v>4.4288000000000001E-2</v>
       </c>
       <c r="E9" s="187" t="s">
         <v>292</v>
       </c>
       <c r="F9" s="194">
         <f ca="1">Statement!AC180</f>
-        <v>-5.5712809453205732E-3</v>
+        <v>-5.5008428710850857E-3</v>
       </c>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B10" s="187" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="72" t="e" cm="1" vm="4">
-        <f t="array" ref="C10">_FV(C3,"Change % (extended hours)",TRUE)</f>
-        <v>#VALUE!</v>
+      <c r="C10" s="72" cm="1">
+        <f t="array" aca="1" ref="C10" ca="1">_FV(C3,"Change % (extended hours)",TRUE)</f>
+        <v>-1.6768999999999999E-2</v>
       </c>
       <c r="E10" s="187" t="s">
         <v>297</v>
@@ -12843,7 +12814,7 @@
       </c>
       <c r="F15" s="194">
         <f ca="1">Statement!AC193</f>
-        <v>-2.1887353931368002E-2</v>
+        <v>-2.1610630665001226E-2</v>
       </c>
     </row>
     <row r="16" spans="2:9" x14ac:dyDescent="0.2">
@@ -12948,7 +12919,7 @@
       <c r="C26" s="171">
         <v>0.21</v>
       </c>
-      <c r="E26" s="187" t="e" vm="5">
+      <c r="E26" s="187" t="e" vm="2">
         <v>#VALUE!</v>
       </c>
       <c r="F26" s="226" cm="1">
@@ -17387,6 +17358,12 @@
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="C3:G3"/>
+    <mergeCell ref="H3:L3"/>
+    <mergeCell ref="P3:W3"/>
+    <mergeCell ref="X3:Z3"/>
+    <mergeCell ref="C5:L5"/>
+    <mergeCell ref="P5:Z5"/>
     <mergeCell ref="C40:L40"/>
     <mergeCell ref="C11:L11"/>
     <mergeCell ref="P11:Z11"/>
@@ -17394,12 +17371,6 @@
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="C26:L26"/>
     <mergeCell ref="C33:L33"/>
-    <mergeCell ref="C3:G3"/>
-    <mergeCell ref="H3:L3"/>
-    <mergeCell ref="P3:W3"/>
-    <mergeCell ref="X3:Z3"/>
-    <mergeCell ref="C5:L5"/>
-    <mergeCell ref="P5:Z5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
@@ -18459,16 +18430,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="AA2:AC2"/>
+    <mergeCell ref="C4:L4"/>
+    <mergeCell ref="S4:AC4"/>
+    <mergeCell ref="C13:L13"/>
+    <mergeCell ref="C18:L18"/>
     <mergeCell ref="C31:L31"/>
     <mergeCell ref="C25:L25"/>
     <mergeCell ref="C2:G2"/>
     <mergeCell ref="H2:L2"/>
     <mergeCell ref="S2:Z2"/>
-    <mergeCell ref="AA2:AC2"/>
-    <mergeCell ref="C4:L4"/>
-    <mergeCell ref="S4:AC4"/>
-    <mergeCell ref="C13:L13"/>
-    <mergeCell ref="C18:L18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -18551,7 +18522,7 @@
       </c>
       <c r="C6" s="132">
         <f ca="1">Overview!C5</f>
-        <v>111.285</v>
+        <v>112.71</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -18560,7 +18531,7 @@
       </c>
       <c r="C7" s="133">
         <f ca="1">C5*C6</f>
-        <v>559318.41</v>
+        <v>566480.46</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -18630,7 +18601,7 @@
       </c>
       <c r="C16" s="46">
         <f ca="1">C8/(C8+C7)</f>
-        <v>7.4511531334166436E-2</v>
+        <v>7.3638848894180986E-2</v>
       </c>
     </row>
     <row r="17" spans="2:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -18639,7 +18610,7 @@
       </c>
       <c r="C17" s="46">
         <f ca="1">C7/(C8+C7)</f>
-        <v>0.92548846866583356</v>
+        <v>0.92636115110581896</v>
       </c>
     </row>
     <row r="18" spans="2:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -18666,7 +18637,7 @@
       </c>
       <c r="C20" s="46">
         <f ca="1">(C17*C19)+(C16*C18)</f>
-        <v>0.13735690560235675</v>
+        <v>0.13744619934229851</v>
       </c>
     </row>
     <row r="21" spans="2:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -18925,7 +18896,7 @@
       </c>
       <c r="L8" s="125">
         <f ca="1">L7*(1+C14)/(C15-C14)</f>
-        <v>-23291.932656446141</v>
+        <v>-23274.223920113993</v>
       </c>
       <c r="N8" s="90"/>
       <c r="O8" s="16"/>
@@ -18979,23 +18950,23 @@
       <c r="G10" s="138"/>
       <c r="H10" s="125">
         <f ca="1">H7/(1+$C$15)^H9</f>
-        <v>-6494.3039834257206</v>
+        <v>-6493.7941565070196</v>
       </c>
       <c r="I10" s="125">
         <f t="shared" ref="I10:L10" ca="1" si="0">I7/(1+$C$15)^I9</f>
-        <v>-5057.8691579644583</v>
+        <v>-5057.0750662070459</v>
       </c>
       <c r="J10" s="125">
         <f t="shared" ca="1" si="0"/>
-        <v>-3565.1001312306958</v>
+        <v>-3564.2605764441973</v>
       </c>
       <c r="K10" s="125">
         <f t="shared" ca="1" si="0"/>
-        <v>-3264.5443554323961</v>
+        <v>-3263.5193608417944</v>
       </c>
       <c r="L10" s="125">
         <f t="shared" ca="1" si="0"/>
-        <v>-1408.0891745177687</v>
+        <v>-1407.5365602091188</v>
       </c>
       <c r="N10" s="90"/>
     </row>
@@ -19014,7 +18985,7 @@
       <c r="K11" s="137"/>
       <c r="L11" s="125">
         <f ca="1">L8/(1+C15)^L9</f>
-        <v>-12238.316532259363</v>
+        <v>-12224.212443256436</v>
       </c>
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.2">
@@ -19037,7 +19008,7 @@
       </c>
       <c r="C15" s="134">
         <f ca="1">IF(WACC!C21&gt;0,WACC!C21,WACC!C20)</f>
-        <v>0.13735690560235675</v>
+        <v>0.13744619934229851</v>
       </c>
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.2">
@@ -19052,7 +19023,7 @@
       </c>
       <c r="C19" s="63">
         <f ca="1">SUM(H10:L10)</f>
-        <v>-19789.90680257104</v>
+        <v>-19786.185720209178</v>
       </c>
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.2">
@@ -19061,7 +19032,7 @@
       </c>
       <c r="C20" s="63">
         <f ca="1">L11</f>
-        <v>-12238.316532259363</v>
+        <v>-12224.212443256436</v>
       </c>
     </row>
     <row r="21" spans="2:3" x14ac:dyDescent="0.2">
@@ -19070,7 +19041,7 @@
       </c>
       <c r="C21" s="93">
         <f ca="1">C19+C20</f>
-        <v>-32028.223334830403</v>
+        <v>-32010.398163465616</v>
       </c>
     </row>
     <row r="22" spans="2:3" x14ac:dyDescent="0.2">
@@ -19097,7 +19068,7 @@
       </c>
       <c r="C24" s="93">
         <f ca="1">C21+C22-C23</f>
-        <v>-44270.2233348304</v>
+        <v>-44252.398163465616</v>
       </c>
     </row>
     <row r="25" spans="2:3" x14ac:dyDescent="0.2">
@@ -19115,7 +19086,7 @@
       </c>
       <c r="C26" s="142">
         <f ca="1">C24/C25</f>
-        <v>-8.808241809556387</v>
+        <v>-8.8046952175618021</v>
       </c>
     </row>
   </sheetData>
@@ -20124,7 +20095,7 @@
       </c>
       <c r="C39" s="134">
         <f ca="1">IF(WACC!C21&gt;0,WACC!C21,WACC!C20)</f>
-        <v>0.13735690560235675</v>
+        <v>0.13744619934229851</v>
       </c>
     </row>
     <row r="40" spans="2:14" x14ac:dyDescent="0.2">
@@ -20168,7 +20139,7 @@
       </c>
       <c r="C44" s="142">
         <f ca="1">C43/(1+C48)^5</f>
-        <v>32.333922448813013</v>
+        <v>32.321232777928991</v>
       </c>
     </row>
     <row r="46" spans="2:14" x14ac:dyDescent="0.2">
@@ -20192,7 +20163,7 @@
       </c>
       <c r="C48" s="134">
         <f ca="1">IF(WACC!C21&gt;0,WACC!C21,WACC!C20)</f>
-        <v>0.13735690560235675</v>
+        <v>0.13744619934229851</v>
       </c>
     </row>
     <row r="49" spans="2:3" x14ac:dyDescent="0.2">
@@ -20227,7 +20198,7 @@
       </c>
       <c r="C52" s="142">
         <f ca="1">C51/(1+C48)^5</f>
-        <v>36.483298773483725</v>
+        <v>36.468980651241303</v>
       </c>
     </row>
     <row r="54" spans="2:3" x14ac:dyDescent="0.2">
@@ -20251,7 +20222,7 @@
       </c>
       <c r="C56" s="134">
         <f ca="1">IF(WACC!C21&gt;0,WACC!C21,WACC!C20)</f>
-        <v>0.13735690560235675</v>
+        <v>0.13744619934229851</v>
       </c>
     </row>
     <row r="57" spans="2:3" x14ac:dyDescent="0.2">
@@ -20295,7 +20266,7 @@
       </c>
       <c r="C61" s="142">
         <f ca="1">C60/(1+C56)^5</f>
-        <v>-10.988884344918722</v>
+        <v>-10.984571681463171</v>
       </c>
     </row>
   </sheetData>
@@ -20359,7 +20330,7 @@
       </c>
       <c r="C5" s="132">
         <f ca="1">DCF!C26</f>
-        <v>-8.808241809556387</v>
+        <v>-8.8046952175618021</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
@@ -20368,7 +20339,7 @@
       </c>
       <c r="C6" s="132">
         <f ca="1">Multiples!C44</f>
-        <v>32.333922448813013</v>
+        <v>32.321232777928991</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.2">
@@ -20377,7 +20348,7 @@
       </c>
       <c r="C7" s="132">
         <f ca="1">Multiples!C52</f>
-        <v>36.483298773483725</v>
+        <v>36.468980651241303</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.2">
@@ -20386,7 +20357,7 @@
       </c>
       <c r="C8" s="132">
         <f ca="1">Multiples!C61</f>
-        <v>-10.988884344918722</v>
+        <v>-10.984571681463171</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.2">
@@ -20395,7 +20366,7 @@
       </c>
       <c r="C9" s="142">
         <f ca="1">AVERAGE(C5:C8)</f>
-        <v>12.255023766955407</v>
+        <v>12.25023663253633</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.2">
@@ -20404,7 +20375,7 @@
       </c>
       <c r="C10" s="132">
         <f ca="1">Overview!C5</f>
-        <v>111.285</v>
+        <v>112.71</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.2">
@@ -20413,7 +20384,7 @@
       </c>
       <c r="C11" s="154">
         <f ca="1">(C9-C10)/C10</f>
-        <v>-0.88987712839146871</v>
+        <v>-0.8913118921787212</v>
       </c>
     </row>
   </sheetData>
@@ -20666,7 +20637,7 @@
       <c r="K8" s="137"/>
       <c r="L8" s="125">
         <f ca="1">L7*(1+C20)/(C21-C20)</f>
-        <v>-964945.54221544415</v>
+        <v>-964211.89909385249</v>
       </c>
       <c r="N8" s="90"/>
       <c r="O8" s="16"/>
@@ -20720,23 +20691,23 @@
       <c r="G10" s="138"/>
       <c r="H10" s="125">
         <f ca="1">H7/(1+$C$21)^H9</f>
-        <v>-13169.786558712953</v>
+        <v>-13168.752681684975</v>
       </c>
       <c r="I10" s="125">
         <f t="shared" ref="I10:L10" ca="1" si="1">I7/(1+$C$21)^I9</f>
-        <v>-19105.830117915226</v>
+        <v>-19102.830478790267</v>
       </c>
       <c r="J10" s="125">
         <f t="shared" ca="1" si="1"/>
-        <v>-27717.438157958284</v>
+        <v>-27710.910905702134</v>
       </c>
       <c r="K10" s="125">
         <f t="shared" ca="1" si="1"/>
-        <v>-40210.573071088947</v>
+        <v>-40197.947842145659</v>
       </c>
       <c r="L10" s="125">
         <f t="shared" ca="1" si="1"/>
-        <v>-58334.763028636487</v>
+        <v>-58311.869148529528</v>
       </c>
       <c r="N10" s="90"/>
     </row>
@@ -20755,7 +20726,7 @@
       <c r="K11" s="137"/>
       <c r="L11" s="125">
         <f ca="1">L8/(1+C21)^L9</f>
-        <v>-507012.84243825806</v>
+        <v>-506428.53378465137</v>
       </c>
     </row>
     <row r="13" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
@@ -20771,7 +20742,7 @@
       </c>
       <c r="C15" s="156">
         <f ca="1">Overview!C5</f>
-        <v>111.285</v>
+        <v>112.71</v>
       </c>
     </row>
     <row r="16" spans="1:28" x14ac:dyDescent="0.2">
@@ -20780,7 +20751,7 @@
       </c>
       <c r="C16" s="156">
         <f ca="1">C36</f>
-        <v>-134.85738825558497</v>
+        <v>-134.73196276193872</v>
       </c>
     </row>
     <row r="17" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -20819,7 +20790,7 @@
       </c>
       <c r="C21" s="161">
         <f ca="1">IF(WACC!C21&gt;0,WACC!C21,WACC!C20)</f>
-        <v>0.13735690560235675</v>
+        <v>0.13744619934229851</v>
       </c>
     </row>
     <row r="22" spans="2:9" x14ac:dyDescent="0.2">
@@ -20837,7 +20808,7 @@
       </c>
       <c r="C23" s="162">
         <f ca="1">C15*C22</f>
-        <v>559318.41</v>
+        <v>566480.46</v>
       </c>
     </row>
     <row r="24" spans="2:9" x14ac:dyDescent="0.2">
@@ -20864,7 +20835,7 @@
       </c>
       <c r="C26" s="163">
         <f ca="1">C23+C25-C24</f>
-        <v>571560.41</v>
+        <v>578722.46</v>
       </c>
     </row>
     <row r="27" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
@@ -20880,7 +20851,7 @@
       </c>
       <c r="C29" s="162">
         <f ca="1">SUM(H10:L10)</f>
-        <v>-158538.3909343119</v>
+        <v>-158492.31105685257</v>
       </c>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.2">
@@ -20889,7 +20860,7 @@
       </c>
       <c r="C30" s="162">
         <f ca="1">L11</f>
-        <v>-507012.84243825806</v>
+        <v>-506428.53378465137</v>
       </c>
     </row>
     <row r="31" spans="2:9" x14ac:dyDescent="0.2">
@@ -20898,7 +20869,7 @@
       </c>
       <c r="C31" s="165">
         <f ca="1">C29+C30</f>
-        <v>-665551.23337257002</v>
+        <v>-664920.844841504</v>
       </c>
     </row>
     <row r="32" spans="2:9" x14ac:dyDescent="0.2">
@@ -20925,7 +20896,7 @@
       </c>
       <c r="C34" s="165">
         <f ca="1">C31+C32-C33</f>
-        <v>-677793.23337257002</v>
+        <v>-677162.844841504</v>
       </c>
     </row>
     <row r="35" spans="2:12" x14ac:dyDescent="0.2">
@@ -20943,7 +20914,7 @@
       </c>
       <c r="C36" s="168">
         <f ca="1">C34/C35</f>
-        <v>-134.85738825558497</v>
+        <v>-134.73196276193872</v>
       </c>
     </row>
     <row r="39" spans="2:12" x14ac:dyDescent="0.2">
@@ -21390,17 +21361,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="E17:I17"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="C39:L39"/>
     <mergeCell ref="C3:G3"/>
     <mergeCell ref="H3:L3"/>
     <mergeCell ref="P3:W3"/>
     <mergeCell ref="X3:Z3"/>
     <mergeCell ref="C5:L5"/>
     <mergeCell ref="P5:Z5"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="E17:I17"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="C39:L39"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -28549,7 +28520,7 @@
       <c r="AA129" s="67"/>
       <c r="AC129" s="62">
         <f ca="1">Overview!C5</f>
-        <v>111.285</v>
+        <v>112.71</v>
       </c>
     </row>
     <row r="130" spans="1:31" x14ac:dyDescent="0.2">
@@ -28596,7 +28567,7 @@
       <c r="AA130" s="67"/>
       <c r="AC130" s="64">
         <f t="shared" ref="AC130" ca="1" si="76">AC129/AC84</f>
-        <v>111.285</v>
+        <v>112.71</v>
       </c>
     </row>
     <row r="132" spans="1:31" x14ac:dyDescent="0.2">
@@ -29444,55 +29415,55 @@
         <v>134</v>
       </c>
       <c r="M159" s="117">
-        <f>M30/M5*365</f>
+        <f t="shared" ref="M159:Q160" si="84">M30/M5*365</f>
         <v>43.680464162785988</v>
       </c>
       <c r="N159" s="117">
-        <f>N30/N5*365</f>
+        <f t="shared" si="84"/>
         <v>23.924651885685286</v>
       </c>
       <c r="O159" s="117">
-        <f>O30/O5*365</f>
+        <f t="shared" si="84"/>
         <v>22.898318211993807</v>
       </c>
       <c r="P159" s="117">
-        <f>P30/P5*365</f>
+        <f t="shared" si="84"/>
         <v>23.906706088397584</v>
       </c>
       <c r="Q159" s="117">
-        <f>Q30/Q5*365</f>
+        <f t="shared" si="84"/>
         <v>26.511929313378616</v>
       </c>
       <c r="T159" s="117">
-        <f t="shared" ref="T159:AA159" si="84">T30/T5*90</f>
+        <f t="shared" ref="T159:AA159" si="85">T30/T5*90</f>
         <v>21.958232681368347</v>
       </c>
       <c r="U159" s="117">
-        <f t="shared" si="84"/>
+        <f t="shared" si="85"/>
         <v>21.144986449864501</v>
       </c>
       <c r="V159" s="117">
-        <f t="shared" si="84"/>
+        <f t="shared" si="85"/>
         <v>21.950911640953716</v>
       </c>
       <c r="W159" s="117">
-        <f t="shared" si="84"/>
+        <f t="shared" si="85"/>
         <v>21.769953422278363</v>
       </c>
       <c r="X159" s="117">
-        <f t="shared" si="84"/>
+        <f t="shared" si="85"/>
         <v>16.517614122404542</v>
       </c>
       <c r="Y159" s="117">
-        <f t="shared" si="84"/>
+        <f t="shared" si="85"/>
         <v>21.107448912326962</v>
       </c>
       <c r="Z159" s="117">
-        <f t="shared" si="84"/>
+        <f t="shared" si="85"/>
         <v>25.267661254936375</v>
       </c>
       <c r="AA159" s="117">
-        <f t="shared" si="84"/>
+        <f t="shared" si="85"/>
         <v>26.952935110849229</v>
       </c>
       <c r="AC159" s="117">
@@ -29505,55 +29476,55 @@
         <v>135</v>
       </c>
       <c r="M160" s="117">
-        <f>M31/M6*365</f>
+        <f t="shared" si="84"/>
         <v>111.71121020193701</v>
       </c>
       <c r="N160" s="117">
-        <f>N31/N6*365</f>
+        <f t="shared" si="84"/>
         <v>133.38012600862163</v>
       </c>
       <c r="O160" s="117">
-        <f>O31/O6*365</f>
+        <f t="shared" si="84"/>
         <v>124.89943721745549</v>
       </c>
       <c r="P160" s="117">
-        <f>P31/P6*365</f>
+        <f t="shared" si="84"/>
         <v>124.51812283253162</v>
       </c>
       <c r="Q160" s="117">
-        <f>Q31/Q6*365</f>
+        <f t="shared" si="84"/>
         <v>122.99350310342828</v>
       </c>
       <c r="T160" s="117">
-        <f t="shared" ref="T160:AA160" si="85">T31/T6*365</f>
+        <f t="shared" ref="T160:AA160" si="86">T31/T6*365</f>
         <v>495.30050687907317</v>
       </c>
       <c r="U160" s="117">
-        <f t="shared" si="85"/>
+        <f t="shared" si="86"/>
         <v>390.06201825108536</v>
       </c>
       <c r="V160" s="117">
-        <f t="shared" si="85"/>
+        <f t="shared" si="86"/>
         <v>513.17081604425994</v>
       </c>
       <c r="W160" s="117">
-        <f t="shared" si="85"/>
+        <f t="shared" si="86"/>
         <v>560.6710444027517</v>
       </c>
       <c r="X160" s="117">
-        <f t="shared" si="85"/>
+        <f t="shared" si="86"/>
         <v>445.70194268541377</v>
       </c>
       <c r="Y160" s="117">
-        <f t="shared" si="85"/>
+        <f t="shared" si="86"/>
         <v>497.15293420272673</v>
       </c>
       <c r="Z160" s="117">
-        <f t="shared" si="85"/>
+        <f t="shared" si="86"/>
         <v>485.6912152101707</v>
       </c>
       <c r="AA160" s="117">
-        <f t="shared" si="85"/>
+        <f t="shared" si="86"/>
         <v>551.09234507897929</v>
       </c>
       <c r="AC160" s="117">
@@ -29586,35 +29557,35 @@
         <v>104.6154069261558</v>
       </c>
       <c r="T161" s="117">
-        <f t="shared" ref="T161:AA161" si="86">T37/T6*90</f>
+        <f t="shared" ref="T161:AA161" si="87">T37/T6*90</f>
         <v>104.46777697320782</v>
       </c>
       <c r="U161" s="117">
-        <f t="shared" si="86"/>
+        <f t="shared" si="87"/>
         <v>88.301585895277753</v>
       </c>
       <c r="V161" s="117">
-        <f t="shared" si="86"/>
+        <f t="shared" si="87"/>
         <v>130.24896265560164</v>
       </c>
       <c r="W161" s="117">
-        <f t="shared" si="86"/>
+        <f t="shared" si="87"/>
         <v>122.65666041275797</v>
       </c>
       <c r="X161" s="117">
-        <f t="shared" si="86"/>
+        <f t="shared" si="87"/>
         <v>103.03101856820865</v>
       </c>
       <c r="Y161" s="117">
-        <f t="shared" si="86"/>
+        <f t="shared" si="87"/>
         <v>109.55779490219324</v>
       </c>
       <c r="Z161" s="117">
-        <f t="shared" si="86"/>
+        <f t="shared" si="87"/>
         <v>101.86462031840568</v>
       </c>
       <c r="AA161" s="117">
-        <f t="shared" si="86"/>
+        <f t="shared" si="87"/>
         <v>78.287970838396106</v>
       </c>
       <c r="AC161" s="117">
@@ -29631,55 +29602,55 @@
         <v>95.814435590545941</v>
       </c>
       <c r="N162" s="117">
-        <f t="shared" ref="N162:Q162" si="87">N159+N160-N161</f>
+        <f t="shared" ref="N162:Q162" si="88">N159+N160-N161</f>
         <v>60.527531293223674</v>
       </c>
       <c r="O162" s="117">
-        <f t="shared" si="87"/>
+        <f t="shared" si="88"/>
         <v>51.577931952498773</v>
       </c>
       <c r="P162" s="117">
-        <f t="shared" si="87"/>
+        <f t="shared" si="88"/>
         <v>20.252214534532527</v>
       </c>
       <c r="Q162" s="117">
-        <f t="shared" si="87"/>
+        <f t="shared" si="88"/>
         <v>44.890025490651112</v>
       </c>
       <c r="T162" s="117">
-        <f t="shared" ref="T162" si="88">T159+T160-T161</f>
+        <f t="shared" ref="T162" si="89">T159+T160-T161</f>
         <v>412.79096258723371</v>
       </c>
       <c r="U162" s="117">
-        <f t="shared" ref="U162" si="89">U159+U160-U161</f>
+        <f t="shared" ref="U162" si="90">U159+U160-U161</f>
         <v>322.90541880567213</v>
       </c>
       <c r="V162" s="117">
-        <f t="shared" ref="V162" si="90">V159+V160-V161</f>
+        <f t="shared" ref="V162" si="91">V159+V160-V161</f>
         <v>404.87276502961197</v>
       </c>
       <c r="W162" s="117">
-        <f t="shared" ref="W162" si="91">W159+W160-W161</f>
+        <f t="shared" ref="W162" si="92">W159+W160-W161</f>
         <v>459.78433741227212</v>
       </c>
       <c r="X162" s="117">
-        <f t="shared" ref="X162" si="92">X159+X160-X161</f>
+        <f t="shared" ref="X162" si="93">X159+X160-X161</f>
         <v>359.18853823960967</v>
       </c>
       <c r="Y162" s="117">
-        <f t="shared" ref="Y162" si="93">Y159+Y160-Y161</f>
+        <f t="shared" ref="Y162" si="94">Y159+Y160-Y161</f>
         <v>408.70258821286052</v>
       </c>
       <c r="Z162" s="117">
-        <f t="shared" ref="Z162:AA162" si="94">Z159+Z160-Z161</f>
+        <f t="shared" ref="Z162:AA162" si="95">Z159+Z160-Z161</f>
         <v>409.09425614670141</v>
       </c>
       <c r="AA162" s="117">
-        <f t="shared" si="94"/>
+        <f t="shared" si="95"/>
         <v>499.75730935143241</v>
       </c>
       <c r="AC162" s="117">
-        <f t="shared" ref="AC162" si="95">AC159+AC160-AC161</f>
+        <f t="shared" ref="AC162" si="96">AC159+AC160-AC161</f>
         <v>82.9857136586363</v>
       </c>
     </row>
@@ -29708,35 +29679,35 @@
         <v>0.40763556496705489</v>
       </c>
       <c r="T163" s="117">
-        <f t="shared" ref="T163:AA163" si="96">T121/T48</f>
+        <f t="shared" ref="T163:AA163" si="97">T121/T48</f>
         <v>0.46020533025540444</v>
       </c>
       <c r="U163" s="117">
-        <f t="shared" si="96"/>
+        <f t="shared" si="97"/>
         <v>0.50472209942531043</v>
       </c>
       <c r="V163" s="117">
-        <f t="shared" si="96"/>
+        <f t="shared" si="97"/>
         <v>0.50378764984386015</v>
       </c>
       <c r="W163" s="117">
-        <f t="shared" si="96"/>
+        <f t="shared" si="97"/>
         <v>0.50273667749308315</v>
       </c>
       <c r="X163" s="117">
-        <f t="shared" si="96"/>
+        <f t="shared" si="97"/>
         <v>0.51854765383161527</v>
       </c>
       <c r="Y163" s="117">
-        <f t="shared" si="96"/>
+        <f t="shared" si="97"/>
         <v>0.43762690832518614</v>
       </c>
       <c r="Z163" s="117">
-        <f t="shared" si="96"/>
+        <f t="shared" si="97"/>
         <v>0.40763556496705489</v>
       </c>
       <c r="AA163" s="117">
-        <f t="shared" si="96"/>
+        <f t="shared" si="97"/>
         <v>0.40424978005996731</v>
       </c>
       <c r="AC163" s="117">
@@ -29769,35 +29740,35 @@
         <v>8.0232059572457368E-2</v>
       </c>
       <c r="T164" s="181">
-        <f t="shared" ref="T164:AA164" si="97">(T121-T120)/T48</f>
+        <f t="shared" ref="T164:AA164" si="98">(T121-T120)/T48</f>
         <v>0.20616337901049214</v>
       </c>
       <c r="U164" s="181">
-        <f t="shared" si="97"/>
+        <f t="shared" si="98"/>
         <v>0.26272957440823053</v>
       </c>
       <c r="V164" s="181">
-        <f t="shared" si="97"/>
+        <f t="shared" si="98"/>
         <v>0.28154528054800038</v>
       </c>
       <c r="W164" s="181">
-        <f t="shared" si="97"/>
+        <f t="shared" si="98"/>
         <v>0.29174185011427883</v>
       </c>
       <c r="X164" s="181">
-        <f t="shared" si="97"/>
+        <f t="shared" si="98"/>
         <v>0.30190124945087504</v>
       </c>
       <c r="Y164" s="181">
-        <f t="shared" si="97"/>
+        <f t="shared" si="98"/>
         <v>0.1468188313153343</v>
       </c>
       <c r="Z164" s="181">
-        <f t="shared" si="97"/>
+        <f t="shared" si="98"/>
         <v>8.0232059572457368E-2</v>
       </c>
       <c r="AA164" s="181">
-        <f t="shared" si="97"/>
+        <f t="shared" si="98"/>
         <v>0.10989819918487531</v>
       </c>
       <c r="AC164" s="181">
@@ -29830,35 +29801,35 @@
         <v>1.306571654790182</v>
       </c>
       <c r="T165" s="117">
-        <f t="shared" ref="T165:AA165" si="98">(T120+T30)/T39</f>
+        <f t="shared" ref="T165:AA165" si="99">(T120+T30)/T39</f>
         <v>1.0117713179504793</v>
       </c>
       <c r="U165" s="117">
-        <f t="shared" si="98"/>
+        <f t="shared" si="99"/>
         <v>0.77382746949571946</v>
       </c>
       <c r="V165" s="117">
-        <f t="shared" si="98"/>
+        <f t="shared" si="99"/>
         <v>0.71608815118039593</v>
       </c>
       <c r="W165" s="117">
-        <f t="shared" si="98"/>
+        <f t="shared" si="99"/>
         <v>0.7494250015540499</v>
       </c>
       <c r="X165" s="117">
-        <f t="shared" si="98"/>
+        <f t="shared" si="99"/>
         <v>0.67396899845564262</v>
       </c>
       <c r="Y165" s="117">
-        <f t="shared" si="98"/>
+        <f t="shared" si="99"/>
         <v>1.0569712357184877</v>
       </c>
       <c r="Z165" s="117">
-        <f t="shared" si="98"/>
+        <f t="shared" si="99"/>
         <v>1.306571654790182</v>
       </c>
       <c r="AA165" s="117">
-        <f t="shared" si="98"/>
+        <f t="shared" si="99"/>
         <v>1.3708387576715642</v>
       </c>
       <c r="AC165" s="117">
@@ -29891,35 +29862,35 @@
         <v>2.0170387965162311</v>
       </c>
       <c r="T166" s="117">
-        <f t="shared" ref="T166:AA166" si="99">T32/T39</f>
+        <f t="shared" ref="T166:AA166" si="100">T32/T39</f>
         <v>1.5870671620819934</v>
       </c>
       <c r="U166" s="117">
-        <f t="shared" si="99"/>
+        <f t="shared" si="100"/>
         <v>1.3122386871071419</v>
       </c>
       <c r="V166" s="117">
-        <f t="shared" si="99"/>
+        <f t="shared" si="100"/>
         <v>1.3268659227275277</v>
       </c>
       <c r="W166" s="117">
-        <f t="shared" si="99"/>
+        <f t="shared" si="100"/>
         <v>1.3095667309007273</v>
       </c>
       <c r="X166" s="117">
-        <f t="shared" si="99"/>
+        <f t="shared" si="100"/>
         <v>1.2404907624549562</v>
       </c>
       <c r="Y166" s="117">
-        <f t="shared" si="99"/>
+        <f t="shared" si="100"/>
         <v>1.6017277146484195</v>
       </c>
       <c r="Z166" s="117">
-        <f t="shared" si="99"/>
+        <f t="shared" si="100"/>
         <v>2.0170387965162311</v>
       </c>
       <c r="AA166" s="117">
-        <f t="shared" si="99"/>
+        <f t="shared" si="100"/>
         <v>2.3119583410823878</v>
       </c>
       <c r="AC166" s="117">
@@ -29952,35 +29923,35 @@
         <v>N/A</v>
       </c>
       <c r="T167" s="183" t="str">
-        <f t="shared" ref="T167:AA167" si="100">IF(T13&gt;=0,"N/A",IF(T12&lt;=0,"N/A",T12/-T13))</f>
+        <f t="shared" ref="T167:AA167" si="101">IF(T13&gt;=0,"N/A",IF(T12&lt;=0,"N/A",T12/-T13))</f>
         <v>N/A</v>
       </c>
       <c r="U167" s="183" t="str">
-        <f t="shared" si="100"/>
+        <f t="shared" si="101"/>
         <v>N/A</v>
       </c>
       <c r="V167" s="183" t="str">
-        <f t="shared" si="100"/>
+        <f t="shared" si="101"/>
         <v>N/A</v>
       </c>
       <c r="W167" s="183" t="str">
-        <f t="shared" si="100"/>
+        <f t="shared" si="101"/>
         <v>N/A</v>
       </c>
       <c r="X167" s="183" t="str">
-        <f t="shared" si="100"/>
+        <f t="shared" si="101"/>
         <v>N/A</v>
       </c>
       <c r="Y167" s="183" t="str">
-        <f t="shared" si="100"/>
+        <f t="shared" si="101"/>
         <v>N/A</v>
       </c>
       <c r="Z167" s="183">
-        <f t="shared" si="100"/>
+        <f t="shared" si="101"/>
         <v>5.9793814432989691</v>
       </c>
       <c r="AA167" s="183" t="str">
-        <f t="shared" si="100"/>
+        <f t="shared" si="101"/>
         <v>N/A</v>
       </c>
       <c r="AC167" s="183" t="str">
@@ -30022,7 +29993,7 @@
       <c r="AA168" s="49"/>
       <c r="AC168" s="71">
         <f ca="1">AC130/Statement!AC26</f>
-        <v>-179.49193548387098</v>
+        <v>-181.79032258064515</v>
       </c>
     </row>
     <row r="169" spans="2:29" x14ac:dyDescent="0.2">
@@ -30059,7 +30030,7 @@
       <c r="AA169" s="49"/>
       <c r="AC169" s="71">
         <f ca="1">AC130/(Statement!AC5/Statement!AC22)</f>
-        <v>9.7399990234919915</v>
+        <v>9.8647193236984538</v>
       </c>
     </row>
     <row r="170" spans="2:29" x14ac:dyDescent="0.2">
@@ -30096,7 +30067,7 @@
       <c r="AA170" s="49"/>
       <c r="AC170" s="71">
         <f ca="1">AC130/(Statement!AC48/Statement!AC74)</f>
-        <v>5.0210820151893278</v>
+        <v>5.085376770741691</v>
       </c>
     </row>
     <row r="171" spans="2:29" x14ac:dyDescent="0.2">
@@ -30133,7 +30104,7 @@
       <c r="AA171" s="49"/>
       <c r="AC171" s="143">
         <f ca="1">Statement!AC130*Statement!AC77</f>
-        <v>559318.41</v>
+        <v>566480.46</v>
       </c>
     </row>
     <row r="172" spans="2:29" x14ac:dyDescent="0.2">
@@ -30170,7 +30141,7 @@
       <c r="AA172" s="49"/>
       <c r="AC172" s="143">
         <f ca="1">AC171+AC121-AC120+AC47+AC44</f>
-        <v>585155.41</v>
+        <v>592317.46</v>
       </c>
     </row>
     <row r="173" spans="2:29" x14ac:dyDescent="0.2">
@@ -30207,7 +30178,7 @@
       <c r="AA173" s="49"/>
       <c r="AC173" s="185">
         <f ca="1">AC172/AC5</f>
-        <v>10.883979874634973</v>
+        <v>11.017195096999794</v>
       </c>
     </row>
     <row r="174" spans="2:29" x14ac:dyDescent="0.2">
@@ -30244,7 +30215,7 @@
       <c r="AA174" s="49"/>
       <c r="AC174" s="185">
         <f ca="1">AC172/AC12</f>
-        <v>-115.89530798177857</v>
+        <v>-117.313816597346</v>
       </c>
     </row>
     <row r="175" spans="2:29" x14ac:dyDescent="0.2">
@@ -30272,35 +30243,35 @@
         <v>-7383</v>
       </c>
       <c r="T175" s="63">
-        <f t="shared" ref="T175:AA175" si="101">T58-T53+T123+T64</f>
+        <f t="shared" ref="T175:AA175" si="102">T58-T53+T123+T64</f>
         <v>0</v>
       </c>
       <c r="U175" s="63">
-        <f t="shared" si="101"/>
+        <f t="shared" si="102"/>
         <v>0</v>
       </c>
       <c r="V175" s="63">
-        <f t="shared" si="101"/>
+        <f t="shared" si="102"/>
         <v>0</v>
       </c>
       <c r="W175" s="63">
-        <f t="shared" si="101"/>
+        <f t="shared" si="102"/>
         <v>-5054</v>
       </c>
       <c r="X175" s="63">
-        <f t="shared" si="101"/>
+        <f t="shared" si="102"/>
         <v>-2164</v>
       </c>
       <c r="Y175" s="63">
-        <f t="shared" si="101"/>
+        <f t="shared" si="102"/>
         <v>-427</v>
       </c>
       <c r="Z175" s="63">
-        <f t="shared" si="101"/>
+        <f t="shared" si="102"/>
         <v>262</v>
       </c>
       <c r="AA175" s="63">
-        <f t="shared" si="101"/>
+        <f t="shared" si="102"/>
         <v>-3161</v>
       </c>
       <c r="AC175" s="63">
@@ -30317,19 +30288,19 @@
         <v>5461.985025111735</v>
       </c>
       <c r="N176" s="63">
-        <f t="shared" ref="N176:Q176" si="102">N122+N52+N123+N54+N56+N57+N55</f>
+        <f t="shared" ref="N176:Q176" si="103">N122+N52+N123+N54+N56+N57+N55</f>
         <v>-13983</v>
       </c>
       <c r="O176" s="63">
-        <f t="shared" si="102"/>
+        <f t="shared" si="103"/>
         <v>-16624</v>
       </c>
       <c r="P176" s="63">
-        <f t="shared" si="102"/>
+        <f t="shared" si="103"/>
         <v>-23140</v>
       </c>
       <c r="Q176" s="63">
-        <f t="shared" si="102"/>
+        <f t="shared" si="103"/>
         <v>-6901</v>
       </c>
       <c r="T176" s="49"/>
@@ -30354,19 +30325,19 @@
         <v>24.234480257856571</v>
       </c>
       <c r="N177" s="71">
-        <f t="shared" ref="N177:Q177" si="103">N171/N175</f>
+        <f t="shared" ref="N177:Q177" si="104">N171/N175</f>
         <v>-8.7516835473323233</v>
       </c>
       <c r="O177" s="71">
-        <f t="shared" si="103"/>
+        <f t="shared" si="104"/>
         <v>-12.197995202193283</v>
       </c>
       <c r="P177" s="71">
-        <f t="shared" si="103"/>
+        <f t="shared" si="104"/>
         <v>-4.6102486100912623</v>
       </c>
       <c r="Q177" s="71">
-        <f t="shared" si="103"/>
+        <f t="shared" si="104"/>
         <v>-24.491263713937425</v>
       </c>
       <c r="T177" s="49"/>
@@ -30378,8 +30349,8 @@
       <c r="Z177" s="49"/>
       <c r="AA177" s="49"/>
       <c r="AC177" s="71">
-        <f t="shared" ref="AC177:AC178" ca="1" si="104">AC171/AC175</f>
-        <v>-101.8794918032787</v>
+        <f t="shared" ref="AC177:AC178" ca="1" si="105">AC171/AC175</f>
+        <v>-103.18405464480874</v>
       </c>
     </row>
     <row r="178" spans="2:29" x14ac:dyDescent="0.2">
@@ -30391,19 +30362,19 @@
         <v>40.317380766801932</v>
       </c>
       <c r="N178" s="71">
-        <f t="shared" ref="N178:Q178" si="105">N172/N176</f>
+        <f t="shared" ref="N178:Q178" si="106">N172/N176</f>
         <v>-8.9618365157691464</v>
       </c>
       <c r="O178" s="71">
-        <f t="shared" si="105"/>
+        <f t="shared" si="106"/>
         <v>-14.56746270452358</v>
       </c>
       <c r="P178" s="71">
-        <f t="shared" si="105"/>
+        <f t="shared" si="106"/>
         <v>-5.255401901469317</v>
       </c>
       <c r="Q178" s="71">
-        <f t="shared" si="105"/>
+        <f t="shared" si="106"/>
         <v>-29.280828865381828</v>
       </c>
       <c r="T178" s="49"/>
@@ -30415,8 +30386,8 @@
       <c r="Z178" s="49"/>
       <c r="AA178" s="49"/>
       <c r="AC178" s="71">
-        <f t="shared" ca="1" si="104"/>
-        <v>-68.255617636766601</v>
+        <f t="shared" ca="1" si="105"/>
+        <v>-69.091036976554292</v>
       </c>
     </row>
     <row r="179" spans="2:29" x14ac:dyDescent="0.2">
@@ -30428,19 +30399,19 @@
         <v>4.1263521617131038E-2</v>
       </c>
       <c r="N179" s="73">
-        <f t="shared" ref="N179:Q179" si="106">N175/N171</f>
+        <f t="shared" ref="N179:Q179" si="107">N175/N171</f>
         <v>-0.11426372932609277</v>
       </c>
       <c r="O179" s="73">
-        <f t="shared" si="106"/>
+        <f t="shared" si="107"/>
         <v>-8.1980684811237922E-2</v>
       </c>
       <c r="P179" s="73">
-        <f t="shared" si="106"/>
+        <f t="shared" si="107"/>
         <v>-0.21690804218478027</v>
       </c>
       <c r="Q179" s="73">
-        <f t="shared" si="106"/>
+        <f t="shared" si="107"/>
         <v>-4.0830886134753538E-2</v>
       </c>
       <c r="T179" s="49"/>
@@ -30452,8 +30423,8 @@
       <c r="Z179" s="49"/>
       <c r="AA179" s="49"/>
       <c r="AC179" s="73">
-        <f t="shared" ref="AC179" ca="1" si="107">AC175/AC171</f>
-        <v>-9.8155181410889015E-3</v>
+        <f t="shared" ref="AC179" ca="1" si="108">AC175/AC171</f>
+        <v>-9.6914198946950452E-3</v>
       </c>
     </row>
     <row r="180" spans="2:29" x14ac:dyDescent="0.2">
@@ -30465,19 +30436,19 @@
         <v>9.471837848372637E-2</v>
       </c>
       <c r="N180" s="73">
-        <f t="shared" ref="N180:Q180" si="108">N26/N130</f>
+        <f t="shared" ref="N180:Q180" si="109">N26/N130</f>
         <v>7.3401437760121077E-2</v>
       </c>
       <c r="O180" s="73">
-        <f t="shared" si="108"/>
+        <f t="shared" si="109"/>
         <v>7.9601990049751256E-3</v>
       </c>
       <c r="P180" s="73">
-        <f t="shared" si="108"/>
+        <f t="shared" si="109"/>
         <v>-0.21576354679802953</v>
       </c>
       <c r="Q180" s="73">
-        <f t="shared" si="108"/>
+        <f t="shared" si="109"/>
         <v>-1.6574585635359114E-3</v>
       </c>
       <c r="T180" s="49"/>
@@ -30489,8 +30460,8 @@
       <c r="Z180" s="49"/>
       <c r="AA180" s="49"/>
       <c r="AC180" s="73">
-        <f t="shared" ref="AC180" ca="1" si="109">AC26/AC130</f>
-        <v>-5.5712809453205732E-3</v>
+        <f t="shared" ref="AC180" ca="1" si="110">AC26/AC130</f>
+        <v>-5.5008428710850857E-3</v>
       </c>
     </row>
     <row r="181" spans="2:29" x14ac:dyDescent="0.2">
@@ -30502,19 +30473,19 @@
         <v>2.7090235821477293E-2</v>
       </c>
       <c r="N181" s="154">
-        <f t="shared" ref="N181:Q181" si="110">N81/N130</f>
+        <f t="shared" ref="N181:Q181" si="111">N81/N130</f>
         <v>5.5240257283390083E-2</v>
       </c>
       <c r="O181" s="154">
-        <f t="shared" si="110"/>
+        <f t="shared" si="111"/>
         <v>1.472636815920398E-2</v>
       </c>
       <c r="P181" s="154">
-        <f t="shared" si="110"/>
+        <f t="shared" si="111"/>
         <v>1.8719211822660099E-2</v>
       </c>
       <c r="Q181" s="154">
-        <f t="shared" si="110"/>
+        <f t="shared" si="111"/>
         <v>0</v>
       </c>
       <c r="T181" s="49"/>
@@ -30526,7 +30497,7 @@
       <c r="Z181" s="49"/>
       <c r="AA181" s="49"/>
       <c r="AC181" s="154">
-        <f t="shared" ref="AC181" ca="1" si="111">AC81/AC130</f>
+        <f t="shared" ref="AC181" ca="1" si="112">AC81/AC130</f>
         <v>0</v>
       </c>
     </row>
@@ -30814,35 +30785,35 @@
         <v>7.4906906906906903</v>
       </c>
       <c r="T189" s="71">
-        <f t="shared" ref="T189:AA189" si="112">T120/T74</f>
+        <f t="shared" ref="T189:AA189" si="113">T120/T74</f>
         <v>6.8458840037418147</v>
       </c>
       <c r="U189" s="71">
-        <f t="shared" si="112"/>
+        <f t="shared" si="113"/>
         <v>5.5845119406445631</v>
       </c>
       <c r="V189" s="71">
-        <f t="shared" si="112"/>
+        <f t="shared" si="113"/>
         <v>5.0951501154734409</v>
       </c>
       <c r="W189" s="71">
-        <f t="shared" si="112"/>
+        <f t="shared" si="113"/>
         <v>4.825309491059147</v>
       </c>
       <c r="X189" s="71">
-        <f t="shared" si="112"/>
+        <f t="shared" si="113"/>
         <v>4.8448709161526162</v>
       </c>
       <c r="Y189" s="71">
-        <f t="shared" si="112"/>
+        <f t="shared" si="113"/>
         <v>6.4853249475890982</v>
       </c>
       <c r="Z189" s="71">
-        <f t="shared" si="112"/>
+        <f t="shared" si="113"/>
         <v>7.4906906906906903</v>
       </c>
       <c r="AA189" s="71">
-        <f t="shared" si="112"/>
+        <f t="shared" si="113"/>
         <v>6.5238758456028654</v>
       </c>
       <c r="AC189" s="71">
@@ -30875,27 +30846,27 @@
         <v>0.25100546560791998</v>
       </c>
       <c r="T190" s="154" t="e">
-        <f t="shared" ref="T190:Y190" si="113">T53/T58</f>
+        <f t="shared" ref="T190:Y190" si="114">T53/T58</f>
         <v>#DIV/0!</v>
       </c>
       <c r="U190" s="154" t="e">
-        <f t="shared" si="113"/>
+        <f t="shared" si="114"/>
         <v>#DIV/0!</v>
       </c>
       <c r="V190" s="154" t="e">
-        <f t="shared" si="113"/>
+        <f t="shared" si="114"/>
         <v>#DIV/0!</v>
       </c>
       <c r="W190" s="154">
-        <f t="shared" si="113"/>
+        <f t="shared" si="114"/>
         <v>0.84132841328413288</v>
       </c>
       <c r="X190" s="154">
-        <f t="shared" si="113"/>
+        <f t="shared" si="114"/>
         <v>0.32390243902439025</v>
       </c>
       <c r="Y190" s="154">
-        <f t="shared" si="113"/>
+        <f t="shared" si="114"/>
         <v>0.2152395915161037</v>
       </c>
       <c r="Z190" s="154">
@@ -30936,27 +30907,27 @@
         <v>4.6052258149963103E-2</v>
       </c>
       <c r="T191" s="154">
-        <f t="shared" ref="T191:Y191" si="114">T53/T5</f>
+        <f t="shared" ref="T191:Y191" si="115">T53/T5</f>
         <v>0</v>
       </c>
       <c r="U191" s="154">
-        <f t="shared" si="114"/>
+        <f t="shared" si="115"/>
         <v>0</v>
       </c>
       <c r="V191" s="154">
-        <f t="shared" si="114"/>
+        <f t="shared" si="115"/>
         <v>0</v>
       </c>
       <c r="W191" s="154">
-        <f t="shared" si="114"/>
+        <f t="shared" si="115"/>
         <v>5.3998578984763561E-2</v>
       </c>
       <c r="X191" s="154">
-        <f t="shared" si="114"/>
+        <f t="shared" si="115"/>
         <v>5.1636985768722297E-2</v>
       </c>
       <c r="Y191" s="154">
-        <f t="shared" si="114"/>
+        <f t="shared" si="115"/>
         <v>4.0137698674284038E-2</v>
       </c>
       <c r="Z191" s="154">
@@ -30997,35 +30968,35 @@
         <v>-1.8356356356356356</v>
       </c>
       <c r="T192" s="71">
-        <f t="shared" ref="T192:AA192" si="115">(T120-T121)/T74</f>
+        <f t="shared" ref="T192:AA192" si="116">(T120-T121)/T74</f>
         <v>-5.5556594948550044</v>
       </c>
       <c r="U192" s="71">
-        <f t="shared" si="115"/>
+        <f t="shared" si="116"/>
         <v>-6.06306515186645</v>
       </c>
       <c r="V192" s="71">
-        <f t="shared" si="115"/>
+        <f t="shared" si="116"/>
         <v>-6.4547344110854503</v>
       </c>
       <c r="W192" s="71">
-        <f t="shared" si="115"/>
+        <f t="shared" si="116"/>
         <v>-6.6719394773039893</v>
       </c>
       <c r="X192" s="71">
-        <f t="shared" si="115"/>
+        <f t="shared" si="116"/>
         <v>-6.7514279186657529</v>
       </c>
       <c r="Y192" s="71">
-        <f t="shared" si="115"/>
+        <f t="shared" si="116"/>
         <v>-3.2742138364779874</v>
       </c>
       <c r="Z192" s="71">
-        <f t="shared" si="115"/>
+        <f t="shared" si="116"/>
         <v>-1.8356356356356356</v>
       </c>
       <c r="AA192" s="71">
-        <f t="shared" si="115"/>
+        <f t="shared" si="116"/>
         <v>-2.435734182252288</v>
       </c>
       <c r="AC192" s="71">
@@ -31067,7 +31038,7 @@
       <c r="AA193" s="49"/>
       <c r="AC193" s="154">
         <f ca="1">(AC120-AC121)/AC171</f>
-        <v>-2.1887353931368002E-2</v>
+        <v>-2.1610630665001226E-2</v>
       </c>
     </row>
     <row r="194" spans="2:29" x14ac:dyDescent="0.2">
@@ -31095,35 +31066,35 @@
         <v>0.27710820577829071</v>
       </c>
       <c r="T194" s="154">
-        <f t="shared" ref="T194:AA194" si="116">-T123/T5</f>
+        <f t="shared" ref="T194:AA194" si="117">-T123/T5</f>
         <v>0</v>
       </c>
       <c r="U194" s="154">
-        <f t="shared" si="116"/>
+        <f t="shared" si="117"/>
         <v>0</v>
       </c>
       <c r="V194" s="154">
-        <f t="shared" si="116"/>
+        <f t="shared" si="117"/>
         <v>0</v>
       </c>
       <c r="W194" s="154">
-        <f t="shared" si="116"/>
+        <f t="shared" si="117"/>
         <v>0.40917344280413676</v>
       </c>
       <c r="X194" s="154">
-        <f t="shared" si="116"/>
+        <f t="shared" si="117"/>
         <v>0.27607123415506651</v>
       </c>
       <c r="Y194" s="154">
-        <f t="shared" si="116"/>
+        <f t="shared" si="117"/>
         <v>0.17761664103127517</v>
       </c>
       <c r="Z194" s="154">
-        <f t="shared" si="116"/>
+        <f t="shared" si="117"/>
         <v>0.25508263858417435</v>
       </c>
       <c r="AA194" s="154">
-        <f t="shared" si="116"/>
+        <f t="shared" si="117"/>
         <v>0.2678058481255064</v>
       </c>
       <c r="AC194" s="154">
@@ -31156,27 +31127,27 @@
         <v>1.5103640301124059</v>
       </c>
       <c r="T195" s="154" t="e">
-        <f t="shared" ref="T195:Y195" si="117">-(T123/T58)</f>
+        <f t="shared" ref="T195:Y195" si="118">-(T123/T58)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="U195" s="154" t="e">
-        <f t="shared" si="117"/>
+        <f t="shared" si="118"/>
         <v>#DIV/0!</v>
       </c>
       <c r="V195" s="154" t="e">
-        <f t="shared" si="117"/>
+        <f t="shared" si="118"/>
         <v>#DIV/0!</v>
       </c>
       <c r="W195" s="154">
-        <f t="shared" si="117"/>
+        <f t="shared" si="118"/>
         <v>6.375153751537515</v>
       </c>
       <c r="X195" s="154">
-        <f t="shared" si="117"/>
+        <f t="shared" si="118"/>
         <v>1.7317073170731707</v>
       </c>
       <c r="Y195" s="154">
-        <f t="shared" si="117"/>
+        <f t="shared" si="118"/>
         <v>0.95247446975648076</v>
       </c>
       <c r="Z195" s="154">
@@ -31217,27 +31188,27 @@
         <v>1.2511532547411583</v>
       </c>
       <c r="T196" s="154" t="e">
-        <f t="shared" ref="T196:Y196" si="118">-T123/T52</f>
+        <f t="shared" ref="T196:Y196" si="119">-T123/T52</f>
         <v>#DIV/0!</v>
       </c>
       <c r="U196" s="154" t="e">
-        <f t="shared" si="118"/>
+        <f t="shared" si="119"/>
         <v>#DIV/0!</v>
       </c>
       <c r="V196" s="154" t="e">
-        <f t="shared" si="118"/>
+        <f t="shared" si="119"/>
         <v>#DIV/0!</v>
       </c>
       <c r="W196" s="154">
-        <f t="shared" si="118"/>
+        <f t="shared" si="119"/>
         <v>1.9382946896035902</v>
       </c>
       <c r="X196" s="154">
-        <f t="shared" si="118"/>
+        <f t="shared" si="119"/>
         <v>1.1782276800531033</v>
       </c>
       <c r="Y196" s="154">
-        <f t="shared" si="118"/>
+        <f t="shared" si="119"/>
         <v>0.81049465240641716</v>
       </c>
       <c r="Z196" s="154">
@@ -31300,61 +31271,61 @@
       <c r="K200" s="80"/>
       <c r="L200" s="80"/>
       <c r="M200" s="80">
-        <f t="shared" ref="M200:Q204" si="119">IF(L105=0,
+        <f t="shared" ref="M200:Q204" si="120">IF(L105=0,
 IF(M105=0,0,IF(M105&gt;0,1,-1)),
 (M105-L105)/ABS(L105)
 )</f>
         <v>1</v>
       </c>
       <c r="N200" s="80">
-        <f t="shared" si="119"/>
+        <f t="shared" si="120"/>
         <v>-0.22657676298045326</v>
       </c>
       <c r="O200" s="80">
-        <f t="shared" si="119"/>
+        <f t="shared" si="120"/>
         <v>-7.9155257608661447E-2</v>
       </c>
       <c r="P200" s="80">
-        <f t="shared" si="119"/>
+        <f t="shared" si="120"/>
         <v>0.139722469068289</v>
       </c>
       <c r="Q200" s="80">
-        <f t="shared" si="119"/>
+        <f t="shared" si="120"/>
         <v>-3.3527259641336293E-2</v>
       </c>
       <c r="T200" s="80">
-        <f t="shared" ref="T200:AA204" si="120">IF(S105=0,
+        <f t="shared" ref="T200:AA204" si="121">IF(S105=0,
 IF(T105=0,0,IF(T105&gt;0,1,-1)),
 (T105-S105)/ABS(S105)
 )</f>
         <v>1</v>
       </c>
       <c r="U200" s="80">
-        <f t="shared" si="120"/>
+        <f t="shared" si="121"/>
         <v>2.2104875353063983E-3</v>
       </c>
       <c r="V200" s="80">
-        <f t="shared" si="120"/>
+        <f t="shared" si="121"/>
         <v>7.4500673937017522E-2</v>
       </c>
       <c r="W200" s="80">
-        <f t="shared" si="120"/>
+        <f t="shared" si="121"/>
         <v>-0.13000342114266164</v>
       </c>
       <c r="X200" s="80">
-        <f t="shared" si="120"/>
+        <f t="shared" si="121"/>
         <v>3.1721064359680168E-2</v>
       </c>
       <c r="Y200" s="80">
-        <f t="shared" si="120"/>
+        <f t="shared" si="121"/>
         <v>8.436030999872951E-2</v>
       </c>
       <c r="Z200" s="80">
-        <f t="shared" si="120"/>
+        <f t="shared" si="121"/>
         <v>-4.0070298769771528E-2</v>
       </c>
       <c r="AA200" s="80">
-        <f t="shared" si="120"/>
+        <f t="shared" si="121"/>
         <v>-5.687782253142927E-2</v>
       </c>
       <c r="AC200" s="49"/>
@@ -31364,55 +31335,55 @@
         <v>363</v>
       </c>
       <c r="M201" s="80">
-        <f t="shared" si="119"/>
-        <v>1</v>
-      </c>
-      <c r="N201" s="80">
-        <f t="shared" si="119"/>
-        <v>-8.4923946253162061E-2</v>
-      </c>
-      <c r="O201" s="80">
-        <f t="shared" si="119"/>
-        <v>-0.23547784878293962</v>
-      </c>
-      <c r="P201" s="80">
-        <f t="shared" si="119"/>
-        <v>-0.242779995304062</v>
-      </c>
-      <c r="Q201" s="80">
-        <f t="shared" si="119"/>
-        <v>4.9240310077519382E-2</v>
-      </c>
-      <c r="T201" s="80">
         <f t="shared" si="120"/>
         <v>1</v>
       </c>
+      <c r="N201" s="80">
+        <f t="shared" si="120"/>
+        <v>-8.4923946253162061E-2</v>
+      </c>
+      <c r="O201" s="80">
+        <f t="shared" si="120"/>
+        <v>-0.23547784878293962</v>
+      </c>
+      <c r="P201" s="80">
+        <f t="shared" si="120"/>
+        <v>-0.242779995304062</v>
+      </c>
+      <c r="Q201" s="80">
+        <f t="shared" si="120"/>
+        <v>4.9240310077519382E-2</v>
+      </c>
+      <c r="T201" s="80">
+        <f t="shared" si="121"/>
+        <v>1</v>
+      </c>
       <c r="U201" s="80">
-        <f t="shared" si="120"/>
+        <f t="shared" si="121"/>
         <v>8.8304862023653091E-2</v>
       </c>
       <c r="V201" s="80">
-        <f t="shared" si="120"/>
+        <f t="shared" si="121"/>
         <v>5.0712388312001935E-2</v>
       </c>
       <c r="W201" s="80">
-        <f t="shared" si="120"/>
+        <f t="shared" si="121"/>
         <v>-5.1712250057458053E-2</v>
       </c>
       <c r="X201" s="80">
-        <f t="shared" si="120"/>
+        <f t="shared" si="121"/>
         <v>-4.5322346097915654E-2</v>
       </c>
       <c r="Y201" s="80">
-        <f t="shared" si="120"/>
+        <f t="shared" si="121"/>
         <v>4.5189134298045192E-2</v>
       </c>
       <c r="Z201" s="80">
-        <f t="shared" si="120"/>
+        <f t="shared" si="121"/>
         <v>0.15059509351469516</v>
       </c>
       <c r="AA201" s="80">
-        <f t="shared" si="120"/>
+        <f t="shared" si="121"/>
         <v>6.6497783407219763E-2</v>
       </c>
       <c r="AC201" s="49"/>
@@ -31422,55 +31393,55 @@
         <v>364</v>
       </c>
       <c r="M202" s="80">
-        <f t="shared" si="119"/>
-        <v>1</v>
-      </c>
-      <c r="N202" s="80">
-        <f t="shared" si="119"/>
-        <v>-0.16628914988814317</v>
-      </c>
-      <c r="O202" s="80">
-        <f t="shared" si="119"/>
-        <v>-0.1521793818236705</v>
-      </c>
-      <c r="P202" s="80">
-        <f t="shared" si="119"/>
-        <v>-2.1403279726227919E-2</v>
-      </c>
-      <c r="Q202" s="80">
-        <f t="shared" si="119"/>
-        <v>-6.5492915041135214E-3</v>
-      </c>
-      <c r="T202" s="80">
         <f t="shared" si="120"/>
         <v>1</v>
       </c>
+      <c r="N202" s="80">
+        <f t="shared" si="120"/>
+        <v>-0.16628914988814317</v>
+      </c>
+      <c r="O202" s="80">
+        <f t="shared" si="120"/>
+        <v>-0.1521793818236705</v>
+      </c>
+      <c r="P202" s="80">
+        <f t="shared" si="120"/>
+        <v>-2.1403279726227919E-2</v>
+      </c>
+      <c r="Q202" s="80">
+        <f t="shared" si="120"/>
+        <v>-6.5492915041135214E-3</v>
+      </c>
+      <c r="T202" s="80">
+        <f t="shared" si="121"/>
+        <v>1</v>
+      </c>
       <c r="U202" s="80">
-        <f t="shared" si="120"/>
+        <f t="shared" si="121"/>
         <v>2.9628389688650822E-2</v>
       </c>
       <c r="V202" s="80">
-        <f t="shared" si="120"/>
+        <f t="shared" si="121"/>
         <v>6.6493253129572424E-2</v>
       </c>
       <c r="W202" s="80">
-        <f t="shared" si="120"/>
+        <f t="shared" si="121"/>
         <v>-0.10403963414634146</v>
       </c>
       <c r="X202" s="80">
-        <f t="shared" si="120"/>
+        <f t="shared" si="121"/>
         <v>4.6788600595491277E-3</v>
       </c>
       <c r="Y202" s="80">
-        <f t="shared" si="120"/>
+        <f t="shared" si="121"/>
         <v>7.1295512277730733E-2</v>
       </c>
       <c r="Z202" s="80">
-        <f t="shared" si="120"/>
+        <f t="shared" si="121"/>
         <v>2.1972810622826432E-2</v>
       </c>
       <c r="AA202" s="80">
-        <f t="shared" si="120"/>
+        <f t="shared" si="121"/>
         <v>-1.1678267594740912E-2</v>
       </c>
       <c r="AC202" s="49"/>
@@ -31480,55 +31451,55 @@
         <v>365</v>
       </c>
       <c r="M203" s="80">
-        <f t="shared" si="119"/>
-        <v>1</v>
-      </c>
-      <c r="N203" s="80">
-        <f t="shared" si="119"/>
-        <v>0.35158501440922191</v>
-      </c>
-      <c r="O203" s="80">
-        <f t="shared" si="119"/>
-        <v>1.0298507462686568</v>
-      </c>
-      <c r="P203" s="80">
-        <f t="shared" si="119"/>
-        <v>17.190126050420169</v>
-      </c>
-      <c r="Q203" s="80">
-        <f t="shared" si="119"/>
-        <v>2.9393081942599757E-2</v>
-      </c>
-      <c r="T203" s="80">
         <f t="shared" si="120"/>
         <v>1</v>
       </c>
+      <c r="N203" s="80">
+        <f t="shared" si="120"/>
+        <v>0.35158501440922191</v>
+      </c>
+      <c r="O203" s="80">
+        <f t="shared" si="120"/>
+        <v>1.0298507462686568</v>
+      </c>
+      <c r="P203" s="80">
+        <f t="shared" si="120"/>
+        <v>17.190126050420169</v>
+      </c>
+      <c r="Q203" s="80">
+        <f t="shared" si="120"/>
+        <v>2.9393081942599757E-2</v>
+      </c>
+      <c r="T203" s="80">
+        <f t="shared" si="121"/>
+        <v>1</v>
+      </c>
       <c r="U203" s="80">
-        <f t="shared" si="120"/>
+        <f t="shared" si="121"/>
         <v>1.3311536665109761E-2</v>
       </c>
       <c r="V203" s="80">
-        <f t="shared" si="120"/>
+        <f t="shared" si="121"/>
         <v>2.3046784973496196E-4</v>
       </c>
       <c r="W203" s="80">
-        <f t="shared" si="120"/>
+        <f t="shared" si="121"/>
         <v>7.5345622119815672E-2</v>
       </c>
       <c r="X203" s="80">
-        <f t="shared" si="120"/>
+        <f t="shared" si="121"/>
         <v>-5.3567602314120423E-2</v>
       </c>
       <c r="Y203" s="80">
-        <f t="shared" si="120"/>
+        <f t="shared" si="121"/>
         <v>-4.1204437400950873E-2</v>
       </c>
       <c r="Z203" s="80">
-        <f t="shared" si="120"/>
+        <f t="shared" si="121"/>
         <v>6.4226682408500588E-2</v>
       </c>
       <c r="AA203" s="80">
-        <f t="shared" si="120"/>
+        <f t="shared" si="121"/>
         <v>0.2027956512092301</v>
       </c>
       <c r="AC203" s="49"/>
@@ -31538,55 +31509,55 @@
         <v>366</v>
       </c>
       <c r="M204" s="80">
-        <f t="shared" si="119"/>
-        <v>1</v>
-      </c>
-      <c r="N204" s="80">
-        <f t="shared" si="119"/>
-        <v>-0.58669833729216148</v>
-      </c>
-      <c r="O204" s="80">
-        <f t="shared" si="119"/>
-        <v>-7.9445571331981074E-2</v>
-      </c>
-      <c r="P204" s="80">
-        <f t="shared" si="119"/>
-        <v>0.32243848696290855</v>
-      </c>
-      <c r="Q204" s="80">
-        <f t="shared" si="119"/>
-        <v>-1.0552624271035824E-2</v>
-      </c>
-      <c r="T204" s="80">
         <f t="shared" si="120"/>
         <v>1</v>
       </c>
+      <c r="N204" s="80">
+        <f t="shared" si="120"/>
+        <v>-0.58669833729216148</v>
+      </c>
+      <c r="O204" s="80">
+        <f t="shared" si="120"/>
+        <v>-7.9445571331981074E-2</v>
+      </c>
+      <c r="P204" s="80">
+        <f t="shared" si="120"/>
+        <v>0.32243848696290855</v>
+      </c>
+      <c r="Q204" s="80">
+        <f t="shared" si="120"/>
+        <v>-1.0552624271035824E-2</v>
+      </c>
+      <c r="T204" s="80">
+        <f t="shared" si="121"/>
+        <v>1</v>
+      </c>
       <c r="U204" s="80">
-        <f t="shared" si="120"/>
+        <f t="shared" si="121"/>
         <v>9.4211123723041995E-2</v>
       </c>
       <c r="V204" s="80">
-        <f t="shared" si="120"/>
+        <f t="shared" si="121"/>
         <v>0.1545643153526971</v>
       </c>
       <c r="W204" s="80">
-        <f t="shared" si="120"/>
+        <f t="shared" si="121"/>
         <v>-0.1527403414195867</v>
       </c>
       <c r="X204" s="80">
-        <f t="shared" si="120"/>
+        <f t="shared" si="121"/>
         <v>0.11664899257688228</v>
       </c>
       <c r="Y204" s="80">
-        <f t="shared" si="120"/>
+        <f t="shared" si="121"/>
         <v>-5.6980056980056981E-2</v>
       </c>
       <c r="Z204" s="80">
-        <f t="shared" si="120"/>
+        <f t="shared" si="121"/>
         <v>-0.42195367573011078</v>
       </c>
       <c r="AA204" s="80">
-        <f t="shared" si="120"/>
+        <f t="shared" si="121"/>
         <v>9.4076655052264813E-2</v>
       </c>
       <c r="AC204" s="49"/>
@@ -31749,7 +31720,7 @@
       </c>
       <c r="C5" s="174">
         <f ca="1">Overview!C5</f>
-        <v>111.285</v>
+        <v>112.71</v>
       </c>
       <c r="E5" s="12"/>
       <c r="F5" s="131" t="s">
@@ -31765,7 +31736,7 @@
       </c>
       <c r="C6" s="175">
         <f ca="1">Statement!AC171</f>
-        <v>559318.41</v>
+        <v>566480.46</v>
       </c>
       <c r="E6" s="20" t="s">
         <v>19</v>
@@ -31785,7 +31756,7 @@
       </c>
       <c r="C7" s="175">
         <f ca="1">Statement!AC172</f>
-        <v>585155.41</v>
+        <v>592317.46</v>
       </c>
       <c r="E7" s="20" t="s">
         <v>29</v>
@@ -31805,7 +31776,7 @@
       </c>
       <c r="C8" s="176">
         <f ca="1">Statement!AC168</f>
-        <v>-179.49193548387098</v>
+        <v>-181.79032258064515</v>
       </c>
       <c r="E8" s="20" t="s">
         <v>246</v>
@@ -31825,7 +31796,7 @@
       </c>
       <c r="C9" s="176">
         <f ca="1">Statement!AC169</f>
-        <v>9.7399990234919915</v>
+        <v>9.8647193236984538</v>
       </c>
       <c r="E9" s="20" t="s">
         <v>247</v>
@@ -31845,7 +31816,7 @@
       </c>
       <c r="C10" s="176">
         <f ca="1">Statement!AC170</f>
-        <v>5.0210820151893278</v>
+        <v>5.085376770741691</v>
       </c>
       <c r="E10" s="20" t="s">
         <v>1</v>
@@ -31865,7 +31836,7 @@
       </c>
       <c r="C11" s="176">
         <f ca="1">Statement!AC173</f>
-        <v>10.883979874634973</v>
+        <v>11.017195096999794</v>
       </c>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.2">
@@ -31874,7 +31845,7 @@
       </c>
       <c r="C12" s="176">
         <f ca="1">Statement!AC174</f>
-        <v>-115.89530798177857</v>
+        <v>-117.313816597346</v>
       </c>
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.2">
@@ -32110,7 +32081,7 @@
       </c>
       <c r="C38" s="177">
         <f ca="1">Statement!AC180</f>
-        <v>-5.5712809453205732E-3</v>
+        <v>-5.5008428710850857E-3</v>
       </c>
       <c r="E38" s="20" t="s">
         <v>274</v>
@@ -32126,7 +32097,7 @@
       </c>
       <c r="C39" s="217">
         <f ca="1">Statement!AC179</f>
-        <v>-9.8155181410889015E-3</v>
+        <v>-9.6914198946950452E-3</v>
       </c>
       <c r="E39" s="20" t="s">
         <v>276</v>
@@ -32211,7 +32182,7 @@
       </c>
       <c r="F48" s="177">
         <f ca="1">Statement!AC193</f>
-        <v>-2.1887353931368002E-2</v>
+        <v>-2.1610630665001226E-2</v>
       </c>
     </row>
     <row r="51" spans="2:6" x14ac:dyDescent="0.2">
@@ -32390,7 +32361,7 @@
       </c>
       <c r="I6" s="174">
         <f ca="1">Statement!AC129</f>
-        <v>111.285</v>
+        <v>112.71</v>
       </c>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.2">
@@ -32419,7 +32390,7 @@
       </c>
       <c r="I7" s="175">
         <f ca="1">Statement!AC171</f>
-        <v>559318.41</v>
+        <v>566480.46</v>
       </c>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.2">
@@ -32448,7 +32419,7 @@
       </c>
       <c r="I8" s="175">
         <f ca="1">Statement!AC172</f>
-        <v>585155.41</v>
+        <v>592317.46</v>
       </c>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.2">
@@ -32477,7 +32448,7 @@
       </c>
       <c r="I9" s="176">
         <f ca="1">Statement!AC168</f>
-        <v>-179.49193548387098</v>
+        <v>-181.79032258064515</v>
       </c>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.2">
@@ -32506,7 +32477,7 @@
       </c>
       <c r="I10" s="176">
         <f ca="1">Statement!AC169</f>
-        <v>9.7399990234919915</v>
+        <v>9.8647193236984538</v>
       </c>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.2">
@@ -32535,7 +32506,7 @@
       </c>
       <c r="I11" s="176">
         <f ca="1">Statement!AC170</f>
-        <v>5.0210820151893278</v>
+        <v>5.085376770741691</v>
       </c>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.2">
@@ -32564,7 +32535,7 @@
       </c>
       <c r="I12" s="176">
         <f ca="1">Statement!AC173</f>
-        <v>10.883979874634973</v>
+        <v>11.017195096999794</v>
       </c>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.2">
@@ -32593,7 +32564,7 @@
       </c>
       <c r="I13" s="176">
         <f ca="1">Statement!AC174</f>
-        <v>-115.89530798177857</v>
+        <v>-117.313816597346</v>
       </c>
     </row>
     <row r="15" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -33366,7 +33337,7 @@
       </c>
       <c r="I51" s="177">
         <f ca="1">Statement!AC180</f>
-        <v>-5.5712809453205732E-3</v>
+        <v>-5.5008428710850857E-3</v>
       </c>
     </row>
     <row r="52" spans="2:9" x14ac:dyDescent="0.2">
@@ -33395,7 +33366,7 @@
       </c>
       <c r="I52" s="177">
         <f ca="1">Statement!AC179</f>
-        <v>-9.8155181410889015E-3</v>
+        <v>-9.6914198946950452E-3</v>
       </c>
     </row>
     <row r="53" spans="2:9" x14ac:dyDescent="0.2">
@@ -33718,7 +33689,7 @@
       </c>
       <c r="I68" s="198">
         <f ca="1">Statement!AC193</f>
-        <v>-2.1887353931368002E-2</v>
+        <v>-2.1610630665001226E-2</v>
       </c>
     </row>
     <row r="70" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -34256,14 +34227,14 @@
     <row r="1" spans="2:7" ht="12" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="3" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B3" s="8"/>
-      <c r="C3" s="232" t="s">
+      <c r="C3" s="234" t="s">
         <v>317</v>
       </c>
-      <c r="D3" s="233"/>
-      <c r="F3" s="234" t="s">
+      <c r="D3" s="235"/>
+      <c r="F3" s="236" t="s">
         <v>318</v>
       </c>
-      <c r="G3" s="233"/>
+      <c r="G3" s="235"/>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B4" s="8"/>
@@ -34330,19 +34301,19 @@
       <c r="B7" s="208" t="s">
         <v>319</v>
       </c>
-      <c r="C7" s="235">
+      <c r="C7" s="232">
         <f>Statement!AA88</f>
         <v>-7.0937545707181514E-3</v>
       </c>
-      <c r="D7" s="236"/>
-      <c r="F7" s="235">
+      <c r="D7" s="233"/>
+      <c r="F7" s="232">
         <f>IF(F6=0,
 IF(G6=0,0,IF(G6&gt;0,1,-1)),
 (G6-F6)/ABS(F6)
 )</f>
         <v>7.1840214731191288E-2</v>
       </c>
-      <c r="G7" s="236"/>
+      <c r="G7" s="233"/>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B8" s="209" t="s">
@@ -34369,19 +34340,19 @@
       <c r="B9" s="208" t="s">
         <v>319</v>
       </c>
-      <c r="C9" s="235">
+      <c r="C9" s="232">
         <f>Statement!AA89</f>
         <v>-5.7381743213835761E-2</v>
       </c>
-      <c r="D9" s="236"/>
-      <c r="F9" s="235">
+      <c r="D9" s="233"/>
+      <c r="F9" s="232">
         <f>IF(F8=0,
 IF(G8=0,0,IF(G8&gt;0,1,-1)),
 (G8-F8)/ABS(F8)
 )</f>
         <v>2.9393370856785492E-2</v>
       </c>
-      <c r="G9" s="236"/>
+      <c r="G9" s="233"/>
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B10" s="209" t="s">
@@ -34408,19 +34379,19 @@
       <c r="B11" s="208" t="s">
         <v>319</v>
       </c>
-      <c r="C11" s="235">
+      <c r="C11" s="232">
         <f>Statement!AA90</f>
         <v>8.1731741857171761E-2</v>
       </c>
-      <c r="D11" s="236"/>
-      <c r="F11" s="235">
+      <c r="D11" s="233"/>
+      <c r="F11" s="232">
         <f>IF(F10=0,
 IF(G10=0,0,IF(G10&gt;0,1,-1)),
 (G10-F10)/ABS(F10)
 )</f>
         <v>0.1444777397260274</v>
       </c>
-      <c r="G11" s="236"/>
+      <c r="G11" s="233"/>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B12" s="209" t="s">
@@ -34447,19 +34418,19 @@
       <c r="B13" s="208" t="s">
         <v>319</v>
       </c>
-      <c r="C13" s="235">
+      <c r="C13" s="232">
         <f>Statement!AA94</f>
         <v>0.94430437772175113</v>
       </c>
-      <c r="D13" s="236"/>
-      <c r="F13" s="235">
+      <c r="D13" s="233"/>
+      <c r="F13" s="232">
         <f>IF(F12=0,
 IF(G12=0,0,IF(G12&gt;0,1,-1)),
 (G12-F12)/ABS(F12)
 )</f>
         <v>0.70581138145988342</v>
       </c>
-      <c r="G13" s="236"/>
+      <c r="G13" s="233"/>
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B14" s="209" t="s">
@@ -34486,19 +34457,19 @@
       <c r="B15" s="208" t="s">
         <v>319</v>
       </c>
-      <c r="C15" s="235">
+      <c r="C15" s="232">
         <f>Statement!AA95</f>
         <v>-6.4068965517241381</v>
       </c>
-      <c r="D15" s="236"/>
-      <c r="F15" s="235">
+      <c r="D15" s="233"/>
+      <c r="F15" s="232">
         <f>IF(F14=0,
 IF(G14=0,0,IF(G14&gt;0,1,-1)),
 (G14-F14)/ABS(F14)
 )</f>
         <v>-9.4186046511627914</v>
       </c>
-      <c r="G15" s="236"/>
+      <c r="G15" s="233"/>
     </row>
     <row r="16" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B16" s="209" t="s">
@@ -34525,19 +34496,19 @@
       <c r="B17" s="208" t="s">
         <v>319</v>
       </c>
-      <c r="C17" s="235">
+      <c r="C17" s="232">
         <f>Statement!AA97</f>
         <v>-5.3079526226734348</v>
       </c>
-      <c r="D17" s="236"/>
-      <c r="F17" s="235">
+      <c r="D17" s="233"/>
+      <c r="F17" s="232">
         <f>IF(F16=0,
 IF(G16=0,0,IF(G16&gt;0,1,-1)),
 (G16-F16)/ABS(F16)
 )</f>
         <v>-3.5408038976857492</v>
       </c>
-      <c r="G17" s="236"/>
+      <c r="G17" s="233"/>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B18" s="209" t="s">
@@ -34564,22 +34535,22 @@
       <c r="B19" s="208" t="s">
         <v>319</v>
       </c>
-      <c r="C19" s="235">
+      <c r="C19" s="232">
         <f>IF(C18=0,
 IF(D18=0,0,IF(D18&gt;0,1,-1)),
 (D18-C18)/ABS(C18)
 )</f>
         <v>4.6746293245469521E-2</v>
       </c>
-      <c r="D19" s="236"/>
-      <c r="F19" s="235">
+      <c r="D19" s="233"/>
+      <c r="F19" s="232">
         <f>IF(F18=0,
 IF(G18=0,0,IF(G18&gt;0,1,-1)),
 (G18-F18)/ABS(F18)
 )</f>
         <v>0.17038913193644947</v>
       </c>
-      <c r="G19" s="236"/>
+      <c r="G19" s="233"/>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B20" s="209" t="s">
@@ -34606,22 +34577,22 @@
       <c r="B21" s="208" t="s">
         <v>319</v>
       </c>
-      <c r="C21" s="235">
+      <c r="C21" s="232">
         <f>IF(C20=0,
 IF(D20=0,0,IF(D20&gt;0,1,-1)),
 (D20-C20)/ABS(C20)
 )</f>
         <v>-5.083333333333333</v>
       </c>
-      <c r="D21" s="236"/>
-      <c r="F21" s="235">
+      <c r="D21" s="233"/>
+      <c r="F21" s="232">
         <f>IF(F20=0,
 IF(G20=0,0,IF(G20&gt;0,1,-1)),
 (G20-F20)/ABS(F20)
 )</f>
         <v>-2.8421052631578947</v>
       </c>
-      <c r="G21" s="236"/>
+      <c r="G21" s="233"/>
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B23" s="8" t="s">
@@ -34669,22 +34640,22 @@
       <c r="B25" s="208" t="s">
         <v>319</v>
       </c>
-      <c r="C25" s="235">
+      <c r="C25" s="232">
         <f>IF(C24=0,
 IF(D24=0,0,IF(D24&gt;0,1,-1)),
 (D24-C24)/ABS(C24)
 )</f>
         <v>-5.687782253142927E-2</v>
       </c>
-      <c r="D25" s="236"/>
-      <c r="F25" s="235">
+      <c r="D25" s="233"/>
+      <c r="F25" s="232">
         <f>IF(F24=0,
 IF(G24=0,0,IF(G24&gt;0,1,-1)),
 (G24-F24)/ABS(F24)
 )</f>
         <v>1.284572027788701E-2</v>
       </c>
-      <c r="G25" s="236"/>
+      <c r="G25" s="233"/>
     </row>
     <row r="26" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B26" s="20" t="s">
@@ -34711,22 +34682,22 @@
       <c r="B27" s="208" t="s">
         <v>319</v>
       </c>
-      <c r="C27" s="235">
+      <c r="C27" s="232">
         <f>IF(C26=0,
 IF(D26=0,0,IF(D26&gt;0,1,-1)),
 (D26-C26)/ABS(C26)
 )</f>
         <v>6.6497783407219763E-2</v>
       </c>
-      <c r="D27" s="236"/>
-      <c r="F27" s="235">
+      <c r="D27" s="233"/>
+      <c r="F27" s="232">
         <f>IF(F26=0,
 IF(G26=0,0,IF(G26&gt;0,1,-1)),
 (G26-F26)/ABS(F26)
 )</f>
         <v>0.22443044110518662</v>
       </c>
-      <c r="G27" s="236"/>
+      <c r="G27" s="233"/>
     </row>
     <row r="28" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B28" s="20" t="s">
@@ -34753,22 +34724,22 @@
       <c r="B29" s="208" t="s">
         <v>319</v>
       </c>
-      <c r="C29" s="235">
+      <c r="C29" s="232">
         <f>IF(C28=0,
 IF(D28=0,0,IF(D28&gt;0,1,-1)),
 (D28-C28)/ABS(C28)
 )</f>
         <v>-1.1678267594740912E-2</v>
       </c>
-      <c r="D29" s="236"/>
-      <c r="F29" s="235">
+      <c r="D29" s="233"/>
+      <c r="F29" s="232">
         <f>IF(F28=0,
 IF(G28=0,0,IF(G28&gt;0,1,-1)),
 (G28-F28)/ABS(F28)
 )</f>
         <v>8.7111867290514677E-2</v>
       </c>
-      <c r="G29" s="236"/>
+      <c r="G29" s="233"/>
     </row>
     <row r="30" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B30" s="20" t="s">
@@ -34795,22 +34766,22 @@
       <c r="B31" s="208" t="s">
         <v>319</v>
       </c>
-      <c r="C31" s="235">
+      <c r="C31" s="232">
         <f>IF(C30=0,
 IF(D30=0,0,IF(D30&gt;0,1,-1)),
 (D30-C30)/ABS(C30)
 )</f>
         <v>0.2027956512092301</v>
       </c>
-      <c r="D31" s="236"/>
-      <c r="F31" s="235">
+      <c r="D31" s="233"/>
+      <c r="F31" s="232">
         <f>IF(F30=0,
 IF(G30=0,0,IF(G30&gt;0,1,-1)),
 (G30-F30)/ABS(F30)
 )</f>
         <v>0.16155988857938719</v>
       </c>
-      <c r="G31" s="236"/>
+      <c r="G31" s="233"/>
     </row>
     <row r="32" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B32" s="20" t="s">
@@ -34837,25 +34808,37 @@
       <c r="B33" s="208" t="s">
         <v>319</v>
       </c>
-      <c r="C33" s="235">
+      <c r="C33" s="232">
         <f>IF(C32=0,
 IF(D32=0,0,IF(D32&gt;0,1,-1)),
 (D32-C32)/ABS(C32)
 )</f>
         <v>9.4076655052264813E-2</v>
       </c>
-      <c r="D33" s="236"/>
-      <c r="F33" s="235">
+      <c r="D33" s="233"/>
+      <c r="F33" s="232">
         <f>IF(F32=0,
 IF(G32=0,0,IF(G32&gt;0,1,-1)),
 (G32-F32)/ABS(F32)
 )</f>
         <v>-0.33404029692470838</v>
       </c>
-      <c r="G33" s="236"/>
+      <c r="G33" s="233"/>
     </row>
   </sheetData>
   <mergeCells count="28">
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="F15:G15"/>
     <mergeCell ref="C31:D31"/>
     <mergeCell ref="F31:G31"/>
     <mergeCell ref="C33:D33"/>
@@ -34872,18 +34855,6 @@
     <mergeCell ref="F27:G27"/>
     <mergeCell ref="C29:D29"/>
     <mergeCell ref="F29:G29"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="F15:G15"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="F9:G9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>

</xml_diff>

<commit_message>
Finished the NVDA model
</commit_message>
<xml_diff>
--- a/INTC.xlsx
+++ b/INTC.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/KINGSTON/MyStockData/Finance-StockLists/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{827F1DB6-3DE9-3540-B461-125F6B35ED3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD78E10F-6111-134C-8080-3241887127FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="14400" xr2:uid="{AEC0C047-6E16-294C-82BD-58123BA913A1}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="14400" activeTab="4" xr2:uid="{AEC0C047-6E16-294C-82BD-58123BA913A1}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -2248,12 +2248,6 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="168" fontId="18" fillId="17" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="18" fillId="17" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2261,6 +2255,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="18" fillId="17" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="18" fillId="17" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -11693,11 +11693,11 @@
     <v>Powered by Refinitiv</v>
     <v>132.75</v>
     <v>18.965</v>
-    <v>2.2317999999999998</v>
-    <v>4.78</v>
-    <v>4.4288000000000001E-2</v>
-    <v>-1.89</v>
-    <v>-1.6768999999999999E-2</v>
+    <v>2.2513000000000001</v>
+    <v>-12.61</v>
+    <v>-0.11281100000000001</v>
+    <v>-2.2450999999999999</v>
+    <v>-2.2638999999999999E-2</v>
     <v>USD</v>
     <v>Intel Corporation is a global designer and manufacturer of semiconductor products. The Company's segments include Intel Products, Intel Foundry, and All Other. Its Intel Products comprise Client Computing Group (CCG) and Data Center and AI (DCAI). CCG delivers platforms and processors that power PCs and edge devices, enabling enhanced performance, connectivity and user experience for consumer and commercial markets with capabilities that also support retail, industrial robotics and AI ecosystems at the edge. DCAI delivers workload-optimized solutions based upon its x86 architecture for data centers, including CPUs, AI accelerators, NICs, IPUs and custom ASICs, enabling performance and scalability for cloud, enterprise, telecommunication and HPC environments. The Intel Foundry segment comprises technology development, manufacturing and foundry services, developing new semiconductor process technologies and advanced packaging technologies. All Other segments include Mobileye and Other.</v>
     <v>83200</v>
@@ -11705,25 +11705,25 @@
     <v>XNAS</v>
     <v>XNAS</v>
     <v>2200 Mission College Blvd, Rnb-4-151, SANTA CLARA, CA, 95054 US</v>
-    <v>118.29</v>
+    <v>106.48</v>
     <v>Semiconductors &amp; Semiconductor Equipment</v>
     <v>Stock</v>
-    <v>46176.925423043751</v>
+    <v>46178.999997430466</v>
     <v>0</v>
-    <v>110.86</v>
-    <v>566480460000</v>
+    <v>98.33</v>
+    <v>498428420000</v>
     <v>INTEL CORPORATION</v>
     <v>INTEL CORPORATION</v>
-    <v>116.42</v>
+    <v>106.48</v>
     <v>0</v>
-    <v>107.93</v>
-    <v>112.71</v>
-    <v>110.82</v>
+    <v>111.78</v>
+    <v>99.17</v>
+    <v>96.924899999999994</v>
     <v>5026000000</v>
     <v>INTC</v>
     <v>INTEL CORPORATION (XNAS:INTC)</v>
-    <v>118418472</v>
-    <v>145048030</v>
+    <v>145209405</v>
+    <v>137584440</v>
     <v>1989</v>
   </rv>
   <rv s="2">
@@ -11747,17 +11747,17 @@
     <v>Powered by Refinitiv</v>
     <v>46.87</v>
     <v>39.47</v>
-    <v>-0.2</v>
-    <v>-4.4689999999999999E-3</v>
+    <v>0.59</v>
+    <v>1.3178E-2</v>
     <v>US</v>
-    <v>44.63</v>
+    <v>45.54</v>
     <v>Index</v>
     <v>3</v>
-    <v>44.28</v>
+    <v>44.65</v>
     <v>10 Y TSY YLD NDX</v>
-    <v>44.3</v>
-    <v>44.75</v>
-    <v>44.55</v>
+    <v>44.67</v>
+    <v>44.77</v>
+    <v>45.36</v>
     <v>TNX</v>
     <v>10 Y TSY YLD NDX</v>
   </rv>
@@ -11979,9 +11979,9 @@
       <v>at close</v>
       <v>from previous close</v>
       <v>from previous close</v>
-      <v>Source: Nasdaq Last Sale</v>
+      <v>Source: Nasdaq</v>
       <v>GMT</v>
-      <v>Real-Time Nasdaq Last Sale</v>
+      <v>Delayed 15 minutes</v>
       <v>from close</v>
       <v>from close</v>
     </spb>
@@ -12581,7 +12581,7 @@
       </c>
       <c r="F3" s="189">
         <f ca="1">Statement!AC171</f>
-        <v>566480.46</v>
+        <v>498428.42</v>
       </c>
       <c r="H3" s="187" t="str">
         <f>'AVG target price'!B5</f>
@@ -12589,7 +12589,7 @@
       </c>
       <c r="I3" s="213">
         <f ca="1">'AVG target price'!C5</f>
-        <v>-8.8046952175618021</v>
+        <v>-8.7808283251417247</v>
       </c>
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.2">
@@ -12605,7 +12605,7 @@
       </c>
       <c r="F4" s="190">
         <f ca="1">Statement!AC172</f>
-        <v>592317.46</v>
+        <v>524265.41999999993</v>
       </c>
       <c r="H4" s="187" t="str">
         <f>'AVG target price'!B6</f>
@@ -12613,7 +12613,7 @@
       </c>
       <c r="I4" s="213">
         <f ca="1">'AVG target price'!C6</f>
-        <v>32.321232777928991</v>
+        <v>32.235530728427833</v>
       </c>
     </row>
     <row r="5" spans="2:9" x14ac:dyDescent="0.2">
@@ -12622,7 +12622,7 @@
       </c>
       <c r="C5" s="210" cm="1">
         <f t="array" aca="1" ref="C5" ca="1">_FV(C3,"Price",TRUE)</f>
-        <v>112.71</v>
+        <v>99.17</v>
       </c>
       <c r="E5" s="187" t="s">
         <v>246</v>
@@ -12637,7 +12637,7 @@
       </c>
       <c r="I5" s="213">
         <f ca="1">'AVG target price'!C7</f>
-        <v>36.468980651241303</v>
+        <v>36.372280552996166</v>
       </c>
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.2">
@@ -12646,14 +12646,14 @@
       </c>
       <c r="C6" s="210" cm="1">
         <f t="array" aca="1" ref="C6" ca="1">_FV(C3,"Price (Extended hours)",TRUE)</f>
-        <v>110.82</v>
+        <v>96.924899999999994</v>
       </c>
       <c r="E6" s="187" t="s">
         <v>240</v>
       </c>
       <c r="F6" s="192">
         <f ca="1">Statement!AC168</f>
-        <v>-181.79032258064515</v>
+        <v>-159.95161290322582</v>
       </c>
       <c r="H6" s="187" t="str">
         <f>'AVG target price'!B8</f>
@@ -12661,7 +12661,7 @@
       </c>
       <c r="I6" s="213">
         <f ca="1">'AVG target price'!C8</f>
-        <v>-10.984571681463171</v>
+        <v>-10.955445307711837</v>
       </c>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.2">
@@ -12670,14 +12670,14 @@
       </c>
       <c r="C7" s="6" cm="1">
         <f t="array" aca="1" ref="C7" ca="1">_FV(C3,"Change")</f>
-        <v>4.78</v>
+        <v>-12.61</v>
       </c>
       <c r="E7" s="188" t="s">
         <v>197</v>
       </c>
       <c r="F7" s="193">
         <f ca="1">Statement!AC169</f>
-        <v>9.8647193236984538</v>
+        <v>8.6796576641928471</v>
       </c>
       <c r="H7" s="186" t="str">
         <f>'AVG target price'!B9</f>
@@ -12685,7 +12685,7 @@
       </c>
       <c r="I7" s="214">
         <f ca="1">'AVG target price'!C9</f>
-        <v>12.25023663253633</v>
+        <v>12.21788441214261</v>
       </c>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.2">
@@ -12694,14 +12694,14 @@
       </c>
       <c r="C8" s="6" cm="1">
         <f t="array" aca="1" ref="C8" ca="1">_FV(C3,"Change (extended hours)",TRUE)</f>
-        <v>-1.89</v>
+        <v>-2.2450999999999999</v>
       </c>
       <c r="E8" s="187" t="s">
         <v>268</v>
       </c>
       <c r="F8" s="194">
         <f ca="1">Statement!AC179</f>
-        <v>-9.6914198946950452E-3</v>
+        <v>-1.1014620715247336E-2</v>
       </c>
       <c r="H8" s="186" t="str">
         <f>'AVG target price'!B11</f>
@@ -12709,7 +12709,7 @@
       </c>
       <c r="I8" s="215">
         <f ca="1">'AVG target price'!C11</f>
-        <v>-0.8913118921787212</v>
+        <v>-0.87679858412682654</v>
       </c>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.2">
@@ -12718,14 +12718,14 @@
       </c>
       <c r="C9" s="72" cm="1">
         <f t="array" aca="1" ref="C9" ca="1">_FV(C3,"Change (%)",TRUE)</f>
-        <v>4.4288000000000001E-2</v>
+        <v>-0.11281100000000001</v>
       </c>
       <c r="E9" s="187" t="s">
         <v>292</v>
       </c>
       <c r="F9" s="194">
         <f ca="1">Statement!AC180</f>
-        <v>-5.5008428710850857E-3</v>
+        <v>-6.2518906927498232E-3</v>
       </c>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.2">
@@ -12734,7 +12734,7 @@
       </c>
       <c r="C10" s="72" cm="1">
         <f t="array" aca="1" ref="C10" ca="1">_FV(C3,"Change % (extended hours)",TRUE)</f>
-        <v>-1.6768999999999999E-2</v>
+        <v>-2.2638999999999999E-2</v>
       </c>
       <c r="E10" s="187" t="s">
         <v>297</v>
@@ -12782,7 +12782,7 @@
       </c>
       <c r="C13" s="211" cm="1">
         <f t="array" aca="1" ref="C13" ca="1">_FV(C3,"Beta")</f>
-        <v>2.2317999999999998</v>
+        <v>2.2513000000000001</v>
       </c>
       <c r="E13" s="187" t="s">
         <v>99</v>
@@ -12798,7 +12798,7 @@
       </c>
       <c r="C14" s="212" cm="1">
         <f t="array" aca="1" ref="C14" ca="1">_FV(C3,"Volume average",TRUE)</f>
-        <v>145048030</v>
+        <v>137584440</v>
       </c>
       <c r="E14" s="188" t="s">
         <v>100</v>
@@ -12814,7 +12814,7 @@
       </c>
       <c r="F15" s="194">
         <f ca="1">Statement!AC193</f>
-        <v>-2.1610630665001226E-2</v>
+        <v>-2.4561199780702713E-2</v>
       </c>
     </row>
     <row r="16" spans="2:9" x14ac:dyDescent="0.2">
@@ -12924,7 +12924,7 @@
       </c>
       <c r="F26" s="226" cm="1">
         <f t="array" aca="1" ref="F26" ca="1">_FV(E26,"Price")</f>
-        <v>44.55</v>
+        <v>45.36</v>
       </c>
     </row>
     <row r="27" spans="2:9" x14ac:dyDescent="0.2">
@@ -12939,7 +12939,7 @@
       </c>
       <c r="F27" s="227">
         <f ca="1">F26/1000</f>
-        <v>4.4549999999999999E-2</v>
+        <v>4.5359999999999998E-2</v>
       </c>
     </row>
     <row r="31" spans="2:9" x14ac:dyDescent="0.2">
@@ -17358,12 +17358,6 @@
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="C3:G3"/>
-    <mergeCell ref="H3:L3"/>
-    <mergeCell ref="P3:W3"/>
-    <mergeCell ref="X3:Z3"/>
-    <mergeCell ref="C5:L5"/>
-    <mergeCell ref="P5:Z5"/>
     <mergeCell ref="C40:L40"/>
     <mergeCell ref="C11:L11"/>
     <mergeCell ref="P11:Z11"/>
@@ -17371,6 +17365,12 @@
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="C26:L26"/>
     <mergeCell ref="C33:L33"/>
+    <mergeCell ref="C3:G3"/>
+    <mergeCell ref="H3:L3"/>
+    <mergeCell ref="P3:W3"/>
+    <mergeCell ref="X3:Z3"/>
+    <mergeCell ref="C5:L5"/>
+    <mergeCell ref="P5:Z5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
@@ -18430,16 +18430,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="C31:L31"/>
+    <mergeCell ref="C25:L25"/>
+    <mergeCell ref="C2:G2"/>
+    <mergeCell ref="H2:L2"/>
+    <mergeCell ref="S2:Z2"/>
     <mergeCell ref="AA2:AC2"/>
     <mergeCell ref="C4:L4"/>
     <mergeCell ref="S4:AC4"/>
     <mergeCell ref="C13:L13"/>
     <mergeCell ref="C18:L18"/>
-    <mergeCell ref="C31:L31"/>
-    <mergeCell ref="C25:L25"/>
-    <mergeCell ref="C2:G2"/>
-    <mergeCell ref="H2:L2"/>
-    <mergeCell ref="S2:Z2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -18522,7 +18522,7 @@
       </c>
       <c r="C6" s="132">
         <f ca="1">Overview!C5</f>
-        <v>112.71</v>
+        <v>99.17</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -18531,7 +18531,7 @@
       </c>
       <c r="C7" s="133">
         <f ca="1">C5*C6</f>
-        <v>566480.46</v>
+        <v>498428.42</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -18549,7 +18549,7 @@
       </c>
       <c r="C9" s="134">
         <f ca="1">Overview!F27</f>
-        <v>4.4549999999999999E-2</v>
+        <v>4.5359999999999998E-2</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -18558,7 +18558,7 @@
       </c>
       <c r="C10" s="132">
         <f ca="1">Overview!C13</f>
-        <v>2.2317999999999998</v>
+        <v>2.2513000000000001</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -18601,7 +18601,7 @@
       </c>
       <c r="C16" s="46">
         <f ca="1">C8/(C8+C7)</f>
-        <v>7.3638848894180986E-2</v>
+        <v>8.285991252115936E-2</v>
       </c>
     </row>
     <row r="17" spans="2:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -18610,7 +18610,7 @@
       </c>
       <c r="C17" s="46">
         <f ca="1">C7/(C8+C7)</f>
-        <v>0.92636115110581896</v>
+        <v>0.91714008747884079</v>
       </c>
     </row>
     <row r="18" spans="2:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -18628,7 +18628,7 @@
       </c>
       <c r="C19" s="46">
         <f ca="1">C9+C10*C11</f>
-        <v>0.144981</v>
+        <v>0.14666849999999998</v>
       </c>
     </row>
     <row r="20" spans="2:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -18637,7 +18637,7 @@
       </c>
       <c r="C20" s="46">
         <f ca="1">(C17*C19)+(C16*C18)</f>
-        <v>0.13744619934229851</v>
+        <v>0.13805036478854302</v>
       </c>
     </row>
     <row r="21" spans="2:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -18896,7 +18896,7 @@
       </c>
       <c r="L8" s="125">
         <f ca="1">L7*(1+C14)/(C15-C14)</f>
-        <v>-23274.223920113993</v>
+        <v>-23155.109659807575</v>
       </c>
       <c r="N8" s="90"/>
       <c r="O8" s="16"/>
@@ -18950,23 +18950,23 @@
       <c r="G10" s="138"/>
       <c r="H10" s="125">
         <f ca="1">H7/(1+$C$15)^H9</f>
-        <v>-6493.7941565070196</v>
+        <v>-6490.3467466508528</v>
       </c>
       <c r="I10" s="125">
         <f t="shared" ref="I10:L10" ca="1" si="0">I7/(1+$C$15)^I9</f>
-        <v>-5057.0750662070459</v>
+        <v>-5051.7071157001965</v>
       </c>
       <c r="J10" s="125">
         <f t="shared" ca="1" si="0"/>
-        <v>-3564.2605764441973</v>
+        <v>-3558.5870311676535</v>
       </c>
       <c r="K10" s="125">
         <f t="shared" ca="1" si="0"/>
-        <v>-3263.5193608417944</v>
+        <v>-3256.594760152715</v>
       </c>
       <c r="L10" s="125">
         <f t="shared" ca="1" si="0"/>
-        <v>-1407.5365602091188</v>
+        <v>-1403.8043768240807</v>
       </c>
       <c r="N10" s="90"/>
     </row>
@@ -18985,7 +18985,7 @@
       <c r="K11" s="137"/>
       <c r="L11" s="125">
         <f ca="1">L8/(1+C15)^L9</f>
-        <v>-12224.212443256436</v>
+        <v>-12129.403131666804</v>
       </c>
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.2">
@@ -19008,7 +19008,7 @@
       </c>
       <c r="C15" s="134">
         <f ca="1">IF(WACC!C21&gt;0,WACC!C21,WACC!C20)</f>
-        <v>0.13744619934229851</v>
+        <v>0.13805036478854302</v>
       </c>
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.2">
@@ -19023,7 +19023,7 @@
       </c>
       <c r="C19" s="63">
         <f ca="1">SUM(H10:L10)</f>
-        <v>-19786.185720209178</v>
+        <v>-19761.0400304955</v>
       </c>
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.2">
@@ -19032,7 +19032,7 @@
       </c>
       <c r="C20" s="63">
         <f ca="1">L11</f>
-        <v>-12224.212443256436</v>
+        <v>-12129.403131666804</v>
       </c>
     </row>
     <row r="21" spans="2:3" x14ac:dyDescent="0.2">
@@ -19041,7 +19041,7 @@
       </c>
       <c r="C21" s="93">
         <f ca="1">C19+C20</f>
-        <v>-32010.398163465616</v>
+        <v>-31890.443162162304</v>
       </c>
     </row>
     <row r="22" spans="2:3" x14ac:dyDescent="0.2">
@@ -19068,7 +19068,7 @@
       </c>
       <c r="C24" s="93">
         <f ca="1">C21+C22-C23</f>
-        <v>-44252.398163465616</v>
+        <v>-44132.443162162308</v>
       </c>
     </row>
     <row r="25" spans="2:3" x14ac:dyDescent="0.2">
@@ -19086,7 +19086,7 @@
       </c>
       <c r="C26" s="142">
         <f ca="1">C24/C25</f>
-        <v>-8.8046952175618021</v>
+        <v>-8.7808283251417247</v>
       </c>
     </row>
   </sheetData>
@@ -20095,7 +20095,7 @@
       </c>
       <c r="C39" s="134">
         <f ca="1">IF(WACC!C21&gt;0,WACC!C21,WACC!C20)</f>
-        <v>0.13744619934229851</v>
+        <v>0.13805036478854302</v>
       </c>
     </row>
     <row r="40" spans="2:14" x14ac:dyDescent="0.2">
@@ -20139,7 +20139,7 @@
       </c>
       <c r="C44" s="142">
         <f ca="1">C43/(1+C48)^5</f>
-        <v>32.321232777928991</v>
+        <v>32.235530728427833</v>
       </c>
     </row>
     <row r="46" spans="2:14" x14ac:dyDescent="0.2">
@@ -20163,7 +20163,7 @@
       </c>
       <c r="C48" s="134">
         <f ca="1">IF(WACC!C21&gt;0,WACC!C21,WACC!C20)</f>
-        <v>0.13744619934229851</v>
+        <v>0.13805036478854302</v>
       </c>
     </row>
     <row r="49" spans="2:3" x14ac:dyDescent="0.2">
@@ -20198,7 +20198,7 @@
       </c>
       <c r="C52" s="142">
         <f ca="1">C51/(1+C48)^5</f>
-        <v>36.468980651241303</v>
+        <v>36.372280552996166</v>
       </c>
     </row>
     <row r="54" spans="2:3" x14ac:dyDescent="0.2">
@@ -20222,7 +20222,7 @@
       </c>
       <c r="C56" s="134">
         <f ca="1">IF(WACC!C21&gt;0,WACC!C21,WACC!C20)</f>
-        <v>0.13744619934229851</v>
+        <v>0.13805036478854302</v>
       </c>
     </row>
     <row r="57" spans="2:3" x14ac:dyDescent="0.2">
@@ -20266,7 +20266,7 @@
       </c>
       <c r="C61" s="142">
         <f ca="1">C60/(1+C56)^5</f>
-        <v>-10.984571681463171</v>
+        <v>-10.955445307711837</v>
       </c>
     </row>
   </sheetData>
@@ -20330,7 +20330,7 @@
       </c>
       <c r="C5" s="132">
         <f ca="1">DCF!C26</f>
-        <v>-8.8046952175618021</v>
+        <v>-8.7808283251417247</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
@@ -20339,7 +20339,7 @@
       </c>
       <c r="C6" s="132">
         <f ca="1">Multiples!C44</f>
-        <v>32.321232777928991</v>
+        <v>32.235530728427833</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.2">
@@ -20348,7 +20348,7 @@
       </c>
       <c r="C7" s="132">
         <f ca="1">Multiples!C52</f>
-        <v>36.468980651241303</v>
+        <v>36.372280552996166</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.2">
@@ -20357,7 +20357,7 @@
       </c>
       <c r="C8" s="132">
         <f ca="1">Multiples!C61</f>
-        <v>-10.984571681463171</v>
+        <v>-10.955445307711837</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.2">
@@ -20366,7 +20366,7 @@
       </c>
       <c r="C9" s="142">
         <f ca="1">AVERAGE(C5:C8)</f>
-        <v>12.25023663253633</v>
+        <v>12.21788441214261</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.2">
@@ -20375,7 +20375,7 @@
       </c>
       <c r="C10" s="132">
         <f ca="1">Overview!C5</f>
-        <v>112.71</v>
+        <v>99.17</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.2">
@@ -20384,7 +20384,7 @@
       </c>
       <c r="C11" s="154">
         <f ca="1">(C9-C10)/C10</f>
-        <v>-0.8913118921787212</v>
+        <v>-0.87679858412682654</v>
       </c>
     </row>
   </sheetData>
@@ -20637,7 +20637,7 @@
       <c r="K8" s="137"/>
       <c r="L8" s="125">
         <f ca="1">L7*(1+C20)/(C21-C20)</f>
-        <v>-964211.89909385249</v>
+        <v>-959277.1958988749</v>
       </c>
       <c r="N8" s="90"/>
       <c r="O8" s="16"/>
@@ -20691,23 +20691,23 @@
       <c r="G10" s="138"/>
       <c r="H10" s="125">
         <f ca="1">H7/(1+$C$21)^H9</f>
-        <v>-13168.752681684975</v>
+        <v>-13161.76168586741</v>
       </c>
       <c r="I10" s="125">
         <f t="shared" ref="I10:L10" ca="1" si="1">I7/(1+$C$21)^I9</f>
-        <v>-19102.830478790267</v>
+        <v>-19082.553332968146</v>
       </c>
       <c r="J10" s="125">
         <f t="shared" ca="1" si="1"/>
-        <v>-27710.910905702134</v>
+        <v>-27666.801025319983</v>
       </c>
       <c r="K10" s="125">
         <f t="shared" ca="1" si="1"/>
-        <v>-40197.947842145659</v>
+        <v>-40112.65503197661</v>
       </c>
       <c r="L10" s="125">
         <f t="shared" ca="1" si="1"/>
-        <v>-58311.869148529528</v>
+        <v>-58157.251076545435</v>
       </c>
       <c r="N10" s="90"/>
     </row>
@@ -20726,7 +20726,7 @@
       <c r="K11" s="137"/>
       <c r="L11" s="125">
         <f ca="1">L8/(1+C21)^L9</f>
-        <v>-506428.53378465137</v>
+        <v>-502500.74368117063</v>
       </c>
     </row>
     <row r="13" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
@@ -20742,7 +20742,7 @@
       </c>
       <c r="C15" s="156">
         <f ca="1">Overview!C5</f>
-        <v>112.71</v>
+        <v>99.17</v>
       </c>
     </row>
     <row r="16" spans="1:28" x14ac:dyDescent="0.2">
@@ -20751,7 +20751,7 @@
       </c>
       <c r="C16" s="156">
         <f ca="1">C36</f>
-        <v>-134.73196276193872</v>
+        <v>-133.88853279622924</v>
       </c>
     </row>
     <row r="17" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -20790,7 +20790,7 @@
       </c>
       <c r="C21" s="161">
         <f ca="1">IF(WACC!C21&gt;0,WACC!C21,WACC!C20)</f>
-        <v>0.13744619934229851</v>
+        <v>0.13805036478854302</v>
       </c>
     </row>
     <row r="22" spans="2:9" x14ac:dyDescent="0.2">
@@ -20808,7 +20808,7 @@
       </c>
       <c r="C23" s="162">
         <f ca="1">C15*C22</f>
-        <v>566480.46</v>
+        <v>498428.42</v>
       </c>
     </row>
     <row r="24" spans="2:9" x14ac:dyDescent="0.2">
@@ -20835,7 +20835,7 @@
       </c>
       <c r="C26" s="163">
         <f ca="1">C23+C25-C24</f>
-        <v>578722.46</v>
+        <v>510670.41999999993</v>
       </c>
     </row>
     <row r="27" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
@@ -20851,7 +20851,7 @@
       </c>
       <c r="C29" s="162">
         <f ca="1">SUM(H10:L10)</f>
-        <v>-158492.31105685257</v>
+        <v>-158181.02215267759</v>
       </c>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.2">
@@ -20860,7 +20860,7 @@
       </c>
       <c r="C30" s="162">
         <f ca="1">L11</f>
-        <v>-506428.53378465137</v>
+        <v>-502500.74368117063</v>
       </c>
     </row>
     <row r="31" spans="2:9" x14ac:dyDescent="0.2">
@@ -20869,7 +20869,7 @@
       </c>
       <c r="C31" s="165">
         <f ca="1">C29+C30</f>
-        <v>-664920.844841504</v>
+        <v>-660681.76583384816</v>
       </c>
     </row>
     <row r="32" spans="2:9" x14ac:dyDescent="0.2">
@@ -20896,7 +20896,7 @@
       </c>
       <c r="C34" s="165">
         <f ca="1">C31+C32-C33</f>
-        <v>-677162.844841504</v>
+        <v>-672923.76583384816</v>
       </c>
     </row>
     <row r="35" spans="2:12" x14ac:dyDescent="0.2">
@@ -20914,7 +20914,7 @@
       </c>
       <c r="C36" s="168">
         <f ca="1">C34/C35</f>
-        <v>-134.73196276193872</v>
+        <v>-133.88853279622924</v>
       </c>
     </row>
     <row r="39" spans="2:12" x14ac:dyDescent="0.2">
@@ -21361,17 +21361,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="E17:I17"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="C39:L39"/>
     <mergeCell ref="C3:G3"/>
     <mergeCell ref="H3:L3"/>
     <mergeCell ref="P3:W3"/>
     <mergeCell ref="X3:Z3"/>
     <mergeCell ref="C5:L5"/>
     <mergeCell ref="P5:Z5"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="E17:I17"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="C39:L39"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -28520,7 +28520,7 @@
       <c r="AA129" s="67"/>
       <c r="AC129" s="62">
         <f ca="1">Overview!C5</f>
-        <v>112.71</v>
+        <v>99.17</v>
       </c>
     </row>
     <row r="130" spans="1:31" x14ac:dyDescent="0.2">
@@ -28567,7 +28567,7 @@
       <c r="AA130" s="67"/>
       <c r="AC130" s="64">
         <f t="shared" ref="AC130" ca="1" si="76">AC129/AC84</f>
-        <v>112.71</v>
+        <v>99.17</v>
       </c>
     </row>
     <row r="132" spans="1:31" x14ac:dyDescent="0.2">
@@ -29993,7 +29993,7 @@
       <c r="AA168" s="49"/>
       <c r="AC168" s="71">
         <f ca="1">AC130/Statement!AC26</f>
-        <v>-181.79032258064515</v>
+        <v>-159.95161290322582</v>
       </c>
     </row>
     <row r="169" spans="2:29" x14ac:dyDescent="0.2">
@@ -30030,7 +30030,7 @@
       <c r="AA169" s="49"/>
       <c r="AC169" s="71">
         <f ca="1">AC130/(Statement!AC5/Statement!AC22)</f>
-        <v>9.8647193236984538</v>
+        <v>8.6796576641928471</v>
       </c>
     </row>
     <row r="170" spans="2:29" x14ac:dyDescent="0.2">
@@ -30067,7 +30067,7 @@
       <c r="AA170" s="49"/>
       <c r="AC170" s="71">
         <f ca="1">AC130/(Statement!AC48/Statement!AC74)</f>
-        <v>5.085376770741691</v>
+        <v>4.4744637951774777</v>
       </c>
     </row>
     <row r="171" spans="2:29" x14ac:dyDescent="0.2">
@@ -30104,7 +30104,7 @@
       <c r="AA171" s="49"/>
       <c r="AC171" s="143">
         <f ca="1">Statement!AC130*Statement!AC77</f>
-        <v>566480.46</v>
+        <v>498428.42</v>
       </c>
     </row>
     <row r="172" spans="2:29" x14ac:dyDescent="0.2">
@@ -30141,7 +30141,7 @@
       <c r="AA172" s="49"/>
       <c r="AC172" s="143">
         <f ca="1">AC171+AC121-AC120+AC47+AC44</f>
-        <v>592317.46</v>
+        <v>524265.41999999993</v>
       </c>
     </row>
     <row r="173" spans="2:29" x14ac:dyDescent="0.2">
@@ -30178,7 +30178,7 @@
       <c r="AA173" s="49"/>
       <c r="AC173" s="185">
         <f ca="1">AC172/AC5</f>
-        <v>11.017195096999794</v>
+        <v>9.7514167736175423</v>
       </c>
     </row>
     <row r="174" spans="2:29" x14ac:dyDescent="0.2">
@@ -30215,7 +30215,7 @@
       <c r="AA174" s="49"/>
       <c r="AC174" s="185">
         <f ca="1">AC172/AC12</f>
-        <v>-117.313816597346</v>
+        <v>-103.83549613784906</v>
       </c>
     </row>
     <row r="175" spans="2:29" x14ac:dyDescent="0.2">
@@ -30350,7 +30350,7 @@
       <c r="AA177" s="49"/>
       <c r="AC177" s="71">
         <f t="shared" ref="AC177:AC178" ca="1" si="105">AC171/AC175</f>
-        <v>-103.18405464480874</v>
+        <v>-90.788418943533699</v>
       </c>
     </row>
     <row r="178" spans="2:29" x14ac:dyDescent="0.2">
@@ -30387,7 +30387,7 @@
       <c r="AA178" s="49"/>
       <c r="AC178" s="71">
         <f t="shared" ca="1" si="105"/>
-        <v>-69.091036976554292</v>
+        <v>-61.153087600606547</v>
       </c>
     </row>
     <row r="179" spans="2:29" x14ac:dyDescent="0.2">
@@ -30424,7 +30424,7 @@
       <c r="AA179" s="49"/>
       <c r="AC179" s="73">
         <f t="shared" ref="AC179" ca="1" si="108">AC175/AC171</f>
-        <v>-9.6914198946950452E-3</v>
+        <v>-1.1014620715247336E-2</v>
       </c>
     </row>
     <row r="180" spans="2:29" x14ac:dyDescent="0.2">
@@ -30461,7 +30461,7 @@
       <c r="AA180" s="49"/>
       <c r="AC180" s="73">
         <f t="shared" ref="AC180" ca="1" si="110">AC26/AC130</f>
-        <v>-5.5008428710850857E-3</v>
+        <v>-6.2518906927498232E-3</v>
       </c>
     </row>
     <row r="181" spans="2:29" x14ac:dyDescent="0.2">
@@ -31038,7 +31038,7 @@
       <c r="AA193" s="49"/>
       <c r="AC193" s="154">
         <f ca="1">(AC120-AC121)/AC171</f>
-        <v>-2.1610630665001226E-2</v>
+        <v>-2.4561199780702713E-2</v>
       </c>
     </row>
     <row r="194" spans="2:29" x14ac:dyDescent="0.2">
@@ -31720,7 +31720,7 @@
       </c>
       <c r="C5" s="174">
         <f ca="1">Overview!C5</f>
-        <v>112.71</v>
+        <v>99.17</v>
       </c>
       <c r="E5" s="12"/>
       <c r="F5" s="131" t="s">
@@ -31736,7 +31736,7 @@
       </c>
       <c r="C6" s="175">
         <f ca="1">Statement!AC171</f>
-        <v>566480.46</v>
+        <v>498428.42</v>
       </c>
       <c r="E6" s="20" t="s">
         <v>19</v>
@@ -31756,7 +31756,7 @@
       </c>
       <c r="C7" s="175">
         <f ca="1">Statement!AC172</f>
-        <v>592317.46</v>
+        <v>524265.41999999993</v>
       </c>
       <c r="E7" s="20" t="s">
         <v>29</v>
@@ -31776,7 +31776,7 @@
       </c>
       <c r="C8" s="176">
         <f ca="1">Statement!AC168</f>
-        <v>-181.79032258064515</v>
+        <v>-159.95161290322582</v>
       </c>
       <c r="E8" s="20" t="s">
         <v>246</v>
@@ -31796,7 +31796,7 @@
       </c>
       <c r="C9" s="176">
         <f ca="1">Statement!AC169</f>
-        <v>9.8647193236984538</v>
+        <v>8.6796576641928471</v>
       </c>
       <c r="E9" s="20" t="s">
         <v>247</v>
@@ -31816,17 +31816,17 @@
       </c>
       <c r="C10" s="176">
         <f ca="1">Statement!AC170</f>
-        <v>5.085376770741691</v>
+        <v>4.4744637951774777</v>
       </c>
       <c r="E10" s="20" t="s">
         <v>1</v>
       </c>
       <c r="F10" s="180">
-        <f>IF(Statement!M129&lt;=0,"N/A",_xlfn.RRI(4,Statement!M129,Statement!Q129))</f>
+        <f>IF(Statement!M130&lt;=0,"N/A",_xlfn.RRI(4,Statement!M130,Statement!Q130))</f>
         <v>-8.3512303772420138E-2</v>
       </c>
       <c r="G10" s="180" t="str">
-        <f>IF(Statement!H129&lt;=0,"N/A",_xlfn.RRI(9,Statement!H129,Statement!Q129))</f>
+        <f>IF(Statement!H130&lt;=0,"N/A",_xlfn.RRI(9,Statement!H130,Statement!Q130))</f>
         <v>N/A</v>
       </c>
     </row>
@@ -31836,7 +31836,7 @@
       </c>
       <c r="C11" s="176">
         <f ca="1">Statement!AC173</f>
-        <v>11.017195096999794</v>
+        <v>9.7514167736175423</v>
       </c>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.2">
@@ -31845,7 +31845,7 @@
       </c>
       <c r="C12" s="176">
         <f ca="1">Statement!AC174</f>
-        <v>-117.313816597346</v>
+        <v>-103.83549613784906</v>
       </c>
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.2">
@@ -32081,7 +32081,7 @@
       </c>
       <c r="C38" s="177">
         <f ca="1">Statement!AC180</f>
-        <v>-5.5008428710850857E-3</v>
+        <v>-6.2518906927498232E-3</v>
       </c>
       <c r="E38" s="20" t="s">
         <v>274</v>
@@ -32097,7 +32097,7 @@
       </c>
       <c r="C39" s="217">
         <f ca="1">Statement!AC179</f>
-        <v>-9.6914198946950452E-3</v>
+        <v>-1.1014620715247336E-2</v>
       </c>
       <c r="E39" s="20" t="s">
         <v>276</v>
@@ -32182,7 +32182,7 @@
       </c>
       <c r="F48" s="177">
         <f ca="1">Statement!AC193</f>
-        <v>-2.1610630665001226E-2</v>
+        <v>-2.4561199780702713E-2</v>
       </c>
     </row>
     <row r="51" spans="2:6" x14ac:dyDescent="0.2">
@@ -32361,7 +32361,7 @@
       </c>
       <c r="I6" s="174">
         <f ca="1">Statement!AC129</f>
-        <v>112.71</v>
+        <v>99.17</v>
       </c>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.2">
@@ -32390,7 +32390,7 @@
       </c>
       <c r="I7" s="175">
         <f ca="1">Statement!AC171</f>
-        <v>566480.46</v>
+        <v>498428.42</v>
       </c>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.2">
@@ -32419,7 +32419,7 @@
       </c>
       <c r="I8" s="175">
         <f ca="1">Statement!AC172</f>
-        <v>592317.46</v>
+        <v>524265.41999999993</v>
       </c>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.2">
@@ -32448,7 +32448,7 @@
       </c>
       <c r="I9" s="176">
         <f ca="1">Statement!AC168</f>
-        <v>-181.79032258064515</v>
+        <v>-159.95161290322582</v>
       </c>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.2">
@@ -32477,7 +32477,7 @@
       </c>
       <c r="I10" s="176">
         <f ca="1">Statement!AC169</f>
-        <v>9.8647193236984538</v>
+        <v>8.6796576641928471</v>
       </c>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.2">
@@ -32506,7 +32506,7 @@
       </c>
       <c r="I11" s="176">
         <f ca="1">Statement!AC170</f>
-        <v>5.085376770741691</v>
+        <v>4.4744637951774777</v>
       </c>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.2">
@@ -32535,7 +32535,7 @@
       </c>
       <c r="I12" s="176">
         <f ca="1">Statement!AC173</f>
-        <v>11.017195096999794</v>
+        <v>9.7514167736175423</v>
       </c>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.2">
@@ -32564,7 +32564,7 @@
       </c>
       <c r="I13" s="176">
         <f ca="1">Statement!AC174</f>
-        <v>-117.313816597346</v>
+        <v>-103.83549613784906</v>
       </c>
     </row>
     <row r="15" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -33337,7 +33337,7 @@
       </c>
       <c r="I51" s="177">
         <f ca="1">Statement!AC180</f>
-        <v>-5.5008428710850857E-3</v>
+        <v>-6.2518906927498232E-3</v>
       </c>
     </row>
     <row r="52" spans="2:9" x14ac:dyDescent="0.2">
@@ -33366,7 +33366,7 @@
       </c>
       <c r="I52" s="177">
         <f ca="1">Statement!AC179</f>
-        <v>-9.6914198946950452E-3</v>
+        <v>-1.1014620715247336E-2</v>
       </c>
     </row>
     <row r="53" spans="2:9" x14ac:dyDescent="0.2">
@@ -33689,7 +33689,7 @@
       </c>
       <c r="I68" s="198">
         <f ca="1">Statement!AC193</f>
-        <v>-2.1610630665001226E-2</v>
+        <v>-2.4561199780702713E-2</v>
       </c>
     </row>
     <row r="70" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -34227,14 +34227,14 @@
     <row r="1" spans="2:7" ht="12" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="3" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B3" s="8"/>
-      <c r="C3" s="234" t="s">
+      <c r="C3" s="232" t="s">
         <v>317</v>
       </c>
-      <c r="D3" s="235"/>
-      <c r="F3" s="236" t="s">
+      <c r="D3" s="233"/>
+      <c r="F3" s="234" t="s">
         <v>318</v>
       </c>
-      <c r="G3" s="235"/>
+      <c r="G3" s="233"/>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B4" s="8"/>
@@ -34301,19 +34301,19 @@
       <c r="B7" s="208" t="s">
         <v>319</v>
       </c>
-      <c r="C7" s="232">
+      <c r="C7" s="235">
         <f>Statement!AA88</f>
         <v>-7.0937545707181514E-3</v>
       </c>
-      <c r="D7" s="233"/>
-      <c r="F7" s="232">
+      <c r="D7" s="236"/>
+      <c r="F7" s="235">
         <f>IF(F6=0,
 IF(G6=0,0,IF(G6&gt;0,1,-1)),
 (G6-F6)/ABS(F6)
 )</f>
         <v>7.1840214731191288E-2</v>
       </c>
-      <c r="G7" s="233"/>
+      <c r="G7" s="236"/>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B8" s="209" t="s">
@@ -34340,19 +34340,19 @@
       <c r="B9" s="208" t="s">
         <v>319</v>
       </c>
-      <c r="C9" s="232">
+      <c r="C9" s="235">
         <f>Statement!AA89</f>
         <v>-5.7381743213835761E-2</v>
       </c>
-      <c r="D9" s="233"/>
-      <c r="F9" s="232">
+      <c r="D9" s="236"/>
+      <c r="F9" s="235">
         <f>IF(F8=0,
 IF(G8=0,0,IF(G8&gt;0,1,-1)),
 (G8-F8)/ABS(F8)
 )</f>
         <v>2.9393370856785492E-2</v>
       </c>
-      <c r="G9" s="233"/>
+      <c r="G9" s="236"/>
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B10" s="209" t="s">
@@ -34379,19 +34379,19 @@
       <c r="B11" s="208" t="s">
         <v>319</v>
       </c>
-      <c r="C11" s="232">
+      <c r="C11" s="235">
         <f>Statement!AA90</f>
         <v>8.1731741857171761E-2</v>
       </c>
-      <c r="D11" s="233"/>
-      <c r="F11" s="232">
+      <c r="D11" s="236"/>
+      <c r="F11" s="235">
         <f>IF(F10=0,
 IF(G10=0,0,IF(G10&gt;0,1,-1)),
 (G10-F10)/ABS(F10)
 )</f>
         <v>0.1444777397260274</v>
       </c>
-      <c r="G11" s="233"/>
+      <c r="G11" s="236"/>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B12" s="209" t="s">
@@ -34418,19 +34418,19 @@
       <c r="B13" s="208" t="s">
         <v>319</v>
       </c>
-      <c r="C13" s="232">
+      <c r="C13" s="235">
         <f>Statement!AA94</f>
         <v>0.94430437772175113</v>
       </c>
-      <c r="D13" s="233"/>
-      <c r="F13" s="232">
+      <c r="D13" s="236"/>
+      <c r="F13" s="235">
         <f>IF(F12=0,
 IF(G12=0,0,IF(G12&gt;0,1,-1)),
 (G12-F12)/ABS(F12)
 )</f>
         <v>0.70581138145988342</v>
       </c>
-      <c r="G13" s="233"/>
+      <c r="G13" s="236"/>
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B14" s="209" t="s">
@@ -34457,19 +34457,19 @@
       <c r="B15" s="208" t="s">
         <v>319</v>
       </c>
-      <c r="C15" s="232">
+      <c r="C15" s="235">
         <f>Statement!AA95</f>
         <v>-6.4068965517241381</v>
       </c>
-      <c r="D15" s="233"/>
-      <c r="F15" s="232">
+      <c r="D15" s="236"/>
+      <c r="F15" s="235">
         <f>IF(F14=0,
 IF(G14=0,0,IF(G14&gt;0,1,-1)),
 (G14-F14)/ABS(F14)
 )</f>
         <v>-9.4186046511627914</v>
       </c>
-      <c r="G15" s="233"/>
+      <c r="G15" s="236"/>
     </row>
     <row r="16" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B16" s="209" t="s">
@@ -34496,19 +34496,19 @@
       <c r="B17" s="208" t="s">
         <v>319</v>
       </c>
-      <c r="C17" s="232">
+      <c r="C17" s="235">
         <f>Statement!AA97</f>
         <v>-5.3079526226734348</v>
       </c>
-      <c r="D17" s="233"/>
-      <c r="F17" s="232">
+      <c r="D17" s="236"/>
+      <c r="F17" s="235">
         <f>IF(F16=0,
 IF(G16=0,0,IF(G16&gt;0,1,-1)),
 (G16-F16)/ABS(F16)
 )</f>
         <v>-3.5408038976857492</v>
       </c>
-      <c r="G17" s="233"/>
+      <c r="G17" s="236"/>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B18" s="209" t="s">
@@ -34535,22 +34535,22 @@
       <c r="B19" s="208" t="s">
         <v>319</v>
       </c>
-      <c r="C19" s="232">
+      <c r="C19" s="235">
         <f>IF(C18=0,
 IF(D18=0,0,IF(D18&gt;0,1,-1)),
 (D18-C18)/ABS(C18)
 )</f>
         <v>4.6746293245469521E-2</v>
       </c>
-      <c r="D19" s="233"/>
-      <c r="F19" s="232">
+      <c r="D19" s="236"/>
+      <c r="F19" s="235">
         <f>IF(F18=0,
 IF(G18=0,0,IF(G18&gt;0,1,-1)),
 (G18-F18)/ABS(F18)
 )</f>
         <v>0.17038913193644947</v>
       </c>
-      <c r="G19" s="233"/>
+      <c r="G19" s="236"/>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B20" s="209" t="s">
@@ -34577,22 +34577,22 @@
       <c r="B21" s="208" t="s">
         <v>319</v>
       </c>
-      <c r="C21" s="232">
+      <c r="C21" s="235">
         <f>IF(C20=0,
 IF(D20=0,0,IF(D20&gt;0,1,-1)),
 (D20-C20)/ABS(C20)
 )</f>
         <v>-5.083333333333333</v>
       </c>
-      <c r="D21" s="233"/>
-      <c r="F21" s="232">
+      <c r="D21" s="236"/>
+      <c r="F21" s="235">
         <f>IF(F20=0,
 IF(G20=0,0,IF(G20&gt;0,1,-1)),
 (G20-F20)/ABS(F20)
 )</f>
         <v>-2.8421052631578947</v>
       </c>
-      <c r="G21" s="233"/>
+      <c r="G21" s="236"/>
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B23" s="8" t="s">
@@ -34640,22 +34640,22 @@
       <c r="B25" s="208" t="s">
         <v>319</v>
       </c>
-      <c r="C25" s="232">
+      <c r="C25" s="235">
         <f>IF(C24=0,
 IF(D24=0,0,IF(D24&gt;0,1,-1)),
 (D24-C24)/ABS(C24)
 )</f>
         <v>-5.687782253142927E-2</v>
       </c>
-      <c r="D25" s="233"/>
-      <c r="F25" s="232">
+      <c r="D25" s="236"/>
+      <c r="F25" s="235">
         <f>IF(F24=0,
 IF(G24=0,0,IF(G24&gt;0,1,-1)),
 (G24-F24)/ABS(F24)
 )</f>
         <v>1.284572027788701E-2</v>
       </c>
-      <c r="G25" s="233"/>
+      <c r="G25" s="236"/>
     </row>
     <row r="26" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B26" s="20" t="s">
@@ -34682,22 +34682,22 @@
       <c r="B27" s="208" t="s">
         <v>319</v>
       </c>
-      <c r="C27" s="232">
+      <c r="C27" s="235">
         <f>IF(C26=0,
 IF(D26=0,0,IF(D26&gt;0,1,-1)),
 (D26-C26)/ABS(C26)
 )</f>
         <v>6.6497783407219763E-2</v>
       </c>
-      <c r="D27" s="233"/>
-      <c r="F27" s="232">
+      <c r="D27" s="236"/>
+      <c r="F27" s="235">
         <f>IF(F26=0,
 IF(G26=0,0,IF(G26&gt;0,1,-1)),
 (G26-F26)/ABS(F26)
 )</f>
         <v>0.22443044110518662</v>
       </c>
-      <c r="G27" s="233"/>
+      <c r="G27" s="236"/>
     </row>
     <row r="28" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B28" s="20" t="s">
@@ -34724,22 +34724,22 @@
       <c r="B29" s="208" t="s">
         <v>319</v>
       </c>
-      <c r="C29" s="232">
+      <c r="C29" s="235">
         <f>IF(C28=0,
 IF(D28=0,0,IF(D28&gt;0,1,-1)),
 (D28-C28)/ABS(C28)
 )</f>
         <v>-1.1678267594740912E-2</v>
       </c>
-      <c r="D29" s="233"/>
-      <c r="F29" s="232">
+      <c r="D29" s="236"/>
+      <c r="F29" s="235">
         <f>IF(F28=0,
 IF(G28=0,0,IF(G28&gt;0,1,-1)),
 (G28-F28)/ABS(F28)
 )</f>
         <v>8.7111867290514677E-2</v>
       </c>
-      <c r="G29" s="233"/>
+      <c r="G29" s="236"/>
     </row>
     <row r="30" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B30" s="20" t="s">
@@ -34766,22 +34766,22 @@
       <c r="B31" s="208" t="s">
         <v>319</v>
       </c>
-      <c r="C31" s="232">
+      <c r="C31" s="235">
         <f>IF(C30=0,
 IF(D30=0,0,IF(D30&gt;0,1,-1)),
 (D30-C30)/ABS(C30)
 )</f>
         <v>0.2027956512092301</v>
       </c>
-      <c r="D31" s="233"/>
-      <c r="F31" s="232">
+      <c r="D31" s="236"/>
+      <c r="F31" s="235">
         <f>IF(F30=0,
 IF(G30=0,0,IF(G30&gt;0,1,-1)),
 (G30-F30)/ABS(F30)
 )</f>
         <v>0.16155988857938719</v>
       </c>
-      <c r="G31" s="233"/>
+      <c r="G31" s="236"/>
     </row>
     <row r="32" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B32" s="20" t="s">
@@ -34808,37 +34808,25 @@
       <c r="B33" s="208" t="s">
         <v>319</v>
       </c>
-      <c r="C33" s="232">
+      <c r="C33" s="235">
         <f>IF(C32=0,
 IF(D32=0,0,IF(D32&gt;0,1,-1)),
 (D32-C32)/ABS(C32)
 )</f>
         <v>9.4076655052264813E-2</v>
       </c>
-      <c r="D33" s="233"/>
-      <c r="F33" s="232">
+      <c r="D33" s="236"/>
+      <c r="F33" s="235">
         <f>IF(F32=0,
 IF(G32=0,0,IF(G32&gt;0,1,-1)),
 (G32-F32)/ABS(F32)
 )</f>
         <v>-0.33404029692470838</v>
       </c>
-      <c r="G33" s="233"/>
+      <c r="G33" s="236"/>
     </row>
   </sheetData>
   <mergeCells count="28">
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="F15:G15"/>
     <mergeCell ref="C31:D31"/>
     <mergeCell ref="F31:G31"/>
     <mergeCell ref="C33:D33"/>
@@ -34855,6 +34843,18 @@
     <mergeCell ref="F27:G27"/>
     <mergeCell ref="C29:D29"/>
     <mergeCell ref="F29:G29"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="F9:G9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>

</xml_diff>

<commit_message>
Deleted old NVDA and AMD files
</commit_message>
<xml_diff>
--- a/INTC.xlsx
+++ b/INTC.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/KINGSTON/MyStockData/Finance-StockLists/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD78E10F-6111-134C-8080-3241887127FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A81E3354-E6F3-8E44-8BA9-0AB58DD17B80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="14400" activeTab="4" xr2:uid="{AEC0C047-6E16-294C-82BD-58123BA913A1}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="14400" activeTab="2" xr2:uid="{AEC0C047-6E16-294C-82BD-58123BA913A1}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -152,7 +152,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="729" uniqueCount="392">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="730" uniqueCount="393">
   <si>
     <t>Ticker</t>
   </si>
@@ -967,9 +967,6 @@
     <t>Dividend yield</t>
   </si>
   <si>
-    <t>FCF/Sales</t>
-  </si>
-  <si>
     <t>Earnings yields</t>
   </si>
   <si>
@@ -1328,6 +1325,12 @@
   </si>
   <si>
     <t>Last market price for period adjusted</t>
+  </si>
+  <si>
+    <t>FCFF/Sales (FCFF Margin)</t>
+  </si>
+  <si>
+    <t>FCFE/Sales (FCFE Margin)</t>
   </si>
 </sst>
 </file>
@@ -12560,11 +12563,11 @@
       </c>
       <c r="C2" s="230"/>
       <c r="E2" s="229" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="F2" s="230"/>
       <c r="H2" s="229" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="I2" s="230"/>
     </row>
@@ -12721,7 +12724,7 @@
         <v>-0.11281100000000001</v>
       </c>
       <c r="E9" s="187" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="F9" s="194">
         <f ca="1">Statement!AC180</f>
@@ -12737,7 +12740,7 @@
         <v>-2.2638999999999999E-2</v>
       </c>
       <c r="E10" s="187" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F10" s="194">
         <f ca="1">Statement!AC182</f>
@@ -12753,7 +12756,7 @@
         <v>132.75</v>
       </c>
       <c r="E11" s="188" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="F11" s="195">
         <f ca="1">Statement!AC181</f>
@@ -12810,19 +12813,19 @@
     </row>
     <row r="15" spans="2:9" x14ac:dyDescent="0.2">
       <c r="E15" s="187" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F15" s="194">
-        <f ca="1">Statement!AC193</f>
+        <f ca="1">Statement!AC194</f>
         <v>-2.4561199780702713E-2</v>
       </c>
     </row>
     <row r="16" spans="2:9" x14ac:dyDescent="0.2">
       <c r="E16" s="188" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="F16" s="193">
-        <f>Statement!AC192</f>
+        <f>Statement!AC193</f>
         <v>-2.435734182252288</v>
       </c>
     </row>
@@ -12832,10 +12835,10 @@
       </c>
       <c r="C17" s="231"/>
       <c r="E17" s="186" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="F17" s="196">
-        <f>Statement!AC188</f>
+        <f>Statement!AC189</f>
         <v>5.9689614007162755E-4</v>
       </c>
     </row>
@@ -12844,10 +12847,10 @@
         <v>12</v>
       </c>
       <c r="C18" s="68" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="E18" s="187" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="F18" s="192">
         <f>Statement!AC162</f>
@@ -12875,10 +12878,10 @@
         <v>88</v>
       </c>
       <c r="C20" s="68" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="E20" s="188" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="F20" s="193">
         <f>Statement!AC165</f>
@@ -12890,7 +12893,7 @@
         <v>89</v>
       </c>
       <c r="C21" s="68" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="I21" s="50"/>
     </row>
@@ -12899,7 +12902,7 @@
         <v>90</v>
       </c>
       <c r="C22" s="68" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="25" spans="2:9" x14ac:dyDescent="0.2">
@@ -12908,7 +12911,7 @@
       </c>
       <c r="C25" s="231"/>
       <c r="E25" s="229" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="F25" s="230"/>
     </row>
@@ -12935,7 +12938,7 @@
         <v>5.3999999999999999E-2</v>
       </c>
       <c r="E27" s="188" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="F27" s="227">
         <f ca="1">F26/1000</f>
@@ -12944,7 +12947,7 @@
     </row>
     <row r="31" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B31" s="228" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="C31" s="228"/>
       <c r="D31" s="228"/>
@@ -12955,18 +12958,18 @@
     </row>
     <row r="33" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B33" s="16" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
     </row>
     <row r="34" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B34" s="16" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="37" spans="2:8" ht="8" customHeight="1" x14ac:dyDescent="0.2">
@@ -12980,7 +12983,7 @@
     </row>
     <row r="40" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B40" s="228" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="C40" s="228"/>
       <c r="D40" s="228"/>
@@ -12991,10 +12994,10 @@
     </row>
     <row r="42" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B42" s="41" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="C42" s="41" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="D42" s="41" t="s">
         <v>86</v>
@@ -13003,12 +13006,12 @@
     </row>
     <row r="43" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B43" s="1" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="44" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B44" s="1" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="47" spans="2:8" ht="7" customHeight="1" x14ac:dyDescent="0.2">
@@ -13309,11 +13312,11 @@
         <v>38452.690209023996</v>
       </c>
       <c r="N6" s="89" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="O6" s="5"/>
       <c r="Q6" s="89" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="R6" s="1" t="str">
         <f>B6</f>
@@ -13408,11 +13411,11 @@
         <v>27957.189758960001</v>
       </c>
       <c r="N7" s="89" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="O7" s="5"/>
       <c r="Q7" s="89" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="R7" s="1" t="str">
         <f t="shared" ref="R7:R10" si="3">B7</f>
@@ -13507,11 +13510,11 @@
         <v>66409.879967984001</v>
       </c>
       <c r="N8" s="89" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="O8" s="5"/>
       <c r="Q8" s="89" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="R8" s="1" t="str">
         <f t="shared" si="3"/>
@@ -13606,11 +13609,11 @@
         <v>6177.5999999999995</v>
       </c>
       <c r="N9" s="89" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="O9" s="5"/>
       <c r="Q9" s="89" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="R9" s="1" t="str">
         <f t="shared" si="3"/>
@@ -13702,11 +13705,11 @@
         <v>4678.557983820001</v>
       </c>
       <c r="N10" s="89" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="O10" s="5"/>
       <c r="Q10" s="89" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="R10" s="1" t="str">
         <f t="shared" si="3"/>
@@ -13797,11 +13800,11 @@
         <v>77266.037951804014</v>
       </c>
       <c r="N11" s="1" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="O11" s="5"/>
       <c r="Q11" s="1" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="R11" s="16" t="s">
         <v>116</v>
@@ -18295,7 +18298,7 @@
     </row>
     <row r="32" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B32" s="16" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="C32" s="12">
         <f>C5</f>
@@ -18941,7 +18944,7 @@
     </row>
     <row r="10" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B10" s="1" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C10" s="137"/>
       <c r="D10" s="137"/>
@@ -20038,7 +20041,7 @@
     </row>
     <row r="34" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B34" s="16" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="C34" s="149">
         <f>C32/C8</f>
@@ -20203,7 +20206,7 @@
     </row>
     <row r="54" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B54" s="228" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="C54" s="228"/>
     </row>
@@ -20353,7 +20356,7 @@
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B8" s="1" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="C8" s="132">
         <f ca="1">Multiples!C61</f>
@@ -20682,7 +20685,7 @@
     </row>
     <row r="10" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B10" s="1" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C10" s="137"/>
       <c r="D10" s="137"/>
@@ -20756,7 +20759,7 @@
     </row>
     <row r="17" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B17" s="157" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C17" s="158">
         <v>0.65</v>
@@ -21065,7 +21068,7 @@
     </row>
     <row r="43" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B43" s="121" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="C43" s="94">
         <f>C41/C42</f>
@@ -21150,7 +21153,7 @@
     </row>
     <row r="45" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B45" s="121" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="C45" s="94">
         <f>C41/C44</f>
@@ -21190,7 +21193,7 @@
     </row>
     <row r="46" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B46" s="121" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="C46" s="137"/>
       <c r="D46" s="94">
@@ -21381,7 +21384,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0548B83C-60BF-4548-84AB-1D4A73B251A4}">
-  <dimension ref="A1:AE208"/>
+  <dimension ref="A1:AE209"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="3.6640625" style="1" customWidth="1"/>
@@ -21418,45 +21421,45 @@
       <c r="H2" s="9"/>
       <c r="I2" s="9"/>
       <c r="M2" s="10" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="N2" s="10" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="O2" s="10" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="P2" s="10" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="Q2" s="10" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="R2" s="7"/>
       <c r="S2" s="7"/>
       <c r="T2" s="10" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="U2" s="10" t="s">
+        <v>349</v>
+      </c>
+      <c r="V2" s="10" t="s">
+        <v>338</v>
+      </c>
+      <c r="W2" s="10" t="s">
+        <v>345</v>
+      </c>
+      <c r="X2" s="10" t="s">
         <v>350</v>
       </c>
-      <c r="V2" s="10" t="s">
-        <v>339</v>
-      </c>
-      <c r="W2" s="10" t="s">
-        <v>346</v>
-      </c>
-      <c r="X2" s="10" t="s">
-        <v>351</v>
-      </c>
       <c r="Y2" s="10" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="Z2" s="10" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="AA2" s="10" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="AB2" s="7"/>
       <c r="AD2" s="7"/>
@@ -21485,16 +21488,16 @@
       <c r="R3" s="11"/>
       <c r="S3" s="11"/>
       <c r="T3" s="10" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="U3" s="10" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="V3" s="10" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="W3" s="10" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="X3" s="10" t="s">
         <v>85</v>
@@ -21815,7 +21818,7 @@
     </row>
     <row r="9" spans="1:31" x14ac:dyDescent="0.2">
       <c r="B9" s="20" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="C9" s="21"/>
       <c r="D9" s="21"/>
@@ -22334,7 +22337,7 @@
     </row>
     <row r="17" spans="1:31" x14ac:dyDescent="0.2">
       <c r="B17" s="23" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C17" s="21"/>
       <c r="D17" s="21"/>
@@ -24023,7 +24026,7 @@
     </row>
     <row r="44" spans="1:31" x14ac:dyDescent="0.2">
       <c r="B44" s="20" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="C44" s="21"/>
       <c r="D44" s="21"/>
@@ -24136,7 +24139,7 @@
     </row>
     <row r="46" spans="1:31" x14ac:dyDescent="0.2">
       <c r="B46" s="20" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C46" s="21"/>
       <c r="D46" s="21"/>
@@ -24194,7 +24197,7 @@
     </row>
     <row r="47" spans="1:31" x14ac:dyDescent="0.2">
       <c r="B47" s="20" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C47" s="21"/>
       <c r="D47" s="21"/>
@@ -25003,7 +25006,7 @@
     </row>
     <row r="63" spans="1:31" x14ac:dyDescent="0.2">
       <c r="B63" s="20" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C63" s="61"/>
       <c r="D63" s="61"/>
@@ -25056,7 +25059,7 @@
     </row>
     <row r="64" spans="1:31" x14ac:dyDescent="0.2">
       <c r="B64" s="20" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="C64" s="61"/>
       <c r="D64" s="61"/>
@@ -25847,7 +25850,7 @@
     </row>
     <row r="78" spans="1:31" x14ac:dyDescent="0.2">
       <c r="B78" s="20" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C78" s="25"/>
       <c r="D78" s="25"/>
@@ -25889,7 +25892,7 @@
     </row>
     <row r="79" spans="1:31" x14ac:dyDescent="0.2">
       <c r="B79" s="20" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C79" s="25"/>
       <c r="D79" s="25"/>
@@ -26569,7 +26572,7 @@
     </row>
     <row r="92" spans="1:31" x14ac:dyDescent="0.2">
       <c r="B92" s="20" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="C92" s="49"/>
       <c r="D92" s="50"/>
@@ -27278,7 +27281,7 @@
     </row>
     <row r="105" spans="1:31" x14ac:dyDescent="0.2">
       <c r="B105" s="218" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="C105" s="61"/>
       <c r="D105" s="61"/>
@@ -27336,7 +27339,7 @@
     </row>
     <row r="106" spans="1:31" x14ac:dyDescent="0.2">
       <c r="B106" s="218" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="C106" s="61"/>
       <c r="D106" s="61"/>
@@ -27397,7 +27400,7 @@
     </row>
     <row r="107" spans="1:31" x14ac:dyDescent="0.2">
       <c r="B107" s="20" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="C107" s="61"/>
       <c r="D107" s="61"/>
@@ -27458,7 +27461,7 @@
     </row>
     <row r="108" spans="1:31" x14ac:dyDescent="0.2">
       <c r="B108" s="20" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="C108" s="21"/>
       <c r="D108" s="21"/>
@@ -27516,7 +27519,7 @@
     </row>
     <row r="109" spans="1:31" x14ac:dyDescent="0.2">
       <c r="B109" s="20" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="C109" s="61"/>
       <c r="D109" s="61"/>
@@ -27603,7 +27606,7 @@
     </row>
     <row r="111" spans="1:31" x14ac:dyDescent="0.2">
       <c r="B111" s="218" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="C111" s="61"/>
       <c r="D111" s="61"/>
@@ -27664,7 +27667,7 @@
     </row>
     <row r="112" spans="1:31" x14ac:dyDescent="0.2">
       <c r="B112" s="218" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="C112" s="61"/>
       <c r="D112" s="61"/>
@@ -27725,7 +27728,7 @@
     </row>
     <row r="113" spans="1:31" x14ac:dyDescent="0.2">
       <c r="B113" s="20" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="C113" s="61"/>
       <c r="D113" s="61"/>
@@ -27786,7 +27789,7 @@
     </row>
     <row r="114" spans="1:31" x14ac:dyDescent="0.2">
       <c r="B114" s="20" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C114" s="61"/>
       <c r="D114" s="61"/>
@@ -27847,7 +27850,7 @@
     </row>
     <row r="115" spans="1:31" x14ac:dyDescent="0.2">
       <c r="B115" s="20" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="C115" s="61"/>
       <c r="D115" s="61"/>
@@ -28245,7 +28248,7 @@
     </row>
     <row r="123" spans="1:31" x14ac:dyDescent="0.2">
       <c r="B123" s="20" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C123" s="25"/>
       <c r="D123" s="25"/>
@@ -28316,7 +28319,7 @@
     </row>
     <row r="124" spans="1:31" x14ac:dyDescent="0.2">
       <c r="B124" s="20" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="C124" s="25"/>
       <c r="D124" s="25"/>
@@ -28387,7 +28390,7 @@
     </row>
     <row r="125" spans="1:31" x14ac:dyDescent="0.2">
       <c r="B125" s="20" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="C125" s="25"/>
       <c r="D125" s="25"/>
@@ -28525,7 +28528,7 @@
     </row>
     <row r="130" spans="1:31" x14ac:dyDescent="0.2">
       <c r="B130" s="20" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="C130" s="26"/>
       <c r="D130" s="26"/>
@@ -28803,7 +28806,7 @@
     </row>
     <row r="142" spans="1:31" x14ac:dyDescent="0.2">
       <c r="B142" s="20" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="M142" s="61">
         <v>0</v>
@@ -28851,7 +28854,7 @@
     </row>
     <row r="143" spans="1:31" x14ac:dyDescent="0.2">
       <c r="B143" s="20" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="M143" s="61">
         <v>0</v>
@@ -29102,7 +29105,7 @@
       <c r="P150" s="49"/>
       <c r="Q150" s="49"/>
       <c r="T150" s="173" t="str">
-        <f t="shared" ref="T150:AA150" si="81">IF(U5&gt;T148, "BEAT", IF(U5&lt;T147, "MISSED", "MET"))</f>
+        <f t="shared" ref="T150:Z150" si="81">IF(T149&gt;T148, "BEAT", IF(T149&lt;T147, "MISSED", "MET"))</f>
         <v>MET</v>
       </c>
       <c r="U150" s="173" t="str">
@@ -29130,14 +29133,14 @@
         <v>BEAT</v>
       </c>
       <c r="AA150" s="173" t="str">
-        <f t="shared" si="81"/>
+        <f>IF(AA149&gt;AA148, "BEAT", IF(AA149&lt;AA147, "MISSED", "MET"))</f>
         <v>MISSED</v>
       </c>
       <c r="AC150" s="49"/>
     </row>
     <row r="151" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B151" s="20" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="C151" s="49"/>
       <c r="D151" s="49"/>
@@ -29182,7 +29185,7 @@
     </row>
     <row r="152" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B152" s="20" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="C152" s="49"/>
       <c r="D152" s="49"/>
@@ -29227,7 +29230,7 @@
     </row>
     <row r="153" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B153" s="20" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="C153" s="49"/>
       <c r="D153" s="49"/>
@@ -29298,7 +29301,7 @@
       <c r="P154" s="49"/>
       <c r="Q154" s="49"/>
       <c r="T154" s="173" t="str">
-        <f t="shared" ref="T154:AA154" si="83">IF(U100&gt;T152, "BEAT", IF(U100&lt;T151, "MISSED", "MET"))</f>
+        <f t="shared" ref="T154:Z154" si="83">IF(T153&gt;T152, "BEAT", IF(T153&lt;T151, "MISSED", "MET"))</f>
         <v>MISSED</v>
       </c>
       <c r="U154" s="173" t="str">
@@ -29326,7 +29329,7 @@
         <v>BEAT</v>
       </c>
       <c r="AA154" s="173" t="str">
-        <f t="shared" si="83"/>
+        <f>IF(AA153&gt;AA152, "BEAT", IF(AA153&lt;AA151, "MISSED", "MET"))</f>
         <v>MISSED</v>
       </c>
       <c r="AC154" s="49"/>
@@ -30503,7 +30506,7 @@
     </row>
     <row r="182" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B182" s="20" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="M182" s="154">
         <f>-M62/M171</f>
@@ -30540,7 +30543,7 @@
     </row>
     <row r="183" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B183" s="20" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="M183" s="154">
         <f>-(M62+M63)/M171</f>
@@ -30577,25 +30580,25 @@
     </row>
     <row r="184" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B184" s="20" t="s">
-        <v>271</v>
-      </c>
-      <c r="M184" s="71">
+        <v>391</v>
+      </c>
+      <c r="M184" s="154">
         <f>M176/M5</f>
         <v>6.9118053061243856E-2</v>
       </c>
-      <c r="N184" s="71">
+      <c r="N184" s="154">
         <f>N176/N5</f>
         <v>-0.22176229898182509</v>
       </c>
-      <c r="O184" s="71">
+      <c r="O184" s="154">
         <f>O176/O5</f>
         <v>-0.30655749797152765</v>
       </c>
-      <c r="P184" s="71">
+      <c r="P184" s="154">
         <f>P176/P5</f>
         <v>-0.43577333760192838</v>
       </c>
-      <c r="Q184" s="71">
+      <c r="Q184" s="154">
         <f>Q176/Q5</f>
         <v>-0.1305696933002857</v>
       </c>
@@ -30607,34 +30610,34 @@
       <c r="Y184" s="49"/>
       <c r="Z184" s="49"/>
       <c r="AA184" s="49"/>
-      <c r="AC184" s="71">
+      <c r="AC184" s="154">
         <f>AC176/AC5</f>
         <v>-0.15945910756468204</v>
       </c>
     </row>
     <row r="185" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B185" s="20" t="s">
-        <v>274</v>
+        <v>392</v>
       </c>
       <c r="M185" s="154">
-        <f>-M63/M175</f>
-        <v>0.64970645792563597</v>
+        <f>M175/M5</f>
+        <v>0.10992862927718161</v>
       </c>
       <c r="N185" s="154">
-        <f>-N63/N175</f>
-        <v>-0.47826780445011563</v>
+        <f t="shared" ref="N185:Q185" si="113">N175/N5</f>
+        <v>-0.19886129349446507</v>
       </c>
       <c r="O185" s="154">
-        <f>-O63/O175</f>
-        <v>-0.1763765135937857</v>
+        <f t="shared" si="113"/>
+        <v>-0.3228590396105333</v>
       </c>
       <c r="P185" s="154">
-        <f>-P63/P175</f>
-        <v>-8.3866568761145496E-2</v>
+        <f t="shared" si="113"/>
+        <v>-0.35905161861358542</v>
       </c>
       <c r="Q185" s="154">
-        <f>-Q63/Q175</f>
-        <v>0</v>
+        <f t="shared" si="113"/>
+        <v>-0.13968932700130551</v>
       </c>
       <c r="T185" s="49"/>
       <c r="U185" s="49"/>
@@ -30645,32 +30648,32 @@
       <c r="Z185" s="49"/>
       <c r="AA185" s="49"/>
       <c r="AC185" s="154">
-        <f>-AC63/AC175</f>
-        <v>0</v>
+        <f t="shared" ref="AC184:AC185" si="114">AC175/AC5</f>
+        <v>-0.1021148373416662</v>
       </c>
     </row>
     <row r="186" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B186" s="20" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="M186" s="154">
-        <f>-M62/M175</f>
-        <v>0.27800161160354553</v>
+        <f>-M63/M175</f>
+        <v>0.64970645792563597</v>
       </c>
       <c r="N186" s="154">
-        <f>-N62/N175</f>
-        <v>0</v>
+        <f>-N63/N175</f>
+        <v>-0.47826780445011563</v>
       </c>
       <c r="O186" s="154">
-        <f>-O62/O175</f>
-        <v>0</v>
+        <f>-O63/O175</f>
+        <v>-0.1763765135937857</v>
       </c>
       <c r="P186" s="154">
-        <f>-P62/P175</f>
-        <v>0</v>
+        <f>-P63/P175</f>
+        <v>-8.3866568761145496E-2</v>
       </c>
       <c r="Q186" s="154">
-        <f>-Q62/Q175</f>
+        <f>-Q63/Q175</f>
         <v>0</v>
       </c>
       <c r="T186" s="49"/>
@@ -30682,32 +30685,32 @@
       <c r="Z186" s="49"/>
       <c r="AA186" s="49"/>
       <c r="AC186" s="154">
-        <f>-AC62/AC175</f>
+        <f>-AC63/AC175</f>
         <v>0</v>
       </c>
     </row>
     <row r="187" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B187" s="20" t="s">
-        <v>287</v>
+        <v>275</v>
       </c>
       <c r="M187" s="154">
-        <f>(-M63-M62)/M175</f>
-        <v>0.9277080695291815</v>
+        <f>-M62/M175</f>
+        <v>0.27800161160354553</v>
       </c>
       <c r="N187" s="154">
-        <f>(-N63-N62)/N175</f>
-        <v>-0.47826780445011563</v>
+        <f>-N62/N175</f>
+        <v>0</v>
       </c>
       <c r="O187" s="154">
-        <f>(-O63-O62)/O175</f>
-        <v>-0.1763765135937857</v>
+        <f>-O62/O175</f>
+        <v>0</v>
       </c>
       <c r="P187" s="154">
-        <f>(-P63-P62)/P175</f>
-        <v>-8.3866568761145496E-2</v>
+        <f>-P62/P175</f>
+        <v>0</v>
       </c>
       <c r="Q187" s="154">
-        <f>(-Q63-Q62)/Q175</f>
+        <f>-Q62/Q175</f>
         <v>0</v>
       </c>
       <c r="T187" s="49"/>
@@ -30719,33 +30722,33 @@
       <c r="Z187" s="49"/>
       <c r="AA187" s="49"/>
       <c r="AC187" s="154">
-        <f>(-AC63-AC62)/AC175</f>
+        <f>-AC62/AC175</f>
         <v>0</v>
       </c>
     </row>
     <row r="188" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B188" s="20" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="M188" s="154">
-        <f>M79/M77</f>
-        <v>4.874482086278333E-4</v>
+        <f>(-M63-M62)/M175</f>
+        <v>0.9277080695291815</v>
       </c>
       <c r="N188" s="154">
-        <f>N79/N77</f>
-        <v>4.8169556840077071E-4</v>
+        <f>(-N63-N62)/N175</f>
+        <v>-0.47826780445011563</v>
       </c>
       <c r="O188" s="154">
-        <f>O79/O77</f>
-        <v>4.7058823529411766E-4</v>
+        <f>(-O63-O62)/O175</f>
+        <v>-0.1763765135937857</v>
       </c>
       <c r="P188" s="154">
-        <f>P79/P77</f>
-        <v>4.6189376443418013E-4</v>
+        <f>(-P63-P62)/P175</f>
+        <v>-8.3866568761145496E-2</v>
       </c>
       <c r="Q188" s="154">
-        <f>Q79/Q77</f>
-        <v>6.0060060060060057E-4</v>
+        <f>(-Q63-Q62)/Q175</f>
+        <v>0</v>
       </c>
       <c r="T188" s="49"/>
       <c r="U188" s="49"/>
@@ -30756,902 +30759,939 @@
       <c r="Z188" s="49"/>
       <c r="AA188" s="49"/>
       <c r="AC188" s="154">
+        <f>(-AC63-AC62)/AC175</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="189" spans="2:29" x14ac:dyDescent="0.2">
+      <c r="B189" s="20" t="s">
+        <v>280</v>
+      </c>
+      <c r="M189" s="154">
+        <f>M79/M77</f>
+        <v>4.874482086278333E-4</v>
+      </c>
+      <c r="N189" s="154">
+        <f>N79/N77</f>
+        <v>4.8169556840077071E-4</v>
+      </c>
+      <c r="O189" s="154">
+        <f>O79/O77</f>
+        <v>4.7058823529411766E-4</v>
+      </c>
+      <c r="P189" s="154">
+        <f>P79/P77</f>
+        <v>4.6189376443418013E-4</v>
+      </c>
+      <c r="Q189" s="154">
+        <f>Q79/Q77</f>
+        <v>6.0060060060060057E-4</v>
+      </c>
+      <c r="T189" s="49"/>
+      <c r="U189" s="49"/>
+      <c r="V189" s="49"/>
+      <c r="W189" s="49"/>
+      <c r="X189" s="49"/>
+      <c r="Y189" s="49"/>
+      <c r="Z189" s="49"/>
+      <c r="AA189" s="49"/>
+      <c r="AC189" s="154">
         <f>AC79/AC77</f>
         <v>5.9689614007162755E-4</v>
       </c>
     </row>
-    <row r="189" spans="2:29" x14ac:dyDescent="0.2">
-      <c r="B189" s="20" t="s">
-        <v>282</v>
-      </c>
-      <c r="M189" s="71">
+    <row r="190" spans="2:29" x14ac:dyDescent="0.2">
+      <c r="B190" s="20" t="s">
+        <v>281</v>
+      </c>
+      <c r="M190" s="71">
         <f>M120/M74</f>
         <v>6.9776522593320234</v>
       </c>
-      <c r="N189" s="71">
+      <c r="N190" s="71">
         <f>N120/N74</f>
         <v>6.8498912255257434</v>
       </c>
-      <c r="O189" s="71">
+      <c r="O190" s="71">
         <f>O120/O74</f>
         <v>5.9210028382213808</v>
       </c>
-      <c r="P189" s="71">
+      <c r="P190" s="71">
         <f>P120/P74</f>
         <v>5.0951501154734409</v>
       </c>
-      <c r="Q189" s="71">
+      <c r="Q190" s="71">
         <f>Q120/Q74</f>
         <v>7.4906906906906903</v>
       </c>
-      <c r="T189" s="71">
-        <f t="shared" ref="T189:AA189" si="113">T120/T74</f>
+      <c r="T190" s="71">
+        <f t="shared" ref="T190:AA190" si="115">T120/T74</f>
         <v>6.8458840037418147</v>
       </c>
-      <c r="U189" s="71">
-        <f t="shared" si="113"/>
+      <c r="U190" s="71">
+        <f t="shared" si="115"/>
         <v>5.5845119406445631</v>
       </c>
-      <c r="V189" s="71">
-        <f t="shared" si="113"/>
+      <c r="V190" s="71">
+        <f t="shared" si="115"/>
         <v>5.0951501154734409</v>
       </c>
-      <c r="W189" s="71">
-        <f t="shared" si="113"/>
+      <c r="W190" s="71">
+        <f t="shared" si="115"/>
         <v>4.825309491059147</v>
       </c>
-      <c r="X189" s="71">
-        <f t="shared" si="113"/>
+      <c r="X190" s="71">
+        <f t="shared" si="115"/>
         <v>4.8448709161526162</v>
       </c>
-      <c r="Y189" s="71">
-        <f t="shared" si="113"/>
+      <c r="Y190" s="71">
+        <f t="shared" si="115"/>
         <v>6.4853249475890982</v>
       </c>
-      <c r="Z189" s="71">
-        <f t="shared" si="113"/>
+      <c r="Z190" s="71">
+        <f t="shared" si="115"/>
         <v>7.4906906906906903</v>
       </c>
-      <c r="AA189" s="71">
-        <f t="shared" si="113"/>
+      <c r="AA190" s="71">
+        <f t="shared" si="115"/>
         <v>6.5238758456028654</v>
       </c>
-      <c r="AC189" s="71">
+      <c r="AC190" s="71">
         <f>AC120/AC74</f>
         <v>6.5238758456028654</v>
       </c>
     </row>
-    <row r="190" spans="2:29" x14ac:dyDescent="0.2">
-      <c r="B190" s="20" t="s">
-        <v>284</v>
-      </c>
-      <c r="M190" s="154">
+    <row r="191" spans="2:29" x14ac:dyDescent="0.2">
+      <c r="B191" s="20" t="s">
+        <v>283</v>
+      </c>
+      <c r="M191" s="154">
         <f>M53/M58</f>
         <v>6.9120043454644217E-2</v>
       </c>
-      <c r="N190" s="154">
+      <c r="N191" s="154">
         <f>N53/N58</f>
         <v>0.20268256333830104</v>
       </c>
-      <c r="O190" s="154">
+      <c r="O191" s="154">
         <f>O53/O58</f>
         <v>0.28149245924505273</v>
       </c>
-      <c r="P190" s="154">
+      <c r="P191" s="154">
         <f>P53/P58</f>
         <v>0.41143822393822393</v>
       </c>
-      <c r="Q190" s="154">
+      <c r="Q191" s="154">
         <f>Q53/Q58</f>
         <v>0.25100546560791998</v>
       </c>
-      <c r="T190" s="154" t="e">
-        <f t="shared" ref="T190:Y190" si="114">T53/T58</f>
+      <c r="T191" s="154" t="e">
+        <f t="shared" ref="T191:Y191" si="116">T53/T58</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="U190" s="154" t="e">
-        <f t="shared" si="114"/>
+      <c r="U191" s="154" t="e">
+        <f t="shared" si="116"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="V190" s="154" t="e">
-        <f t="shared" si="114"/>
+      <c r="V191" s="154" t="e">
+        <f t="shared" si="116"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="W190" s="154">
-        <f t="shared" si="114"/>
+      <c r="W191" s="154">
+        <f t="shared" si="116"/>
         <v>0.84132841328413288</v>
       </c>
-      <c r="X190" s="154">
-        <f t="shared" si="114"/>
+      <c r="X191" s="154">
+        <f t="shared" si="116"/>
         <v>0.32390243902439025</v>
       </c>
-      <c r="Y190" s="154">
-        <f t="shared" si="114"/>
+      <c r="Y191" s="154">
+        <f t="shared" si="116"/>
         <v>0.2152395915161037</v>
       </c>
-      <c r="Z190" s="154">
+      <c r="Z191" s="154">
         <f>W53/W58</f>
         <v>0.84132841328413288</v>
       </c>
-      <c r="AA190" s="154">
+      <c r="AA191" s="154">
         <f>AA53/AA58</f>
         <v>0.56660583941605835</v>
       </c>
-      <c r="AC190" s="154">
+      <c r="AC191" s="154">
         <f>AC53/AC58</f>
         <v>0.2375751503006012</v>
       </c>
     </row>
-    <row r="191" spans="2:29" x14ac:dyDescent="0.2">
-      <c r="B191" s="20" t="s">
-        <v>285</v>
-      </c>
-      <c r="M191" s="154">
+    <row r="192" spans="2:29" x14ac:dyDescent="0.2">
+      <c r="B192" s="20" t="s">
+        <v>284</v>
+      </c>
+      <c r="M192" s="154">
         <f>M53/M5</f>
         <v>2.5764324762097592E-2</v>
       </c>
-      <c r="N191" s="154">
+      <c r="N192" s="154">
         <f>N53/N5</f>
         <v>4.9608272274558315E-2</v>
       </c>
-      <c r="O191" s="154">
+      <c r="O192" s="154">
         <f>O53/O5</f>
         <v>5.9544884561481153E-2</v>
       </c>
-      <c r="P191" s="154">
+      <c r="P192" s="154">
         <f>P53/P5</f>
         <v>6.4217246379540877E-2</v>
       </c>
-      <c r="Q191" s="154">
+      <c r="Q192" s="154">
         <f>Q53/Q5</f>
         <v>4.6052258149963103E-2</v>
       </c>
-      <c r="T191" s="154">
-        <f t="shared" ref="T191:Y191" si="115">T53/T5</f>
-        <v>0</v>
-      </c>
-      <c r="U191" s="154">
-        <f t="shared" si="115"/>
-        <v>0</v>
-      </c>
-      <c r="V191" s="154">
-        <f t="shared" si="115"/>
-        <v>0</v>
-      </c>
-      <c r="W191" s="154">
-        <f t="shared" si="115"/>
+      <c r="T192" s="154">
+        <f t="shared" ref="T192:Y192" si="117">T53/T5</f>
+        <v>0</v>
+      </c>
+      <c r="U192" s="154">
+        <f t="shared" si="117"/>
+        <v>0</v>
+      </c>
+      <c r="V192" s="154">
+        <f t="shared" si="117"/>
+        <v>0</v>
+      </c>
+      <c r="W192" s="154">
+        <f t="shared" si="117"/>
         <v>5.3998578984763561E-2</v>
       </c>
-      <c r="X191" s="154">
-        <f t="shared" si="115"/>
+      <c r="X192" s="154">
+        <f t="shared" si="117"/>
         <v>5.1636985768722297E-2</v>
       </c>
-      <c r="Y191" s="154">
-        <f t="shared" si="115"/>
+      <c r="Y192" s="154">
+        <f t="shared" si="117"/>
         <v>4.0137698674284038E-2</v>
       </c>
-      <c r="Z191" s="154">
+      <c r="Z192" s="154">
         <f>W53/Z5</f>
         <v>5.0021939447125935E-2</v>
       </c>
-      <c r="AA191" s="154">
+      <c r="AA192" s="154">
         <f>AA53/AA5</f>
         <v>4.5739117625395891E-2</v>
       </c>
-      <c r="AC191" s="154">
+      <c r="AC192" s="154">
         <f>AC53/AC5</f>
         <v>4.4100961627885349E-2</v>
       </c>
     </row>
-    <row r="192" spans="2:29" x14ac:dyDescent="0.2">
-      <c r="B192" s="20" t="s">
-        <v>290</v>
-      </c>
-      <c r="M192" s="71">
+    <row r="193" spans="2:29" x14ac:dyDescent="0.2">
+      <c r="B193" s="20" t="s">
+        <v>289</v>
+      </c>
+      <c r="M193" s="71">
         <f>(M120-M121)/M74</f>
         <v>-2.3791748526522594</v>
       </c>
-      <c r="N192" s="71">
+      <c r="N193" s="71">
         <f>(N120-N121)/N74</f>
         <v>-3.3147208121827409</v>
       </c>
-      <c r="O192" s="71">
+      <c r="O193" s="71">
         <f>(O120-O121)/O74</f>
         <v>-5.7313150425733204</v>
       </c>
-      <c r="P192" s="71">
+      <c r="P193" s="71">
         <f>(P120-P121)/P74</f>
         <v>-6.4547344110854503</v>
       </c>
-      <c r="Q192" s="71">
+      <c r="Q193" s="71">
         <f>(Q120-Q121)/Q74</f>
         <v>-1.8356356356356356</v>
       </c>
-      <c r="T192" s="71">
-        <f t="shared" ref="T192:AA192" si="116">(T120-T121)/T74</f>
+      <c r="T193" s="71">
+        <f t="shared" ref="T193:AA193" si="118">(T120-T121)/T74</f>
         <v>-5.5556594948550044</v>
       </c>
-      <c r="U192" s="71">
-        <f t="shared" si="116"/>
+      <c r="U193" s="71">
+        <f t="shared" si="118"/>
         <v>-6.06306515186645</v>
       </c>
-      <c r="V192" s="71">
-        <f t="shared" si="116"/>
+      <c r="V193" s="71">
+        <f t="shared" si="118"/>
         <v>-6.4547344110854503</v>
       </c>
-      <c r="W192" s="71">
-        <f t="shared" si="116"/>
+      <c r="W193" s="71">
+        <f t="shared" si="118"/>
         <v>-6.6719394773039893</v>
       </c>
-      <c r="X192" s="71">
-        <f t="shared" si="116"/>
+      <c r="X193" s="71">
+        <f t="shared" si="118"/>
         <v>-6.7514279186657529</v>
       </c>
-      <c r="Y192" s="71">
-        <f t="shared" si="116"/>
+      <c r="Y193" s="71">
+        <f t="shared" si="118"/>
         <v>-3.2742138364779874</v>
       </c>
-      <c r="Z192" s="71">
-        <f t="shared" si="116"/>
+      <c r="Z193" s="71">
+        <f t="shared" si="118"/>
         <v>-1.8356356356356356</v>
       </c>
-      <c r="AA192" s="71">
-        <f t="shared" si="116"/>
+      <c r="AA193" s="71">
+        <f t="shared" si="118"/>
         <v>-2.435734182252288</v>
       </c>
-      <c r="AC192" s="71">
+      <c r="AC193" s="71">
         <f>(AC120-AC121)/AC74</f>
         <v>-2.435734182252288</v>
       </c>
     </row>
-    <row r="193" spans="2:29" x14ac:dyDescent="0.2">
-      <c r="B193" s="20" t="s">
-        <v>295</v>
-      </c>
-      <c r="M193" s="154">
+    <row r="194" spans="2:29" x14ac:dyDescent="0.2">
+      <c r="B194" s="20" t="s">
+        <v>294</v>
+      </c>
+      <c r="M194" s="154">
         <f>(M120-M121)/M171</f>
         <v>-4.601830291547894E-2</v>
       </c>
-      <c r="N193" s="154">
+      <c r="N194" s="154">
         <f>(N120-N121)/N171</f>
         <v>-0.12496200017933728</v>
       </c>
-      <c r="O193" s="154">
+      <c r="O194" s="154">
         <f>(O120-O121)/O171</f>
         <v>-0.11346561311091601</v>
       </c>
-      <c r="P193" s="154">
+      <c r="P194" s="154">
         <f>(P120-P121)/P171</f>
         <v>-0.31796721236874137</v>
       </c>
-      <c r="Q193" s="154">
+      <c r="Q194" s="154">
         <f>(Q120-Q121)/Q171</f>
         <v>-5.070816673026618E-2</v>
       </c>
-      <c r="T193" s="49"/>
-      <c r="U193" s="49"/>
-      <c r="V193" s="49"/>
-      <c r="W193" s="49"/>
-      <c r="X193" s="49"/>
-      <c r="Y193" s="49"/>
-      <c r="Z193" s="49"/>
-      <c r="AA193" s="49"/>
-      <c r="AC193" s="154">
+      <c r="T194" s="49"/>
+      <c r="U194" s="49"/>
+      <c r="V194" s="49"/>
+      <c r="W194" s="49"/>
+      <c r="X194" s="49"/>
+      <c r="Y194" s="49"/>
+      <c r="Z194" s="49"/>
+      <c r="AA194" s="49"/>
+      <c r="AC194" s="154">
         <f ca="1">(AC120-AC121)/AC171</f>
         <v>-2.4561199780702713E-2</v>
       </c>
     </row>
-    <row r="194" spans="2:29" x14ac:dyDescent="0.2">
-      <c r="B194" s="20" t="s">
-        <v>304</v>
-      </c>
-      <c r="M194" s="154">
+    <row r="195" spans="2:29" x14ac:dyDescent="0.2">
+      <c r="B195" s="20" t="s">
+        <v>303</v>
+      </c>
+      <c r="M195" s="154">
         <f>-M123/M5</f>
         <v>0.23705456570155903</v>
       </c>
-      <c r="N194" s="154">
+      <c r="N195" s="154">
         <f>-N123/N5</f>
         <v>0.39401148222158783</v>
       </c>
-      <c r="O194" s="154">
+      <c r="O195" s="154">
         <f>-O123/O5</f>
         <v>0.4748469425389098</v>
       </c>
-      <c r="P194" s="154">
+      <c r="P195" s="154">
         <f>-P123/P5</f>
         <v>0.45091429539933336</v>
       </c>
-      <c r="Q194" s="154">
+      <c r="Q195" s="154">
         <f>-Q123/Q5</f>
         <v>0.27710820577829071</v>
       </c>
-      <c r="T194" s="154">
-        <f t="shared" ref="T194:AA194" si="117">-T123/T5</f>
-        <v>0</v>
-      </c>
-      <c r="U194" s="154">
-        <f t="shared" si="117"/>
-        <v>0</v>
-      </c>
-      <c r="V194" s="154">
-        <f t="shared" si="117"/>
-        <v>0</v>
-      </c>
-      <c r="W194" s="154">
-        <f t="shared" si="117"/>
+      <c r="T195" s="154">
+        <f t="shared" ref="T195:AA195" si="119">-T123/T5</f>
+        <v>0</v>
+      </c>
+      <c r="U195" s="154">
+        <f t="shared" si="119"/>
+        <v>0</v>
+      </c>
+      <c r="V195" s="154">
+        <f t="shared" si="119"/>
+        <v>0</v>
+      </c>
+      <c r="W195" s="154">
+        <f t="shared" si="119"/>
         <v>0.40917344280413676</v>
       </c>
-      <c r="X194" s="154">
-        <f t="shared" si="117"/>
+      <c r="X195" s="154">
+        <f t="shared" si="119"/>
         <v>0.27607123415506651</v>
       </c>
-      <c r="Y194" s="154">
-        <f t="shared" si="117"/>
+      <c r="Y195" s="154">
+        <f t="shared" si="119"/>
         <v>0.17761664103127517</v>
       </c>
-      <c r="Z194" s="154">
-        <f t="shared" si="117"/>
+      <c r="Z195" s="154">
+        <f t="shared" si="119"/>
         <v>0.25508263858417435</v>
       </c>
-      <c r="AA194" s="154">
-        <f t="shared" si="117"/>
+      <c r="AA195" s="154">
+        <f t="shared" si="119"/>
         <v>0.2678058481255064</v>
       </c>
-      <c r="AC194" s="154">
+      <c r="AC195" s="154">
         <f>-AC123/AC5</f>
         <v>0.24364339787586259</v>
       </c>
     </row>
-    <row r="195" spans="2:29" x14ac:dyDescent="0.2">
-      <c r="B195" s="20" t="s">
-        <v>305</v>
-      </c>
-      <c r="M195" s="154">
+    <row r="196" spans="2:29" x14ac:dyDescent="0.2">
+      <c r="B196" s="20" t="s">
+        <v>304</v>
+      </c>
+      <c r="M196" s="154">
         <f>-(M123/M58)</f>
         <v>0.63596550787615425</v>
       </c>
-      <c r="N195" s="154">
+      <c r="N196" s="154">
         <f>-(N123/N58)</f>
         <v>1.6097971878442299</v>
       </c>
-      <c r="O195" s="154">
+      <c r="O196" s="154">
         <f>-(O123/O58)</f>
         <v>2.2447912126231366</v>
       </c>
-      <c r="P195" s="154">
+      <c r="P196" s="154">
         <f>-(P123/P58)</f>
         <v>2.8889961389961392</v>
       </c>
-      <c r="Q195" s="154">
+      <c r="Q196" s="154">
         <f>-(Q123/Q58)</f>
         <v>1.5103640301124059</v>
       </c>
-      <c r="T195" s="154" t="e">
-        <f t="shared" ref="T195:Y195" si="118">-(T123/T58)</f>
+      <c r="T196" s="154" t="e">
+        <f t="shared" ref="T196:Y196" si="120">-(T123/T58)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="U195" s="154" t="e">
-        <f t="shared" si="118"/>
+      <c r="U196" s="154" t="e">
+        <f t="shared" si="120"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="V195" s="154" t="e">
-        <f t="shared" si="118"/>
+      <c r="V196" s="154" t="e">
+        <f t="shared" si="120"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="W195" s="154">
-        <f t="shared" si="118"/>
+      <c r="W196" s="154">
+        <f t="shared" si="120"/>
         <v>6.375153751537515</v>
       </c>
-      <c r="X195" s="154">
-        <f t="shared" si="118"/>
+      <c r="X196" s="154">
+        <f t="shared" si="120"/>
         <v>1.7317073170731707</v>
       </c>
-      <c r="Y195" s="154">
-        <f t="shared" si="118"/>
+      <c r="Y196" s="154">
+        <f t="shared" si="120"/>
         <v>0.95247446975648076</v>
       </c>
-      <c r="Z195" s="154">
+      <c r="Z196" s="154">
         <f>-(Z123/W58)</f>
         <v>4.2902829028290279</v>
       </c>
-      <c r="AA195" s="154">
+      <c r="AA196" s="154">
         <f>-(AA123/AA58)</f>
         <v>3.3175182481751824</v>
       </c>
-      <c r="AC195" s="154">
+      <c r="AC196" s="154">
         <f>-(AC123/AC58)</f>
         <v>1.3125250501002004</v>
       </c>
     </row>
-    <row r="196" spans="2:29" x14ac:dyDescent="0.2">
-      <c r="B196" s="20" t="s">
-        <v>306</v>
-      </c>
-      <c r="M196" s="154">
+    <row r="197" spans="2:29" x14ac:dyDescent="0.2">
+      <c r="B197" s="20" t="s">
+        <v>305</v>
+      </c>
+      <c r="M197" s="154">
         <f>-M123/M52</f>
         <v>1.5886194029850746</v>
       </c>
-      <c r="N196" s="154">
+      <c r="N197" s="154">
         <f>-N123/N52</f>
         <v>1.9059455312619868</v>
       </c>
-      <c r="O196" s="154">
+      <c r="O197" s="154">
         <f>-O123/O52</f>
         <v>2.6817329722974379</v>
       </c>
-      <c r="P196" s="154">
+      <c r="P197" s="154">
         <f>-P123/P52</f>
         <v>2.1042270849811056</v>
       </c>
-      <c r="Q196" s="154">
+      <c r="Q197" s="154">
         <f>-Q123/Q52</f>
         <v>1.2511532547411583</v>
       </c>
-      <c r="T196" s="154" t="e">
-        <f t="shared" ref="T196:Y196" si="119">-T123/T52</f>
+      <c r="T197" s="154" t="e">
+        <f t="shared" ref="T197:Y197" si="121">-T123/T52</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="U196" s="154" t="e">
-        <f t="shared" si="119"/>
+      <c r="U197" s="154" t="e">
+        <f t="shared" si="121"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="V196" s="154" t="e">
-        <f t="shared" si="119"/>
+      <c r="V197" s="154" t="e">
+        <f t="shared" si="121"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="W196" s="154">
-        <f t="shared" si="119"/>
+      <c r="W197" s="154">
+        <f t="shared" si="121"/>
         <v>1.9382946896035902</v>
       </c>
-      <c r="X196" s="154">
-        <f t="shared" si="119"/>
+      <c r="X197" s="154">
+        <f t="shared" si="121"/>
         <v>1.1782276800531033</v>
       </c>
-      <c r="Y196" s="154">
-        <f t="shared" si="119"/>
+      <c r="Y197" s="154">
+        <f t="shared" si="121"/>
         <v>0.81049465240641716</v>
       </c>
-      <c r="Z196" s="154">
+      <c r="Z197" s="154">
         <f>-Z123/W52</f>
         <v>1.3044128646222888</v>
       </c>
-      <c r="AA196" s="154">
+      <c r="AA197" s="154">
         <f>-AA123/AA52</f>
         <v>1.159438775510204</v>
       </c>
-      <c r="AC196" s="154">
+      <c r="AC197" s="154">
         <f>-AC123/AC52</f>
         <v>1.0765121630506247</v>
       </c>
     </row>
-    <row r="198" spans="2:29" x14ac:dyDescent="0.2">
-      <c r="B198" s="1"/>
-    </row>
-    <row r="199" spans="2:29" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B199" s="14" t="s">
-        <v>315</v>
-      </c>
-      <c r="C199" s="172"/>
-      <c r="D199" s="172"/>
-      <c r="E199" s="172"/>
-      <c r="F199" s="172"/>
-      <c r="G199" s="172"/>
-      <c r="H199" s="172"/>
-      <c r="I199" s="172"/>
-      <c r="J199" s="172"/>
-      <c r="K199" s="172"/>
-      <c r="L199" s="172"/>
-      <c r="M199" s="172"/>
-      <c r="N199" s="172"/>
-      <c r="O199" s="172"/>
-      <c r="P199" s="172"/>
-      <c r="Q199" s="172"/>
-      <c r="T199" s="172"/>
-      <c r="U199" s="172"/>
-      <c r="V199" s="172"/>
-      <c r="W199" s="172"/>
-      <c r="X199" s="172"/>
-      <c r="Y199" s="172"/>
-      <c r="Z199" s="172"/>
-      <c r="AA199" s="172"/>
-      <c r="AC199" s="172"/>
-    </row>
-    <row r="200" spans="2:29" x14ac:dyDescent="0.2">
-      <c r="B200" s="218" t="s">
-        <v>362</v>
-      </c>
-      <c r="C200" s="80"/>
-      <c r="D200" s="80"/>
-      <c r="E200" s="80"/>
-      <c r="F200" s="80"/>
-      <c r="G200" s="80"/>
-      <c r="H200" s="80"/>
-      <c r="I200" s="80"/>
-      <c r="J200" s="80"/>
-      <c r="K200" s="80"/>
-      <c r="L200" s="80"/>
-      <c r="M200" s="80">
-        <f t="shared" ref="M200:Q204" si="120">IF(L105=0,
+    <row r="199" spans="2:29" x14ac:dyDescent="0.2">
+      <c r="B199" s="1"/>
+    </row>
+    <row r="200" spans="2:29" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B200" s="14" t="s">
+        <v>314</v>
+      </c>
+      <c r="C200" s="172"/>
+      <c r="D200" s="172"/>
+      <c r="E200" s="172"/>
+      <c r="F200" s="172"/>
+      <c r="G200" s="172"/>
+      <c r="H200" s="172"/>
+      <c r="I200" s="172"/>
+      <c r="J200" s="172"/>
+      <c r="K200" s="172"/>
+      <c r="L200" s="172"/>
+      <c r="M200" s="172"/>
+      <c r="N200" s="172"/>
+      <c r="O200" s="172"/>
+      <c r="P200" s="172"/>
+      <c r="Q200" s="172"/>
+      <c r="T200" s="172"/>
+      <c r="U200" s="172"/>
+      <c r="V200" s="172"/>
+      <c r="W200" s="172"/>
+      <c r="X200" s="172"/>
+      <c r="Y200" s="172"/>
+      <c r="Z200" s="172"/>
+      <c r="AA200" s="172"/>
+      <c r="AC200" s="172"/>
+    </row>
+    <row r="201" spans="2:29" x14ac:dyDescent="0.2">
+      <c r="B201" s="218" t="s">
+        <v>361</v>
+      </c>
+      <c r="C201" s="80"/>
+      <c r="D201" s="80"/>
+      <c r="E201" s="80"/>
+      <c r="F201" s="80"/>
+      <c r="G201" s="80"/>
+      <c r="H201" s="80"/>
+      <c r="I201" s="80"/>
+      <c r="J201" s="80"/>
+      <c r="K201" s="80"/>
+      <c r="L201" s="80"/>
+      <c r="M201" s="80">
+        <f t="shared" ref="M201:Q205" si="122">IF(L105=0,
 IF(M105=0,0,IF(M105&gt;0,1,-1)),
 (M105-L105)/ABS(L105)
 )</f>
         <v>1</v>
       </c>
-      <c r="N200" s="80">
-        <f t="shared" si="120"/>
+      <c r="N201" s="80">
+        <f t="shared" si="122"/>
         <v>-0.22657676298045326</v>
       </c>
-      <c r="O200" s="80">
-        <f t="shared" si="120"/>
+      <c r="O201" s="80">
+        <f t="shared" si="122"/>
         <v>-7.9155257608661447E-2</v>
       </c>
-      <c r="P200" s="80">
-        <f t="shared" si="120"/>
+      <c r="P201" s="80">
+        <f t="shared" si="122"/>
         <v>0.139722469068289</v>
       </c>
-      <c r="Q200" s="80">
-        <f t="shared" si="120"/>
+      <c r="Q201" s="80">
+        <f t="shared" si="122"/>
         <v>-3.3527259641336293E-2</v>
       </c>
-      <c r="T200" s="80">
-        <f t="shared" ref="T200:AA204" si="121">IF(S105=0,
+      <c r="T201" s="80">
+        <f t="shared" ref="T201:AA205" si="123">IF(S105=0,
 IF(T105=0,0,IF(T105&gt;0,1,-1)),
 (T105-S105)/ABS(S105)
 )</f>
         <v>1</v>
       </c>
-      <c r="U200" s="80">
-        <f t="shared" si="121"/>
+      <c r="U201" s="80">
+        <f t="shared" si="123"/>
         <v>2.2104875353063983E-3</v>
       </c>
-      <c r="V200" s="80">
-        <f t="shared" si="121"/>
+      <c r="V201" s="80">
+        <f t="shared" si="123"/>
         <v>7.4500673937017522E-2</v>
       </c>
-      <c r="W200" s="80">
-        <f t="shared" si="121"/>
+      <c r="W201" s="80">
+        <f t="shared" si="123"/>
         <v>-0.13000342114266164</v>
       </c>
-      <c r="X200" s="80">
-        <f t="shared" si="121"/>
+      <c r="X201" s="80">
+        <f t="shared" si="123"/>
         <v>3.1721064359680168E-2</v>
       </c>
-      <c r="Y200" s="80">
-        <f t="shared" si="121"/>
+      <c r="Y201" s="80">
+        <f t="shared" si="123"/>
         <v>8.436030999872951E-2</v>
       </c>
-      <c r="Z200" s="80">
-        <f t="shared" si="121"/>
+      <c r="Z201" s="80">
+        <f t="shared" si="123"/>
         <v>-4.0070298769771528E-2</v>
       </c>
-      <c r="AA200" s="80">
-        <f t="shared" si="121"/>
+      <c r="AA201" s="80">
+        <f t="shared" si="123"/>
         <v>-5.687782253142927E-2</v>
       </c>
-      <c r="AC200" s="49"/>
-    </row>
-    <row r="201" spans="2:29" x14ac:dyDescent="0.2">
-      <c r="B201" s="218" t="s">
-        <v>363</v>
-      </c>
-      <c r="M201" s="80">
-        <f t="shared" si="120"/>
+      <c r="AC201" s="49"/>
+    </row>
+    <row r="202" spans="2:29" x14ac:dyDescent="0.2">
+      <c r="B202" s="218" t="s">
+        <v>362</v>
+      </c>
+      <c r="M202" s="80">
+        <f t="shared" si="122"/>
         <v>1</v>
       </c>
-      <c r="N201" s="80">
-        <f t="shared" si="120"/>
+      <c r="N202" s="80">
+        <f t="shared" si="122"/>
         <v>-8.4923946253162061E-2</v>
       </c>
-      <c r="O201" s="80">
-        <f t="shared" si="120"/>
+      <c r="O202" s="80">
+        <f t="shared" si="122"/>
         <v>-0.23547784878293962</v>
       </c>
-      <c r="P201" s="80">
-        <f t="shared" si="120"/>
+      <c r="P202" s="80">
+        <f t="shared" si="122"/>
         <v>-0.242779995304062</v>
       </c>
-      <c r="Q201" s="80">
-        <f t="shared" si="120"/>
+      <c r="Q202" s="80">
+        <f t="shared" si="122"/>
         <v>4.9240310077519382E-2</v>
       </c>
-      <c r="T201" s="80">
-        <f t="shared" si="121"/>
+      <c r="T202" s="80">
+        <f t="shared" si="123"/>
         <v>1</v>
       </c>
-      <c r="U201" s="80">
-        <f t="shared" si="121"/>
+      <c r="U202" s="80">
+        <f t="shared" si="123"/>
         <v>8.8304862023653091E-2</v>
       </c>
-      <c r="V201" s="80">
-        <f t="shared" si="121"/>
+      <c r="V202" s="80">
+        <f t="shared" si="123"/>
         <v>5.0712388312001935E-2</v>
       </c>
-      <c r="W201" s="80">
-        <f t="shared" si="121"/>
+      <c r="W202" s="80">
+        <f t="shared" si="123"/>
         <v>-5.1712250057458053E-2</v>
       </c>
-      <c r="X201" s="80">
-        <f t="shared" si="121"/>
+      <c r="X202" s="80">
+        <f t="shared" si="123"/>
         <v>-4.5322346097915654E-2</v>
       </c>
-      <c r="Y201" s="80">
-        <f t="shared" si="121"/>
+      <c r="Y202" s="80">
+        <f t="shared" si="123"/>
         <v>4.5189134298045192E-2</v>
       </c>
-      <c r="Z201" s="80">
-        <f t="shared" si="121"/>
+      <c r="Z202" s="80">
+        <f t="shared" si="123"/>
         <v>0.15059509351469516</v>
       </c>
-      <c r="AA201" s="80">
-        <f t="shared" si="121"/>
+      <c r="AA202" s="80">
+        <f t="shared" si="123"/>
         <v>6.6497783407219763E-2</v>
-      </c>
-      <c r="AC201" s="49"/>
-    </row>
-    <row r="202" spans="2:29" x14ac:dyDescent="0.2">
-      <c r="B202" s="20" t="s">
-        <v>364</v>
-      </c>
-      <c r="M202" s="80">
-        <f t="shared" si="120"/>
-        <v>1</v>
-      </c>
-      <c r="N202" s="80">
-        <f t="shared" si="120"/>
-        <v>-0.16628914988814317</v>
-      </c>
-      <c r="O202" s="80">
-        <f t="shared" si="120"/>
-        <v>-0.1521793818236705</v>
-      </c>
-      <c r="P202" s="80">
-        <f t="shared" si="120"/>
-        <v>-2.1403279726227919E-2</v>
-      </c>
-      <c r="Q202" s="80">
-        <f t="shared" si="120"/>
-        <v>-6.5492915041135214E-3</v>
-      </c>
-      <c r="T202" s="80">
-        <f t="shared" si="121"/>
-        <v>1</v>
-      </c>
-      <c r="U202" s="80">
-        <f t="shared" si="121"/>
-        <v>2.9628389688650822E-2</v>
-      </c>
-      <c r="V202" s="80">
-        <f t="shared" si="121"/>
-        <v>6.6493253129572424E-2</v>
-      </c>
-      <c r="W202" s="80">
-        <f t="shared" si="121"/>
-        <v>-0.10403963414634146</v>
-      </c>
-      <c r="X202" s="80">
-        <f t="shared" si="121"/>
-        <v>4.6788600595491277E-3</v>
-      </c>
-      <c r="Y202" s="80">
-        <f t="shared" si="121"/>
-        <v>7.1295512277730733E-2</v>
-      </c>
-      <c r="Z202" s="80">
-        <f t="shared" si="121"/>
-        <v>2.1972810622826432E-2</v>
-      </c>
-      <c r="AA202" s="80">
-        <f t="shared" si="121"/>
-        <v>-1.1678267594740912E-2</v>
       </c>
       <c r="AC202" s="49"/>
     </row>
     <row r="203" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B203" s="20" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="M203" s="80">
-        <f t="shared" si="120"/>
+        <f t="shared" si="122"/>
         <v>1</v>
       </c>
       <c r="N203" s="80">
-        <f t="shared" si="120"/>
-        <v>0.35158501440922191</v>
+        <f t="shared" si="122"/>
+        <v>-0.16628914988814317</v>
       </c>
       <c r="O203" s="80">
-        <f t="shared" si="120"/>
-        <v>1.0298507462686568</v>
+        <f t="shared" si="122"/>
+        <v>-0.1521793818236705</v>
       </c>
       <c r="P203" s="80">
-        <f t="shared" si="120"/>
-        <v>17.190126050420169</v>
+        <f t="shared" si="122"/>
+        <v>-2.1403279726227919E-2</v>
       </c>
       <c r="Q203" s="80">
-        <f t="shared" si="120"/>
-        <v>2.9393081942599757E-2</v>
+        <f t="shared" si="122"/>
+        <v>-6.5492915041135214E-3</v>
       </c>
       <c r="T203" s="80">
-        <f t="shared" si="121"/>
+        <f t="shared" si="123"/>
         <v>1</v>
       </c>
       <c r="U203" s="80">
-        <f t="shared" si="121"/>
-        <v>1.3311536665109761E-2</v>
+        <f t="shared" si="123"/>
+        <v>2.9628389688650822E-2</v>
       </c>
       <c r="V203" s="80">
-        <f t="shared" si="121"/>
-        <v>2.3046784973496196E-4</v>
+        <f t="shared" si="123"/>
+        <v>6.6493253129572424E-2</v>
       </c>
       <c r="W203" s="80">
-        <f t="shared" si="121"/>
-        <v>7.5345622119815672E-2</v>
+        <f t="shared" si="123"/>
+        <v>-0.10403963414634146</v>
       </c>
       <c r="X203" s="80">
-        <f t="shared" si="121"/>
-        <v>-5.3567602314120423E-2</v>
+        <f t="shared" si="123"/>
+        <v>4.6788600595491277E-3</v>
       </c>
       <c r="Y203" s="80">
-        <f t="shared" si="121"/>
-        <v>-4.1204437400950873E-2</v>
+        <f t="shared" si="123"/>
+        <v>7.1295512277730733E-2</v>
       </c>
       <c r="Z203" s="80">
-        <f t="shared" si="121"/>
-        <v>6.4226682408500588E-2</v>
+        <f t="shared" si="123"/>
+        <v>2.1972810622826432E-2</v>
       </c>
       <c r="AA203" s="80">
-        <f t="shared" si="121"/>
-        <v>0.2027956512092301</v>
+        <f t="shared" si="123"/>
+        <v>-1.1678267594740912E-2</v>
       </c>
       <c r="AC203" s="49"/>
     </row>
     <row r="204" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B204" s="20" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="M204" s="80">
-        <f t="shared" si="120"/>
+        <f t="shared" si="122"/>
         <v>1</v>
       </c>
       <c r="N204" s="80">
-        <f t="shared" si="120"/>
+        <f t="shared" si="122"/>
+        <v>0.35158501440922191</v>
+      </c>
+      <c r="O204" s="80">
+        <f t="shared" si="122"/>
+        <v>1.0298507462686568</v>
+      </c>
+      <c r="P204" s="80">
+        <f t="shared" si="122"/>
+        <v>17.190126050420169</v>
+      </c>
+      <c r="Q204" s="80">
+        <f t="shared" si="122"/>
+        <v>2.9393081942599757E-2</v>
+      </c>
+      <c r="T204" s="80">
+        <f t="shared" si="123"/>
+        <v>1</v>
+      </c>
+      <c r="U204" s="80">
+        <f t="shared" si="123"/>
+        <v>1.3311536665109761E-2</v>
+      </c>
+      <c r="V204" s="80">
+        <f t="shared" si="123"/>
+        <v>2.3046784973496196E-4</v>
+      </c>
+      <c r="W204" s="80">
+        <f t="shared" si="123"/>
+        <v>7.5345622119815672E-2</v>
+      </c>
+      <c r="X204" s="80">
+        <f t="shared" si="123"/>
+        <v>-5.3567602314120423E-2</v>
+      </c>
+      <c r="Y204" s="80">
+        <f t="shared" si="123"/>
+        <v>-4.1204437400950873E-2</v>
+      </c>
+      <c r="Z204" s="80">
+        <f t="shared" si="123"/>
+        <v>6.4226682408500588E-2</v>
+      </c>
+      <c r="AA204" s="80">
+        <f t="shared" si="123"/>
+        <v>0.2027956512092301</v>
+      </c>
+      <c r="AC204" s="49"/>
+    </row>
+    <row r="205" spans="2:29" x14ac:dyDescent="0.2">
+      <c r="B205" s="20" t="s">
+        <v>365</v>
+      </c>
+      <c r="M205" s="80">
+        <f t="shared" si="122"/>
+        <v>1</v>
+      </c>
+      <c r="N205" s="80">
+        <f t="shared" si="122"/>
         <v>-0.58669833729216148</v>
       </c>
-      <c r="O204" s="80">
-        <f t="shared" si="120"/>
+      <c r="O205" s="80">
+        <f t="shared" si="122"/>
         <v>-7.9445571331981074E-2</v>
       </c>
-      <c r="P204" s="80">
-        <f t="shared" si="120"/>
+      <c r="P205" s="80">
+        <f t="shared" si="122"/>
         <v>0.32243848696290855</v>
       </c>
-      <c r="Q204" s="80">
-        <f t="shared" si="120"/>
+      <c r="Q205" s="80">
+        <f t="shared" si="122"/>
         <v>-1.0552624271035824E-2</v>
       </c>
-      <c r="T204" s="80">
-        <f t="shared" si="121"/>
+      <c r="T205" s="80">
+        <f t="shared" si="123"/>
         <v>1</v>
       </c>
-      <c r="U204" s="80">
-        <f t="shared" si="121"/>
+      <c r="U205" s="80">
+        <f t="shared" si="123"/>
         <v>9.4211123723041995E-2</v>
       </c>
-      <c r="V204" s="80">
-        <f t="shared" si="121"/>
+      <c r="V205" s="80">
+        <f t="shared" si="123"/>
         <v>0.1545643153526971</v>
       </c>
-      <c r="W204" s="80">
-        <f t="shared" si="121"/>
+      <c r="W205" s="80">
+        <f t="shared" si="123"/>
         <v>-0.1527403414195867</v>
       </c>
-      <c r="X204" s="80">
-        <f t="shared" si="121"/>
+      <c r="X205" s="80">
+        <f t="shared" si="123"/>
         <v>0.11664899257688228</v>
       </c>
-      <c r="Y204" s="80">
-        <f t="shared" si="121"/>
+      <c r="Y205" s="80">
+        <f t="shared" si="123"/>
         <v>-5.6980056980056981E-2</v>
       </c>
-      <c r="Z204" s="80">
-        <f t="shared" si="121"/>
+      <c r="Z205" s="80">
+        <f t="shared" si="123"/>
         <v>-0.42195367573011078</v>
       </c>
-      <c r="AA204" s="80">
-        <f t="shared" si="121"/>
+      <c r="AA205" s="80">
+        <f t="shared" si="123"/>
         <v>9.4076655052264813E-2</v>
       </c>
-      <c r="AC204" s="49"/>
-    </row>
-    <row r="206" spans="2:29" x14ac:dyDescent="0.2">
-      <c r="B206" s="1"/>
-    </row>
-    <row r="207" spans="2:29" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B207" s="14" t="s">
-        <v>316</v>
-      </c>
-      <c r="C207" s="172"/>
-      <c r="D207" s="172"/>
-      <c r="E207" s="172"/>
-      <c r="F207" s="172"/>
-      <c r="G207" s="172"/>
-      <c r="H207" s="172"/>
-      <c r="I207" s="172"/>
-      <c r="J207" s="172"/>
-      <c r="K207" s="172"/>
-      <c r="L207" s="172"/>
-      <c r="M207" s="172"/>
-      <c r="N207" s="172"/>
-      <c r="O207" s="172"/>
-      <c r="P207" s="172"/>
-      <c r="Q207" s="172"/>
-      <c r="T207" s="172"/>
-      <c r="U207" s="172"/>
-      <c r="V207" s="172"/>
-      <c r="W207" s="172"/>
-      <c r="X207" s="172"/>
-      <c r="Y207" s="172"/>
-      <c r="Z207" s="172"/>
-      <c r="AA207" s="172"/>
-      <c r="AC207" s="172"/>
-    </row>
-    <row r="208" spans="2:29" x14ac:dyDescent="0.2">
-      <c r="B208" s="20" t="s">
-        <v>288</v>
-      </c>
-      <c r="C208" s="80"/>
-      <c r="D208" s="80"/>
-      <c r="E208" s="80"/>
-      <c r="F208" s="80"/>
-      <c r="G208" s="80"/>
-      <c r="H208" s="80"/>
-      <c r="I208" s="80"/>
-      <c r="J208" s="80"/>
-      <c r="K208" s="80"/>
-      <c r="L208" s="80"/>
-      <c r="M208" s="80">
+      <c r="AC205" s="49"/>
+    </row>
+    <row r="207" spans="2:29" x14ac:dyDescent="0.2">
+      <c r="B207" s="1"/>
+    </row>
+    <row r="208" spans="2:29" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B208" s="14" t="s">
+        <v>315</v>
+      </c>
+      <c r="C208" s="172"/>
+      <c r="D208" s="172"/>
+      <c r="E208" s="172"/>
+      <c r="F208" s="172"/>
+      <c r="G208" s="172"/>
+      <c r="H208" s="172"/>
+      <c r="I208" s="172"/>
+      <c r="J208" s="172"/>
+      <c r="K208" s="172"/>
+      <c r="L208" s="172"/>
+      <c r="M208" s="172"/>
+      <c r="N208" s="172"/>
+      <c r="O208" s="172"/>
+      <c r="P208" s="172"/>
+      <c r="Q208" s="172"/>
+      <c r="T208" s="172"/>
+      <c r="U208" s="172"/>
+      <c r="V208" s="172"/>
+      <c r="W208" s="172"/>
+      <c r="X208" s="172"/>
+      <c r="Y208" s="172"/>
+      <c r="Z208" s="172"/>
+      <c r="AA208" s="172"/>
+      <c r="AC208" s="172"/>
+    </row>
+    <row r="209" spans="2:29" x14ac:dyDescent="0.2">
+      <c r="B209" s="20" t="s">
+        <v>287</v>
+      </c>
+      <c r="C209" s="80"/>
+      <c r="D209" s="80"/>
+      <c r="E209" s="80"/>
+      <c r="F209" s="80"/>
+      <c r="G209" s="80"/>
+      <c r="H209" s="80"/>
+      <c r="I209" s="80"/>
+      <c r="J209" s="80"/>
+      <c r="K209" s="80"/>
+      <c r="L209" s="80"/>
+      <c r="M209" s="80">
         <f>IF(L63=0,
 IF(M63=0,0,IF(M63&gt;0,1,-1)),
 (M63-L63)/L63
 )</f>
         <v>-1</v>
       </c>
-      <c r="N208" s="80">
+      <c r="N209" s="80">
         <f>IF(M63=0,
 IF(N63=0,0,IF(N63&gt;0,1,-1)),
 (N63-M63)/M63
 )</f>
         <v>6.2544294826364283E-2</v>
       </c>
-      <c r="O208" s="80">
+      <c r="O209" s="80">
         <f>IF(N63=0,
 IF(O63=0,0,IF(O63&gt;0,1,-1)),
 (O63-N63)/N63
 )</f>
         <v>-0.48507587126896784</v>
       </c>
-      <c r="P208" s="80">
+      <c r="P209" s="80">
         <f>IF(O63=0,
 IF(P63=0,0,IF(P63&gt;0,1,-1)),
 (P63-O63)/O63
 )</f>
         <v>-0.48218911917098445</v>
       </c>
-      <c r="Q208" s="80">
+      <c r="Q209" s="80">
         <f>IF(P63=0,
 IF(Q63=0,0,IF(Q63&gt;0,1,-1)),
 (Q63-P63)/P63
 )</f>
         <v>-1</v>
       </c>
-      <c r="T208" s="49"/>
-      <c r="U208" s="49"/>
-      <c r="V208" s="49"/>
-      <c r="W208" s="49"/>
-      <c r="X208" s="49"/>
-      <c r="Y208" s="49"/>
-      <c r="Z208" s="49"/>
-      <c r="AA208" s="49"/>
-      <c r="AC208" s="49"/>
+      <c r="T209" s="49"/>
+      <c r="U209" s="49"/>
+      <c r="V209" s="49"/>
+      <c r="W209" s="49"/>
+      <c r="X209" s="49"/>
+      <c r="Y209" s="49"/>
+      <c r="Z209" s="49"/>
+      <c r="AA209" s="49"/>
+      <c r="AC209" s="49"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -31700,7 +31740,7 @@
   <sheetData>
     <row r="1" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B1" s="81" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.2">
@@ -32067,11 +32107,11 @@
     </row>
     <row r="37" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B37" s="228" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C37" s="228"/>
       <c r="E37" s="228" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F37" s="228"/>
     </row>
@@ -32084,26 +32124,26 @@
         <v>-6.2518906927498232E-3</v>
       </c>
       <c r="E38" s="20" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F38" s="177">
-        <f>Statement!AC185</f>
+        <f>Statement!AC186</f>
         <v>0</v>
       </c>
     </row>
     <row r="39" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B39" s="54" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="C39" s="217">
         <f ca="1">Statement!AC179</f>
         <v>-1.1014620715247336E-2</v>
       </c>
       <c r="E39" s="20" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="F39" s="177">
-        <f>Statement!AC186</f>
+        <f>Statement!AC187</f>
         <v>0</v>
       </c>
     </row>
@@ -32116,16 +32156,16 @@
         <v>0</v>
       </c>
       <c r="E40" s="20" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F40" s="177">
-        <f>Statement!AC187</f>
+        <f>Statement!AC188</f>
         <v>0</v>
       </c>
     </row>
     <row r="41" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B41" s="20" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C41" s="177">
         <f ca="1">Statement!AC182</f>
@@ -32134,7 +32174,7 @@
     </row>
     <row r="42" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B42" s="20" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C42" s="177">
         <f ca="1">Statement!AC183</f>
@@ -32143,96 +32183,96 @@
     </row>
     <row r="45" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B45" s="228" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C45" s="228"/>
       <c r="E45" s="228" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="F45" s="228"/>
     </row>
     <row r="46" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B46" s="20" t="s">
+        <v>280</v>
+      </c>
+      <c r="C46" s="177">
+        <f>Statement!AC189</f>
+        <v>5.9689614007162755E-4</v>
+      </c>
+      <c r="E46" s="20" t="s">
         <v>281</v>
       </c>
-      <c r="C46" s="177">
-        <f>Statement!AC188</f>
-        <v>5.9689614007162755E-4</v>
-      </c>
-      <c r="E46" s="20" t="s">
-        <v>282</v>
-      </c>
       <c r="F46" s="176">
-        <f>Statement!AC189</f>
+        <f>Statement!AC190</f>
         <v>6.5238758456028654</v>
       </c>
     </row>
     <row r="47" spans="2:6" x14ac:dyDescent="0.2">
       <c r="E47" s="20" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="F47" s="176">
-        <f>Statement!AC192</f>
+        <f>Statement!AC193</f>
         <v>-2.435734182252288</v>
       </c>
     </row>
     <row r="48" spans="2:6" x14ac:dyDescent="0.2">
       <c r="E48" s="20" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F48" s="177">
-        <f ca="1">Statement!AC193</f>
+        <f ca="1">Statement!AC194</f>
         <v>-2.4561199780702713E-2</v>
       </c>
     </row>
     <row r="51" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B51" s="228" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C51" s="228"/>
       <c r="E51" s="228" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="F51" s="228"/>
     </row>
     <row r="52" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B52" s="20" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C52" s="177">
-        <f>Statement!AC190</f>
+        <f>Statement!AC191</f>
         <v>0.2375751503006012</v>
       </c>
       <c r="E52" s="20" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="F52" s="177">
-        <f>Statement!AC194</f>
+        <f>Statement!AC195</f>
         <v>0.24364339787586259</v>
       </c>
     </row>
     <row r="53" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B53" s="20" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="C53" s="177">
-        <f>Statement!AC191</f>
+        <f>Statement!AC192</f>
         <v>4.4100961627885349E-2</v>
       </c>
       <c r="E53" s="20" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="F53" s="177">
-        <f>Statement!AC195</f>
+        <f>Statement!AC196</f>
         <v>1.3125250501002004</v>
       </c>
     </row>
     <row r="54" spans="2:6" x14ac:dyDescent="0.2">
       <c r="E54" s="20" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="F54" s="177">
-        <f>Statement!AC196</f>
+        <f>Statement!AC197</f>
         <v>1.0765121630506247</v>
       </c>
     </row>
@@ -32921,7 +32961,7 @@
     </row>
     <row r="32" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B32" s="14" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C32" s="14"/>
       <c r="D32" s="14"/>
@@ -33302,7 +33342,7 @@
     </row>
     <row r="50" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B50" s="14" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C50" s="14"/>
       <c r="D50" s="14"/>
@@ -33342,7 +33382,7 @@
     </row>
     <row r="52" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B52" s="20" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="C52" s="177">
         <f>Statement!M179</f>
@@ -33400,7 +33440,7 @@
     </row>
     <row r="54" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B54" s="20" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C54" s="177">
         <f>Statement!M182</f>
@@ -33429,7 +33469,7 @@
     </row>
     <row r="55" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B55" s="20" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C55" s="177">
         <f>Statement!M183</f>
@@ -33458,7 +33498,7 @@
     </row>
     <row r="57" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B57" s="14" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="C57" s="14"/>
       <c r="D57" s="14"/>
@@ -33469,94 +33509,94 @@
     </row>
     <row r="58" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B58" s="20" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C58" s="177">
-        <f>Statement!M185</f>
+        <f>Statement!M186</f>
         <v>0.64970645792563597</v>
       </c>
       <c r="D58" s="177">
-        <f>Statement!N185</f>
+        <f>Statement!N186</f>
         <v>-0.47826780445011563</v>
       </c>
       <c r="E58" s="177">
-        <f>Statement!O185</f>
+        <f>Statement!O186</f>
         <v>-0.1763765135937857</v>
       </c>
       <c r="F58" s="177">
-        <f>Statement!P185</f>
+        <f>Statement!P186</f>
         <v>-8.3866568761145496E-2</v>
       </c>
       <c r="G58" s="177">
-        <f>Statement!Q185</f>
+        <f>Statement!Q186</f>
         <v>0</v>
       </c>
       <c r="I58" s="177">
-        <f>Statement!AC185</f>
+        <f>Statement!AC186</f>
         <v>0</v>
       </c>
     </row>
     <row r="59" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B59" s="20" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C59" s="177">
-        <f>Statement!M186</f>
+        <f>Statement!M187</f>
         <v>0.27800161160354553</v>
       </c>
       <c r="D59" s="177">
-        <f>Statement!N186</f>
+        <f>Statement!N187</f>
         <v>0</v>
       </c>
       <c r="E59" s="177">
-        <f>Statement!O186</f>
+        <f>Statement!O187</f>
         <v>0</v>
       </c>
       <c r="F59" s="177">
-        <f>Statement!P186</f>
+        <f>Statement!P187</f>
         <v>0</v>
       </c>
       <c r="G59" s="177">
-        <f>Statement!Q186</f>
+        <f>Statement!Q187</f>
         <v>0</v>
       </c>
       <c r="I59" s="177">
-        <f>Statement!AC186</f>
+        <f>Statement!AC187</f>
         <v>0</v>
       </c>
     </row>
     <row r="60" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B60" s="20" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="C60" s="177">
-        <f>Statement!M187</f>
+        <f>Statement!M188</f>
         <v>0.9277080695291815</v>
       </c>
       <c r="D60" s="177">
-        <f>Statement!N187</f>
+        <f>Statement!N188</f>
         <v>-0.47826780445011563</v>
       </c>
       <c r="E60" s="177">
-        <f>Statement!O187</f>
+        <f>Statement!O188</f>
         <v>-0.1763765135937857</v>
       </c>
       <c r="F60" s="177">
-        <f>Statement!P187</f>
+        <f>Statement!P188</f>
         <v>-8.3866568761145496E-2</v>
       </c>
       <c r="G60" s="177">
-        <f>Statement!Q187</f>
+        <f>Statement!Q188</f>
         <v>0</v>
       </c>
       <c r="I60" s="177">
-        <f>Statement!AC187</f>
+        <f>Statement!AC188</f>
         <v>0</v>
       </c>
     </row>
     <row r="62" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B62" s="14" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C62" s="14"/>
       <c r="D62" s="14"/>
@@ -33567,36 +33607,36 @@
     </row>
     <row r="63" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B63" s="20" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C63" s="177">
-        <f>Statement!M188</f>
+        <f>Statement!M189</f>
         <v>4.874482086278333E-4</v>
       </c>
       <c r="D63" s="177">
-        <f>Statement!N188</f>
+        <f>Statement!N189</f>
         <v>4.8169556840077071E-4</v>
       </c>
       <c r="E63" s="177">
-        <f>Statement!O188</f>
+        <f>Statement!O189</f>
         <v>4.7058823529411766E-4</v>
       </c>
       <c r="F63" s="177">
-        <f>Statement!P188</f>
+        <f>Statement!P189</f>
         <v>4.6189376443418013E-4</v>
       </c>
       <c r="G63" s="177">
-        <f>Statement!Q188</f>
+        <f>Statement!Q189</f>
         <v>6.0060060060060057E-4</v>
       </c>
       <c r="I63" s="177">
-        <f>Statement!AC188</f>
+        <f>Statement!AC189</f>
         <v>5.9689614007162755E-4</v>
       </c>
     </row>
     <row r="65" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B65" s="14" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C65" s="14"/>
       <c r="D65" s="14"/>
@@ -33607,94 +33647,94 @@
     </row>
     <row r="66" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B66" s="20" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C66" s="176">
-        <f>Statement!M189</f>
+        <f>Statement!M190</f>
         <v>6.9776522593320234</v>
       </c>
       <c r="D66" s="176">
-        <f>Statement!N189</f>
+        <f>Statement!N190</f>
         <v>6.8498912255257434</v>
       </c>
       <c r="E66" s="176">
-        <f>Statement!O189</f>
+        <f>Statement!O190</f>
         <v>5.9210028382213808</v>
       </c>
       <c r="F66" s="176">
-        <f>Statement!P189</f>
+        <f>Statement!P190</f>
         <v>5.0951501154734409</v>
       </c>
       <c r="G66" s="176">
-        <f>Statement!Q189</f>
+        <f>Statement!Q190</f>
         <v>7.4906906906906903</v>
       </c>
       <c r="I66" s="176">
-        <f>Statement!AC189</f>
+        <f>Statement!AC190</f>
         <v>6.5238758456028654</v>
       </c>
     </row>
     <row r="67" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B67" s="20" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C67" s="176">
-        <f>Statement!M192</f>
+        <f>Statement!M193</f>
         <v>-2.3791748526522594</v>
       </c>
       <c r="D67" s="176">
-        <f>Statement!N192</f>
+        <f>Statement!N193</f>
         <v>-3.3147208121827409</v>
       </c>
       <c r="E67" s="176">
-        <f>Statement!O192</f>
+        <f>Statement!O193</f>
         <v>-5.7313150425733204</v>
       </c>
       <c r="F67" s="176">
-        <f>Statement!P192</f>
+        <f>Statement!P193</f>
         <v>-6.4547344110854503</v>
       </c>
       <c r="G67" s="176">
-        <f>Statement!Q192</f>
+        <f>Statement!Q193</f>
         <v>-1.8356356356356356</v>
       </c>
       <c r="I67" s="176">
-        <f>Statement!AC192</f>
+        <f>Statement!AC193</f>
         <v>-2.435734182252288</v>
       </c>
     </row>
     <row r="68" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B68" s="20" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C68" s="198">
-        <f>Statement!M193</f>
+        <f>Statement!M194</f>
         <v>-4.601830291547894E-2</v>
       </c>
       <c r="D68" s="198">
-        <f>Statement!N193</f>
+        <f>Statement!N194</f>
         <v>-0.12496200017933728</v>
       </c>
       <c r="E68" s="198">
-        <f>Statement!O193</f>
+        <f>Statement!O194</f>
         <v>-0.11346561311091601</v>
       </c>
       <c r="F68" s="198">
-        <f>Statement!P193</f>
+        <f>Statement!P194</f>
         <v>-0.31796721236874137</v>
       </c>
       <c r="G68" s="198">
-        <f>Statement!Q193</f>
+        <f>Statement!Q194</f>
         <v>-5.070816673026618E-2</v>
       </c>
       <c r="I68" s="198">
-        <f ca="1">Statement!AC193</f>
+        <f ca="1">Statement!AC194</f>
         <v>-2.4561199780702713E-2</v>
       </c>
     </row>
     <row r="70" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B70" s="14" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="C70" s="14"/>
       <c r="D70" s="14"/>
@@ -33705,65 +33745,65 @@
     </row>
     <row r="71" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B71" s="20" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C71" s="177">
-        <f>Statement!M190</f>
+        <f>Statement!M191</f>
         <v>6.9120043454644217E-2</v>
       </c>
       <c r="D71" s="177">
-        <f>Statement!N190</f>
+        <f>Statement!N191</f>
         <v>0.20268256333830104</v>
       </c>
       <c r="E71" s="177">
-        <f>Statement!O190</f>
+        <f>Statement!O191</f>
         <v>0.28149245924505273</v>
       </c>
       <c r="F71" s="177">
-        <f>Statement!P190</f>
+        <f>Statement!P191</f>
         <v>0.41143822393822393</v>
       </c>
       <c r="G71" s="177">
-        <f>Statement!Q190</f>
+        <f>Statement!Q191</f>
         <v>0.25100546560791998</v>
       </c>
       <c r="I71" s="177">
-        <f>Statement!AC190</f>
+        <f>Statement!AC191</f>
         <v>0.2375751503006012</v>
       </c>
     </row>
     <row r="72" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B72" s="20" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="C72" s="177">
-        <f>Statement!M191</f>
+        <f>Statement!M192</f>
         <v>2.5764324762097592E-2</v>
       </c>
       <c r="D72" s="177">
-        <f>Statement!N191</f>
+        <f>Statement!N192</f>
         <v>4.9608272274558315E-2</v>
       </c>
       <c r="E72" s="177">
-        <f>Statement!O191</f>
+        <f>Statement!O192</f>
         <v>5.9544884561481153E-2</v>
       </c>
       <c r="F72" s="177">
-        <f>Statement!P191</f>
+        <f>Statement!P192</f>
         <v>6.4217246379540877E-2</v>
       </c>
       <c r="G72" s="177">
-        <f>Statement!Q191</f>
+        <f>Statement!Q192</f>
         <v>4.6052258149963103E-2</v>
       </c>
       <c r="I72" s="177">
-        <f>Statement!AC191</f>
+        <f>Statement!AC192</f>
         <v>4.4100961627885349E-2</v>
       </c>
     </row>
     <row r="74" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B74" s="14" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C74" s="14"/>
       <c r="D74" s="14"/>
@@ -33774,88 +33814,88 @@
     </row>
     <row r="75" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B75" s="20" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="C75" s="177">
-        <f>Statement!M194</f>
+        <f>Statement!M195</f>
         <v>0.23705456570155903</v>
       </c>
       <c r="D75" s="177">
-        <f>Statement!N194</f>
+        <f>Statement!N195</f>
         <v>0.39401148222158783</v>
       </c>
       <c r="E75" s="177">
-        <f>Statement!O194</f>
+        <f>Statement!O195</f>
         <v>0.4748469425389098</v>
       </c>
       <c r="F75" s="177">
-        <f>Statement!P194</f>
+        <f>Statement!P195</f>
         <v>0.45091429539933336</v>
       </c>
       <c r="G75" s="177">
-        <f>Statement!Q194</f>
+        <f>Statement!Q195</f>
         <v>0.27710820577829071</v>
       </c>
       <c r="I75" s="177">
-        <f>Statement!AC194</f>
+        <f>Statement!AC195</f>
         <v>0.24364339787586259</v>
       </c>
     </row>
     <row r="76" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B76" s="20" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C76" s="177">
-        <f>Statement!M195</f>
+        <f>Statement!M196</f>
         <v>0.63596550787615425</v>
       </c>
       <c r="D76" s="177">
-        <f>Statement!N195</f>
+        <f>Statement!N196</f>
         <v>1.6097971878442299</v>
       </c>
       <c r="E76" s="177">
-        <f>Statement!O195</f>
+        <f>Statement!O196</f>
         <v>2.2447912126231366</v>
       </c>
       <c r="F76" s="177">
-        <f>Statement!P195</f>
+        <f>Statement!P196</f>
         <v>2.8889961389961392</v>
       </c>
       <c r="G76" s="177">
-        <f>Statement!Q195</f>
+        <f>Statement!Q196</f>
         <v>1.5103640301124059</v>
       </c>
       <c r="I76" s="177">
-        <f>Statement!AC195</f>
+        <f>Statement!AC196</f>
         <v>1.3125250501002004</v>
       </c>
     </row>
     <row r="77" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B77" s="20" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="C77" s="177">
-        <f>Statement!M196</f>
+        <f>Statement!M197</f>
         <v>1.5886194029850746</v>
       </c>
       <c r="D77" s="177">
-        <f>Statement!N196</f>
+        <f>Statement!N197</f>
         <v>1.9059455312619868</v>
       </c>
       <c r="E77" s="177">
-        <f>Statement!O196</f>
+        <f>Statement!O197</f>
         <v>2.6817329722974379</v>
       </c>
       <c r="F77" s="177">
-        <f>Statement!P196</f>
+        <f>Statement!P197</f>
         <v>2.1042270849811056</v>
       </c>
       <c r="G77" s="177">
-        <f>Statement!Q196</f>
+        <f>Statement!Q197</f>
         <v>1.2511532547411583</v>
       </c>
       <c r="I77" s="177">
-        <f>Statement!AC196</f>
+        <f>Statement!AC197</f>
         <v>1.0765121630506247</v>
       </c>
     </row>
@@ -33976,7 +34016,7 @@
     </row>
     <row r="84" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B84" s="20" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C84" s="177">
         <f>Statement!M95</f>
@@ -34002,7 +34042,7 @@
     </row>
     <row r="85" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B85" s="20" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="C85" s="177">
         <f>Statement!M97</f>
@@ -34028,7 +34068,7 @@
     </row>
     <row r="88" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B88" s="14" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="C88" s="14"/>
       <c r="D88" s="14"/>
@@ -34039,137 +34079,137 @@
     </row>
     <row r="89" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B89" s="218" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="C89" s="177">
-        <f>Statement!M200</f>
+        <f>Statement!M201</f>
         <v>1</v>
       </c>
       <c r="D89" s="177">
-        <f>Statement!N200</f>
+        <f>Statement!N201</f>
         <v>-0.22657676298045326</v>
       </c>
       <c r="E89" s="177">
-        <f>Statement!O200</f>
+        <f>Statement!O201</f>
         <v>-7.9155257608661447E-2</v>
       </c>
       <c r="F89" s="177">
-        <f>Statement!P200</f>
+        <f>Statement!P201</f>
         <v>0.139722469068289</v>
       </c>
       <c r="G89" s="177">
-        <f>Statement!Q200</f>
+        <f>Statement!Q201</f>
         <v>-3.3527259641336293E-2</v>
       </c>
       <c r="I89" s="199"/>
     </row>
     <row r="90" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B90" s="218" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="C90" s="177">
-        <f>Statement!M201</f>
+        <f>Statement!M202</f>
         <v>1</v>
       </c>
       <c r="D90" s="177">
-        <f>Statement!N201</f>
+        <f>Statement!N202</f>
         <v>-8.4923946253162061E-2</v>
       </c>
       <c r="E90" s="177">
-        <f>Statement!O201</f>
+        <f>Statement!O202</f>
         <v>-0.23547784878293962</v>
       </c>
       <c r="F90" s="177">
-        <f>Statement!P201</f>
+        <f>Statement!P202</f>
         <v>-0.242779995304062</v>
       </c>
       <c r="G90" s="177">
-        <f>Statement!Q201</f>
+        <f>Statement!Q202</f>
         <v>4.9240310077519382E-2</v>
       </c>
       <c r="I90" s="199"/>
     </row>
     <row r="91" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B91" s="20" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="C91" s="177">
-        <f>Statement!M202</f>
+        <f>Statement!M203</f>
         <v>1</v>
       </c>
       <c r="D91" s="177">
-        <f>Statement!N202</f>
+        <f>Statement!N203</f>
         <v>-0.16628914988814317</v>
       </c>
       <c r="E91" s="177">
-        <f>Statement!O202</f>
+        <f>Statement!O203</f>
         <v>-0.1521793818236705</v>
       </c>
       <c r="F91" s="177">
-        <f>Statement!P202</f>
+        <f>Statement!P203</f>
         <v>-2.1403279726227919E-2</v>
       </c>
       <c r="G91" s="177">
-        <f>Statement!Q202</f>
+        <f>Statement!Q203</f>
         <v>-6.5492915041135214E-3</v>
       </c>
       <c r="I91" s="199"/>
     </row>
     <row r="92" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B92" s="20" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="C92" s="177">
-        <f>Statement!M203</f>
+        <f>Statement!M204</f>
         <v>1</v>
       </c>
       <c r="D92" s="177">
-        <f>Statement!N203</f>
+        <f>Statement!N204</f>
         <v>0.35158501440922191</v>
       </c>
       <c r="E92" s="177">
-        <f>Statement!O203</f>
+        <f>Statement!O204</f>
         <v>1.0298507462686568</v>
       </c>
       <c r="F92" s="177">
-        <f>Statement!P203</f>
+        <f>Statement!P204</f>
         <v>17.190126050420169</v>
       </c>
       <c r="G92" s="177">
-        <f>Statement!Q203</f>
+        <f>Statement!Q204</f>
         <v>2.9393081942599757E-2</v>
       </c>
       <c r="I92" s="199"/>
     </row>
     <row r="93" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B93" s="20" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="C93" s="177">
-        <f>Statement!M204</f>
+        <f>Statement!M205</f>
         <v>1</v>
       </c>
       <c r="D93" s="177">
-        <f>Statement!N204</f>
+        <f>Statement!N205</f>
         <v>-0.58669833729216148</v>
       </c>
       <c r="E93" s="177">
-        <f>Statement!O204</f>
+        <f>Statement!O205</f>
         <v>-7.9445571331981074E-2</v>
       </c>
       <c r="F93" s="177">
-        <f>Statement!P204</f>
+        <f>Statement!P205</f>
         <v>0.32243848696290855</v>
       </c>
       <c r="G93" s="177">
-        <f>Statement!Q204</f>
+        <f>Statement!Q205</f>
         <v>-1.0552624271035824E-2</v>
       </c>
       <c r="I93" s="199"/>
     </row>
     <row r="95" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B95" s="14" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C95" s="14"/>
       <c r="D95" s="14"/>
@@ -34180,26 +34220,26 @@
     </row>
     <row r="96" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B96" s="20" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C96" s="177">
-        <f>Statement!M208</f>
+        <f>Statement!M209</f>
         <v>-1</v>
       </c>
       <c r="D96" s="177">
-        <f>Statement!N208</f>
+        <f>Statement!N209</f>
         <v>6.2544294826364283E-2</v>
       </c>
       <c r="E96" s="177">
-        <f>Statement!O208</f>
+        <f>Statement!O209</f>
         <v>-0.48507587126896784</v>
       </c>
       <c r="F96" s="177">
-        <f>Statement!P208</f>
+        <f>Statement!P209</f>
         <v>-0.48218911917098445</v>
       </c>
       <c r="G96" s="177">
-        <f>Statement!Q208</f>
+        <f>Statement!Q209</f>
         <v>-1</v>
       </c>
       <c r="I96" s="199"/>
@@ -34228,11 +34268,11 @@
     <row r="3" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B3" s="8"/>
       <c r="C3" s="232" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="D3" s="233"/>
       <c r="F3" s="234" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="G3" s="233"/>
     </row>
@@ -34257,7 +34297,7 @@
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B5" s="8" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C5" s="10" t="str">
         <f>Statement!Z3</f>
@@ -34299,7 +34339,7 @@
     </row>
     <row r="7" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B7" s="208" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C7" s="235">
         <f>Statement!AA88</f>
@@ -34338,7 +34378,7 @@
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B9" s="208" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C9" s="235">
         <f>Statement!AA89</f>
@@ -34377,7 +34417,7 @@
     </row>
     <row r="11" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B11" s="208" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C11" s="235">
         <f>Statement!AA90</f>
@@ -34416,7 +34456,7 @@
     </row>
     <row r="13" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B13" s="208" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C13" s="235">
         <f>Statement!AA94</f>
@@ -34434,7 +34474,7 @@
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B14" s="209" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C14" s="202">
         <f>Statement!Z12</f>
@@ -34455,7 +34495,7 @@
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B15" s="208" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C15" s="235">
         <f>Statement!AA95</f>
@@ -34494,7 +34534,7 @@
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B17" s="208" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C17" s="235">
         <f>Statement!AA97</f>
@@ -34512,7 +34552,7 @@
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B18" s="209" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C18" s="202">
         <f>Statement!Z22</f>
@@ -34533,7 +34573,7 @@
     </row>
     <row r="19" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B19" s="208" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C19" s="235">
         <f>IF(C18=0,
@@ -34575,7 +34615,7 @@
     </row>
     <row r="21" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B21" s="208" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C21" s="235">
         <f>IF(C20=0,
@@ -34596,7 +34636,7 @@
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B23" s="8" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C23" s="10" t="str">
         <f>C5</f>
@@ -34617,7 +34657,7 @@
     </row>
     <row r="24" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B24" s="20" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="C24" s="202">
         <f>Statement!Z105</f>
@@ -34638,7 +34678,7 @@
     </row>
     <row r="25" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B25" s="208" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C25" s="235">
         <f>IF(C24=0,
@@ -34659,7 +34699,7 @@
     </row>
     <row r="26" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B26" s="20" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="C26" s="202">
         <f>Statement!Z106</f>
@@ -34680,7 +34720,7 @@
     </row>
     <row r="27" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B27" s="208" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C27" s="235">
         <f>IF(C26=0,
@@ -34701,7 +34741,7 @@
     </row>
     <row r="28" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B28" s="20" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="C28" s="202">
         <f>Statement!Z107</f>
@@ -34722,7 +34762,7 @@
     </row>
     <row r="29" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B29" s="208" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C29" s="235">
         <f>IF(C28=0,
@@ -34743,7 +34783,7 @@
     </row>
     <row r="30" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B30" s="20" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="C30" s="202">
         <f>Statement!Z108</f>
@@ -34764,7 +34804,7 @@
     </row>
     <row r="31" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B31" s="208" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C31" s="235">
         <f>IF(C30=0,
@@ -34785,7 +34825,7 @@
     </row>
     <row r="32" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B32" s="20" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="C32" s="202">
         <f>Statement!Z109</f>
@@ -34806,7 +34846,7 @@
     </row>
     <row r="33" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B33" s="208" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C33" s="235">
         <f>IF(C32=0,
@@ -35321,7 +35361,7 @@
     </row>
     <row r="65" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B65" s="20" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="C65" s="63">
         <f>Statement!H107</f>
@@ -35366,7 +35406,7 @@
     </row>
     <row r="66" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B66" s="20" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="C66" s="63">
         <f>Statement!H108</f>
@@ -35411,7 +35451,7 @@
     </row>
     <row r="67" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B67" s="20" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="C67" s="63">
         <f>Statement!H109</f>
@@ -35899,7 +35939,7 @@
     </row>
     <row r="63" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B63" s="20" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="C63" s="63">
         <f>Statement!T107</f>
@@ -35936,7 +35976,7 @@
     </row>
     <row r="64" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B64" s="20" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="C64" s="63">
         <f>Statement!T108</f>
@@ -35973,7 +36013,7 @@
     </row>
     <row r="65" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B65" s="20" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="C65" s="63">
         <f>Statement!T109</f>

</xml_diff>